<commit_message>
Enrich all 91 papers with full-text Key findings + add 062226ECPCRR.csv
Read deeper into every uploaded PDF and populated the previously-empty
"Key findings" column (61) on all 91 PDF-backed rows with verbatim Results
statistics (effect sizes, 95% CIs, p-values, coefficients, subgroup/
moderation results). Verified design/sample/demographics against full text.

- Accuracy fix: "Disentangling..." meta-analysis sample corrected to 40
  studies / 33,737 students / 76 effect sizes (g=.101), narrowed from 258
  screened (previously conflated the screening funnel with the analytic sample).
- Added age range to Aber "Patterns" demographics.
- Regenerated ECPC_Repository_for_review.xlsx with the Key findings column
  (139 verify-flags unchanged: 112 approximate lat/long, 20 "see abstract",
  7 missing DOI). Key findings cells left un-highlighted (PDF-grounded).
- Added 062226ECPCRR.csv: full enriched dataset (99 rows x 110 cols).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -499,7 +499,7 @@
     <col width="12" customWidth="1" min="59" max="59"/>
     <col width="12" customWidth="1" min="60" max="60"/>
     <col width="12" customWidth="1" min="61" max="61"/>
-    <col width="12" customWidth="1" min="62" max="62"/>
+    <col width="75" customWidth="1" min="62" max="62"/>
     <col width="12" customWidth="1" min="63" max="63"/>
     <col width="12" customWidth="1" min="64" max="64"/>
     <col width="12" customWidth="1" min="65" max="65"/>
@@ -2059,7 +2059,7 @@
       <c r="V9" s="2" t="inlineStr"/>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>2,132 Syrian refugee children; 50.3% female; grades 1–7 (M grade=2.95); ~53% in Akkar, rest Bekaa; mean 4.1 years in Lebanon; 94.5% in extreme poverty; refugees/IDPs</t>
+          <t>2,132 Syrian refugee children; 50.3% female; grades 1–7 (M grade=2.95); ~53% in Akkar, rest Bekaa; mean 4.1 years in Lebanon; 94.5% in extreme poverty; refugees/IDPs; aged 5–16 (M=9.24, SD=2.36; 90% aged 6–12)</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr"/>
@@ -2128,7 +2128,11 @@
       <c r="BG9" s="2" t="inlineStr"/>
       <c r="BH9" s="2" t="inlineStr"/>
       <c r="BI9" s="2" t="inlineStr"/>
-      <c r="BJ9" s="2" t="inlineStr"/>
+      <c r="BJ9" s="2" t="inlineStr">
+        <is>
+          <t>Latent profile analysis of 18 self-regulation &amp; emotional well-being indicators (n=2,132); best-fitting unrestricted 7-profile model (entropy=0.853): Profile 1 Happy &amp; positive (11%), Profile 2 Poorly regulated (9%), Profile 3 Sensitive to interpersonal conflict/otherwise regulated (21%), Profile 4 Troubled in classrooms (13%), Profile 5 Well-regulated/emotionally-adjusted (14%), Profile 6 Moody &amp; frustrated (23%), Profile 7 Teacher's favorites (8%). | Multinomial regression (ref=Profile 5): school-related experiences were the most salient predictors of profile membership — school victimization predicted less-adapted profiles (Moody/frustrated b=1.15, p&lt;.001; Troubled b=1.03; Sensitive b=0.76); higher ASER academic score predicted Teacher's favorites (b=0.99) and lower odds of Poorly regulated (b=-1.50); girls less likely Poorly regulated (b=-0.79), more likely Teacher's favorites (b=1.14). No background characteristics distinguished Profile 5 vs the other well-adjusted group; war violence and family conflict were largely non-significant.</t>
+        </is>
+      </c>
       <c r="BK9" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -2416,7 +2420,11 @@
       <c r="BG10" s="2" t="inlineStr"/>
       <c r="BH10" s="2" t="inlineStr"/>
       <c r="BI10" s="2" t="inlineStr"/>
-      <c r="BJ10" s="2" t="inlineStr"/>
+      <c r="BJ10" s="2" t="inlineStr">
+        <is>
+          <t>Impacts on classroom processes (Emotional Support, Behavior Management, Supporting Student Expression) were moderate (0.5–0.6 SD); impacts on children's academic and social-emotional school-readiness outcomes were small (0.13–0.18 SD), with little evidence of impact heterogeneity by gender or baseline proficiency. | Moderate-sized reductions in teacher burnout and mid-year attrition (much larger in the private sector). | The added parental-awareness intervention rather than enhancing the teacher-training program counter-acted impacts on some dimensions of classroom quality and on ALL child outcomes, including negative impacts on numeracy 2 years later; teacher-training gains were largely sustained one year later, but teachers likely need ongoing support to sustain quality improvement.</t>
+        </is>
+      </c>
       <c r="BK10" s="2" t="inlineStr"/>
       <c r="BL10" s="2" t="inlineStr">
         <is>
@@ -2692,7 +2700,11 @@
       <c r="BG11" s="2" t="inlineStr"/>
       <c r="BH11" s="2" t="inlineStr"/>
       <c r="BI11" s="2" t="inlineStr"/>
-      <c r="BJ11" s="2" t="inlineStr"/>
+      <c r="BJ11" s="2" t="inlineStr">
+        <is>
+          <t>Only Working Memory Functioning predicted academic performance (b=.10, SE=.02, p&lt;.01), above and beyond the other SEL competencies and baseline academic performance. | Increases in academic performance were positively associated with end-of-year Working Memory Functioning (b=.24, SE=.04, p&lt;.001) and negatively associated with end-of-year Emotional Distress &amp; Internalizing Behavior (b=-.11, SE=.04, p&lt;.01). | No other SEL skill (inhibitory control, prosocial behavior, hyperactivity/externalizing) showed bidirectional associations with academics; post-hoc interactions were at most marginal (none met p&lt;.05 except a baseline-academics × initial-hyperactivity term).</t>
+        </is>
+      </c>
       <c r="BK11" s="2" t="inlineStr"/>
       <c r="BL11" s="2" t="inlineStr"/>
       <c r="BM11" s="2" t="inlineStr">
@@ -2944,7 +2956,11 @@
       <c r="BG12" s="2" t="inlineStr"/>
       <c r="BH12" s="2" t="inlineStr"/>
       <c r="BI12" s="2" t="inlineStr"/>
-      <c r="BJ12" s="2" t="inlineStr"/>
+      <c r="BJ12" s="2" t="inlineStr">
+        <is>
+          <t>Independent observation rated delivery quality as generally good: overall mean 2.36/3 (Bhutan, n=60) and 2.44/3 (Rwanda, n=60) across 10 active-teaching/learning qualities. | Workers' duty, confidence, and community respect were strong motivators. Scale-up facilitators: institutionalized training and a knowledgeable workforce in Bhutan (barrier: an overworked workforce); strong follow-up supervision in Rwanda (barrier: high attrition among a volunteer workforce).</t>
+        </is>
+      </c>
       <c r="BK12" s="2" t="inlineStr"/>
       <c r="BL12" s="2" t="inlineStr">
         <is>
@@ -3196,7 +3212,11 @@
       <c r="BG13" s="2" t="inlineStr"/>
       <c r="BH13" s="2" t="inlineStr"/>
       <c r="BI13" s="2" t="inlineStr"/>
-      <c r="BJ13" s="2" t="inlineStr"/>
+      <c r="BJ13" s="2" t="inlineStr">
+        <is>
+          <t>Trial intervention cost US$456 per family (projected to fall below US$200 if scaled through government systems). SM generated a relatively small but efficient impact on early cognitive development — comparable per home-visit session to longer-duration home-visiting programs. | Beyond ECD, SM families showed decreased harsh discipline (IRR=0.741, 95% CI 0.657–0.835) and intimate partner violence (IRR=0.616, 95% CI 0.458–0.828); further analysis is needed to monetize these returns.</t>
+        </is>
+      </c>
       <c r="BK13" s="2" t="inlineStr"/>
       <c r="BL13" s="2" t="inlineStr">
         <is>
@@ -3464,7 +3484,11 @@
       <c r="BG14" s="2" t="inlineStr"/>
       <c r="BH14" s="2" t="inlineStr"/>
       <c r="BI14" s="2" t="inlineStr"/>
-      <c r="BJ14" s="2" t="inlineStr"/>
+      <c r="BJ14" s="2" t="inlineStr">
+        <is>
+          <t>SEM (n=3,176): maternal subjective wellbeing (SWB) had only a weak, inverse total effect on child cognitive/literacy/socioemotional outcomes (≈−0.04), unchanged when standardized or mediated by family investments. | Family investments (early education, children's books, stimulating activities) had the most robust path to child outcomes (total effects 0.79, p&lt;0.001; covariance investment↔child-outcome construct 0.79, p&lt;0.001). Child-development factor loadings: cognition/approaches-to-learning 0.80, socioemotional 0.24, literacy/numeracy 0.23 (all p&lt;0.001); model fit RMSEA=0.0, CFI=1.0, TLI=1.0. Religion and education level predicted higher SWB.</t>
+        </is>
+      </c>
       <c r="BK14" s="2" t="inlineStr"/>
       <c r="BL14" s="2" t="inlineStr">
         <is>
@@ -3712,7 +3736,11 @@
       <c r="BG15" s="2" t="inlineStr"/>
       <c r="BH15" s="2" t="inlineStr"/>
       <c r="BI15" s="2" t="inlineStr"/>
-      <c r="BJ15" s="2" t="inlineStr"/>
+      <c r="BJ15" s="2" t="inlineStr">
+        <is>
+          <t>80 studies (n=18,193) representing 64 different interventions; 43 had evidence of effect on a child/adolescent mental health outcome, and only 3 found no effect on child, adolescent, or caregiver outcomes. | The most common practice elements in effective interventions were caregiver psychoeducation, communication skills, and differential reinforcement; key implementation lessons were non-specialist delivery, engagement of fathers, and integrated/multi-sector care to holistically address family needs.</t>
+        </is>
+      </c>
       <c r="BK15" s="2" t="inlineStr"/>
       <c r="BL15" s="2" t="inlineStr"/>
       <c r="BM15" s="2" t="inlineStr"/>
@@ -3936,7 +3964,11 @@
       <c r="BG16" s="2" t="inlineStr"/>
       <c r="BH16" s="2" t="inlineStr"/>
       <c r="BI16" s="2" t="inlineStr"/>
-      <c r="BJ16" s="2" t="inlineStr"/>
+      <c r="BJ16" s="2" t="inlineStr">
+        <is>
+          <t>Commentary (no statistics). Frames the psychological and social suffering of Palestinian children — the fifth generation to live under occupation and the decades-long Gaza land/air/sea blockade — as a human-rights issue, and calls for rights-based, contextually grounded responses.</t>
+        </is>
+      </c>
       <c r="BK16" s="2" t="inlineStr"/>
       <c r="BL16" s="2" t="inlineStr"/>
       <c r="BM16" s="2" t="inlineStr"/>
@@ -4200,7 +4232,11 @@
       <c r="BG17" s="2" t="inlineStr"/>
       <c r="BH17" s="2" t="inlineStr"/>
       <c r="BI17" s="2" t="inlineStr"/>
-      <c r="BJ17" s="2" t="inlineStr"/>
+      <c r="BJ17" s="2" t="inlineStr">
+        <is>
+          <t>Pilot RCT (80 dual-caregiver households; 160 caregivers, 73% female, mean age 32, SD=12). At post-intervention, FSI-ECD+VP caregivers scored higher than control on observed caregiver–child interaction (OCCI Difference=3.51, 95% CI 0.636–6.386, P=.017) and the HOME inventory (Difference=3.08, 95% CI 0.889–5.273, P=.006), including the HOME 'responsiveness' subscale (Difference=1.66, 95% CI 0.729–2.59, P&lt;.001). | Marginal reduction in physical intimate-partner violence (Difference=−0.095, 95% CI −0.192–0.002, P=.055) and some evidence of fewer depression/anxiety symptoms at 3-month follow-up; caregivers, CHWs and supervisors judged the intervention acceptable, appropriate and feasible.</t>
+        </is>
+      </c>
       <c r="BK17" s="2" t="inlineStr"/>
       <c r="BL17" s="2" t="inlineStr">
         <is>
@@ -4468,7 +4504,11 @@
       <c r="BG18" s="2" t="inlineStr"/>
       <c r="BH18" s="2" t="inlineStr"/>
       <c r="BI18" s="2" t="inlineStr"/>
-      <c r="BJ18" s="2" t="inlineStr"/>
+      <c r="BJ18" s="2" t="inlineStr">
+        <is>
+          <t>No evidence of effect modification by caregiver household type (single vs dual) on any outcome. Three-way (timepoint×treatment×household-type) interaction terms were non-significant for WAZ (β=0.081, 95% CI −0.077–0.239, p=.313), HAZ, and WHZ (β=0.129, 95% CI −0.083–0.341, p=.234), dietary diversity (β=0.256, 95% CI −0.175–0.686, p=.244), and care-seeking for diarrhea (β=2.03, 95% CI −0.92–4.97, p=.178) or fever/cough (β=1.22, 95% CI −0.13–2.56). | Suggests SM's effects are broadly applicable across single- and dual-caregiver household structures.</t>
+        </is>
+      </c>
       <c r="BK18" s="2" t="inlineStr"/>
       <c r="BL18" s="2" t="inlineStr"/>
       <c r="BM18" s="2" t="inlineStr"/>
@@ -4748,7 +4788,11 @@
       <c r="BG19" s="2" t="inlineStr"/>
       <c r="BH19" s="2" t="inlineStr"/>
       <c r="BI19" s="2" t="inlineStr"/>
-      <c r="BJ19" s="2" t="inlineStr"/>
+      <c r="BJ19" s="2" t="inlineStr">
+        <is>
+          <t>At 4-year follow-up (n=1,009; 93.1% retention), compared with usual care, SM caregivers reported more stimulating interaction (b=0.531, 95% CI 0.468–0.594) and less harsh discipline (b=−0.189, 95% CI −0.292 to −0.087), plus more learning materials (b=0.218), language stimulation (b=0.159), varied interactions (b=0.147), more father engagement in play (b=0.253), and better hygiene practices (b=0.189). | NO treatment effects on children's cognitive outcomes, self-regulation, or behavioural problems, and a small negative association with height-for-age (b=−0.038, 95% CI −0.062 to −0.012). (Trial NCT02510313.)</t>
+        </is>
+      </c>
       <c r="BK19" s="2" t="inlineStr"/>
       <c r="BL19" s="2" t="inlineStr"/>
       <c r="BM19" s="2" t="inlineStr"/>
@@ -4972,7 +5016,11 @@
       <c r="BG20" s="2" t="inlineStr"/>
       <c r="BH20" s="2" t="inlineStr"/>
       <c r="BI20" s="2" t="inlineStr"/>
-      <c r="BJ20" s="2" t="inlineStr"/>
+      <c r="BJ20" s="2" t="inlineStr">
+        <is>
+          <t>Commentary (no statistics). With ~473 million children in fragile and conflict-affected settings and &lt;1% of development assistance allocated to mental health, calls for renewed global commitments and funding mechanisms to integrate child mental health responses into recovery, development, and peacebuilding.</t>
+        </is>
+      </c>
       <c r="BK20" s="2" t="inlineStr"/>
       <c r="BL20" s="2" t="inlineStr"/>
       <c r="BM20" s="2" t="inlineStr"/>
@@ -5240,7 +5288,11 @@
       <c r="BG21" s="2" t="inlineStr"/>
       <c r="BH21" s="2" t="inlineStr"/>
       <c r="BI21" s="2" t="inlineStr"/>
-      <c r="BJ21" s="2" t="inlineStr"/>
+      <c r="BJ21" s="2" t="inlineStr">
+        <is>
+          <t>SEM test of the SM theory of change (cluster-RCT, 1,049 families): improvements in positive caregiving captured by the HOME (stimulation, early language learning) explained part of SM's effects on child gross-motor, communication, problem-solving, and personal-social development; increased dietary diversity explained effects on gross-motor, problem-solving, and personal-social development. | Only a borderline direct treatment effect on decreased caregiver emotional dysregulation (Est.=−0.054, 95% CI −0.105–0.002, p=0.046); changes in harsh/violent discipline and caregiver emotion regulation did NOT mediate child outcomes. Baseline caregiver behaviors and child outcomes predicted follow-up values (auto-regressive paths all p&lt;0.05).</t>
+        </is>
+      </c>
       <c r="BK21" s="2" t="inlineStr"/>
       <c r="BL21" s="2" t="inlineStr"/>
       <c r="BM21" s="2" t="inlineStr"/>
@@ -5504,7 +5556,11 @@
       <c r="BG22" s="2" t="inlineStr"/>
       <c r="BH22" s="2" t="inlineStr"/>
       <c r="BI22" s="2" t="inlineStr"/>
-      <c r="BJ22" s="2" t="inlineStr"/>
+      <c r="BJ22" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid Type II Implementation-Effectiveness trial (FSI-R vs usual care; Somali Bantu &amp; Bhutanese resettled refugee families during COVID-19). Bhutanese families receiving FSI-R showed improved parental supervision — poor parental monitoring was significantly reduced at midline vs CAU (B=−0.49, 95% CI −0.96 to −0.02). Bhutanese children also reported lower family arguing (β=−1.32, p=.04) and Bhutanese caregivers reported lower child conduct problems (β=−9.20, p=.01). | Process evaluation: responsiveness to community needs and delivery flexibility supported implementation despite pandemic stressors; Somali Bantu interventionists reported stronger emotional connection with families during in-person delivery. (NCT03796065.)</t>
+        </is>
+      </c>
       <c r="BK22" s="2" t="inlineStr"/>
       <c r="BL22" s="2" t="inlineStr">
         <is>
@@ -5784,7 +5840,11 @@
       <c r="BG23" s="2" t="inlineStr"/>
       <c r="BH23" s="2" t="inlineStr"/>
       <c r="BI23" s="2" t="inlineStr"/>
-      <c r="BJ23" s="2" t="inlineStr"/>
+      <c r="BJ23" s="2" t="inlineStr">
+        <is>
+          <t>Embedded cluster trial (538 households; 778 caregivers, 555 children). Vs control, SM increased home-stimulation quality (HOME B=1.01, 95% CI 0.18–1.84; Cohen's d=0.20, 0.04–0.36), involvement of children in daily activities (B=0.43, 95% CI 0.20–0.66; d=0.37, 0.18–0.57), provision of learning materials (B=0.57, 95% CI 0.24–0.90; d=0.37, 0.16–0.59), stimulating care (d=0.26), father involvement (IRR=1.18), reduced harsh discipline (OR=0.34), increased dietary diversity (d=0.25), improved caregiver mental health (d=−0.13, 95% CI −0.26 to −0.01) and safe water storage (OR=3.14). | Child-protection volunteers delivered SM with high, improving fidelity and competence; the PLAY Collaborative was rated moderately-to-highly on feasibility, leadership, organisation and sustainability — showing SM can be delivered effectively at scale through government systems.</t>
+        </is>
+      </c>
       <c r="BK23" s="2" t="inlineStr"/>
       <c r="BL23" s="2" t="inlineStr">
         <is>
@@ -6012,7 +6072,11 @@
       <c r="BG24" s="2" t="inlineStr"/>
       <c r="BH24" s="2" t="inlineStr"/>
       <c r="BI24" s="2" t="inlineStr"/>
-      <c r="BJ24" s="2" t="inlineStr"/>
+      <c r="BJ24" s="2" t="inlineStr">
+        <is>
+          <t>Commentary (no statistics). With &gt;460 million children living in armed-conflict zones, argues the global response must move BEYOND event-based framings to address the cumulative and intergenerational adversity (violence, poverty, insecurity, family disruption, service deprivation) that shapes children's mental health and development across the life course and across generations, and to pursue contextually relevant opportunities for action.</t>
+        </is>
+      </c>
       <c r="BK24" s="2" t="inlineStr"/>
       <c r="BL24" s="2" t="inlineStr"/>
       <c r="BM24" s="2" t="inlineStr"/>
@@ -6256,7 +6320,11 @@
       <c r="BG25" s="2" t="inlineStr"/>
       <c r="BH25" s="2" t="inlineStr"/>
       <c r="BI25" s="2" t="inlineStr"/>
-      <c r="BJ25" s="2" t="inlineStr"/>
+      <c r="BJ25" s="2" t="inlineStr">
+        <is>
+          <t>Online survey (n=1,444 parents/guardians of 0–36-month-olds across the four UK nations; 17.8% fathers; phase 1 of the ESRC Toddlers, Tech and Talk study, framed by UNCRC General Comment No. 25). Nearly all family homes had Wi-Fi and a wide range of digital devices, and very young children engaged in a wide range of digital activities both with their parents and on their own. | EFA/CFA on parental digital-practice/attitude items identified a three-factor structure as the best fit; parents' mediation practices were shaped by their own digital practices and attitudes, with implications for children's protection, provision and participation rights in the digital environment.</t>
+        </is>
+      </c>
       <c r="BK25" s="2" t="inlineStr"/>
       <c r="BL25" s="2" t="inlineStr">
         <is>
@@ -6508,7 +6576,11 @@
       <c r="BG26" s="2" t="inlineStr"/>
       <c r="BH26" s="2" t="inlineStr"/>
       <c r="BI26" s="2" t="inlineStr"/>
-      <c r="BJ26" s="2" t="inlineStr"/>
+      <c r="BJ26" s="2" t="inlineStr">
+        <is>
+          <t>Development and validation of the 15-item Parental Attitudes to Digital Technology Scale (PADTS) with a nationally balanced UK sample (N=934 parents of 0–3-year-olds; Toddlers, Tech and Talk study). Exploratory and confirmatory factor analyses supported a four-factor structure — perceived risks, perceived learning benefits, parental confidence, and technology-related anxiety — with strong model fit and measurement invariance across parent gender, ethnicity and region (some variation by child age). | Perceived benefits, perceptions and confidence correlated with supportive digital parenting, while technology-related anxiety was more weakly linked. PADTS is offered as a practical, validated tool for researchers, practitioners and policymakers.</t>
+        </is>
+      </c>
       <c r="BK26" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -6720,7 +6792,11 @@
       <c r="BG27" s="2" t="inlineStr"/>
       <c r="BH27" s="2" t="inlineStr"/>
       <c r="BI27" s="2" t="inlineStr"/>
-      <c r="BJ27" s="2" t="inlineStr"/>
+      <c r="BJ27" s="2" t="inlineStr">
+        <is>
+          <t>Commentary (no statistics). Argues climate change is a 'threat multiplier' for violence against children: climate-related shocks and stressors operate through social-ecological pathways (economic hardship, food/water insecurity, displacement, disrupted services, family stress) that increase children's exposure to violence; calls for integrating violence-prevention into climate adaptation, mitigation and child-protection agendas.</t>
+        </is>
+      </c>
       <c r="BK27" s="2" t="inlineStr"/>
       <c r="BL27" s="2" t="inlineStr"/>
       <c r="BM27" s="2" t="inlineStr"/>
@@ -6952,7 +7028,11 @@
       <c r="BG28" s="2" t="inlineStr"/>
       <c r="BH28" s="2" t="inlineStr"/>
       <c r="BI28" s="2" t="inlineStr"/>
-      <c r="BJ28" s="2" t="inlineStr"/>
+      <c r="BJ28" s="2" t="inlineStr">
+        <is>
+          <t>Country-level change analysis across 31 LMICs (≥2 MICS waves, 2010–2019). Each additional country-provided indicator of nurturing care was associated with an additional 0.36 developmental milestones achieved (SE=0.15, P=.03). | Population-level evidence that improvements in countries' provision of nurturing care over the decade track with improvements in countries' child-development outcomes.</t>
+        </is>
+      </c>
       <c r="BK28" s="2" t="inlineStr"/>
       <c r="BL28" s="2" t="inlineStr"/>
       <c r="BM28" s="2" t="inlineStr">
@@ -7188,7 +7268,11 @@
       <c r="BG29" s="2" t="inlineStr"/>
       <c r="BH29" s="2" t="inlineStr"/>
       <c r="BI29" s="2" t="inlineStr"/>
-      <c r="BJ29" s="2" t="inlineStr"/>
+      <c r="BJ29" s="2" t="inlineStr">
+        <is>
+          <t>IV analysis (MICS 2021 + UCDP conflict + satellite climate; rainfall instrument — each 1 mm of 2021 rainfall associated with a 0.3 pp lower likelihood of being in a one-sided-violence conflict zone, p&lt;.01). For households NOT receiving N-Power, living in a conflict zone raised the likelihood of skipping a meal by ~71.8 pp (β=0.718, p&lt;.05), eating less by 58.7 pp (β=0.587, p&lt;.10) and eating few kinds of food by 82.7 pp (β=0.827, p&lt;.05). | The N-Power cash-transfer programme significantly BUFFERED these effects (interaction terms β=−2.510, −2.133, −2.543, all p&lt;.05); buffering was not seen for the most severe indicators or for other transfers (HUP, pensions).</t>
+        </is>
+      </c>
       <c r="BK29" s="2" t="inlineStr"/>
       <c r="BL29" s="2" t="inlineStr"/>
       <c r="BM29" s="2" t="inlineStr">
@@ -7428,7 +7512,11 @@
       <c r="BG30" s="2" t="inlineStr"/>
       <c r="BH30" s="2" t="inlineStr"/>
       <c r="BI30" s="2" t="inlineStr"/>
-      <c r="BJ30" s="2" t="inlineStr"/>
+      <c r="BJ30" s="2" t="inlineStr">
+        <is>
+          <t>Pooled random- and fixed-effects models (N=3,048; four LMIC cohorts): spanking predicted lower numeracy (β=−0.23, SE=0.05, p&lt;.001), literacy (β=−0.24, p&lt;.001), social-emotional (β=−0.22, p&lt;.001) and motor (β=−0.23, p&lt;.001) skills; within-child effect sizes ranged −0.11 to −0.24 SD. | Site-specific: Bhutan (80% of children spanked) — lower social-emotional skills by 0.22 SD (p&lt;.01); Rwanda (59% spanked) — lower numeracy (β=−0.26), literacy (β=−0.33) and motor skills (β=−0.33). No evidence of any positive developmental association.</t>
+        </is>
+      </c>
       <c r="BK30" s="2" t="inlineStr"/>
       <c r="BL30" s="2" t="inlineStr"/>
       <c r="BM30" s="2" t="inlineStr">
@@ -7648,7 +7736,11 @@
       <c r="BG31" s="2" t="inlineStr"/>
       <c r="BH31" s="2" t="inlineStr"/>
       <c r="BI31" s="2" t="inlineStr"/>
-      <c r="BJ31" s="2" t="inlineStr"/>
+      <c r="BJ31" s="2" t="inlineStr">
+        <is>
+          <t>Lower-bound ECCE aid totaled US$3,646 million across 134 LMICs (2007–2021) — only 1.7% of the US$213,279 million total education aid (short of UNICEF's 10% suggested minimum). The World Bank provided US$1,944 million (53.3%). | Low-income countries' per-child ECCE aid fell from US$0.8 (2020) to US$0.6 (2021); over 15 years conflict-affected countries received an average of US$0.3 per child — a quarter of the US$1.2 per child in non-conflict-affected countries. COVID-19-related ECCE funding fell from US$50M (2020) to US$37M (2021).</t>
+        </is>
+      </c>
       <c r="BK31" s="2" t="inlineStr"/>
       <c r="BL31" s="2" t="inlineStr">
         <is>
@@ -7896,7 +7988,11 @@
       <c r="BG32" s="2" t="inlineStr"/>
       <c r="BH32" s="2" t="inlineStr"/>
       <c r="BI32" s="2" t="inlineStr"/>
-      <c r="BJ32" s="2" t="inlineStr"/>
+      <c r="BJ32" s="2" t="inlineStr">
+        <is>
+          <t>Cross-sectional MICS/DHS analysis across 18 LAC countries (children under five). Access to water and sanitation was significantly positively associated with early childhood development (ECDI on-track) and with reduced stunting; improved garbage-collection services were negatively associated with stunting and underweight. | Associations were robust to individual, maternal and household controls (incl. wealth and caregiver stimulation); household mitigation measures (treating water, handwashing cleansers, lidded trash storage) appeared to lessen impacts, pointing to a health-related (illness/diarrhea) mechanism.</t>
+        </is>
+      </c>
       <c r="BK32" s="2" t="inlineStr"/>
       <c r="BL32" s="2" t="inlineStr"/>
       <c r="BM32" s="2" t="inlineStr">
@@ -8148,7 +8244,11 @@
       <c r="BG33" s="2" t="inlineStr"/>
       <c r="BH33" s="2" t="inlineStr"/>
       <c r="BI33" s="2" t="inlineStr"/>
-      <c r="BJ33" s="2" t="inlineStr"/>
+      <c r="BJ33" s="2" t="inlineStr">
+        <is>
+          <t>Qualitative study (no statistics; interviews &amp; focus groups with policymakers N=10, facilitators N=20, parents/caregivers N=38). Intersecting micro (caregivers' capabilities and beliefs), meso (programme content and delivery) and macro (policymakers' vision, existing infrastructure) factors jointly exacerbated risks/imposed barriers versus protected/promoted VAC prevention. | Findings inform the design of acceptable, feasible, effective and sustainable parenting programmes in LMICs.</t>
+        </is>
+      </c>
       <c r="BK33" s="2" t="inlineStr"/>
       <c r="BL33" s="2" t="inlineStr">
         <is>
@@ -8380,7 +8480,11 @@
       <c r="BG34" s="2" t="inlineStr"/>
       <c r="BH34" s="2" t="inlineStr"/>
       <c r="BI34" s="2" t="inlineStr"/>
-      <c r="BJ34" s="2" t="inlineStr"/>
+      <c r="BJ34" s="2" t="inlineStr">
+        <is>
+          <t>Review / benefit-cost modelling (no primary statistics; Lancet Series paper 2 on the 'next 1000 days', ages 2–5). Summarizes benefits and costs of key multisectoral strategies — early childhood care and education (ECCE), parenting interventions, and cash transfers — building on first-1000-days investments. | Argues a minimum package (e.g., 1 year of ECCE for all children) carries substantial but worthwhile costs, and that failing to invest in the next 1000 days carries large human-capital and economic costs; calls for broader multisectoral programming.</t>
+        </is>
+      </c>
       <c r="BK34" s="2" t="inlineStr"/>
       <c r="BL34" s="2" t="inlineStr"/>
       <c r="BM34" s="2" t="inlineStr"/>
@@ -8608,7 +8712,11 @@
       <c r="BG35" s="2" t="inlineStr"/>
       <c r="BH35" s="2" t="inlineStr"/>
       <c r="BI35" s="2" t="inlineStr"/>
-      <c r="BJ35" s="2" t="inlineStr"/>
+      <c r="BJ35" s="2" t="inlineStr">
+        <is>
+          <t>Cross-national analysis (N=19,607 children aged 3–4, six countries; linear probability models with geographic &amp; seasonality fixed effects; temperature bins, ref &lt;26°C). Children exposed to average maximum temperatures above 32°C were less likely to be developmentally on track, with the drop emerging above ~30–31°C. | At 32°C, a 6.9-pp lower likelihood of being on track in the socio-emotional domain (SE=0.034) vs &lt;26°C; effects most pronounced for literacy and numeracy, and especially severe for economically disadvantaged households, urban areas, and children lacking adequate water and sanitation (26°C associated with a 2.2-pp higher likelihood of being on track in the physical domain).</t>
+        </is>
+      </c>
       <c r="BK35" s="2" t="inlineStr"/>
       <c r="BL35" s="2" t="inlineStr"/>
       <c r="BM35" s="2" t="inlineStr">
@@ -8844,7 +8952,11 @@
       <c r="BG36" s="2" t="inlineStr"/>
       <c r="BH36" s="2" t="inlineStr"/>
       <c r="BI36" s="2" t="inlineStr"/>
-      <c r="BJ36" s="2" t="inlineStr"/>
+      <c r="BJ36" s="2" t="inlineStr">
+        <is>
+          <t>Cross-sectional study merging geolocated MICS (six countries; 19,607 mother–child dyads, children 36–59 months; mean max temperature 31.58°C, SD=3.92) with ERA5-Land climate data. A 1 SD increase in recent mean maximum temperature was associated with a 4–8 pp increase in severe physical punishment and a 3–4 pp increase in psychological aggression (standardized βs ≈0.034–0.046, p&lt;.001). | No consistent associations for milder physical punishment; higher temperatures were associated with a decreased probability of nonviolent discipline — suggesting heat is a contextual driver of violent child punishment in the home.</t>
+        </is>
+      </c>
       <c r="BK36" s="2" t="inlineStr"/>
       <c r="BL36" s="2" t="inlineStr"/>
       <c r="BM36" s="2" t="inlineStr">
@@ -9072,7 +9184,11 @@
       <c r="BG37" s="2" t="inlineStr"/>
       <c r="BH37" s="2" t="inlineStr"/>
       <c r="BI37" s="2" t="inlineStr"/>
-      <c r="BJ37" s="2" t="inlineStr"/>
+      <c r="BJ37" s="2" t="inlineStr">
+        <is>
+          <t>Conceptual review/commentary (no statistics). Frames nurturing care — stable environments promoting children's health/nutrition, safety/security, learning opportunities, and emotionally supportive relationships — as a critical buffer between climate-change hazards (heatwaves, wildfires, storms, floods) and adverse child-development outcomes. | Argues caregivers are the primary protective layer for developmentally immature children, yet nurturing care rarely appears in climate research/policy; calls for integrating nurturing-care support into climate response to protect human-capital formation.</t>
+        </is>
+      </c>
       <c r="BK37" s="2" t="inlineStr"/>
       <c r="BL37" s="2" t="inlineStr"/>
       <c r="BM37" s="2" t="inlineStr"/>
@@ -9312,7 +9428,11 @@
       <c r="BG38" s="2" t="inlineStr"/>
       <c r="BH38" s="2" t="inlineStr"/>
       <c r="BI38" s="2" t="inlineStr"/>
-      <c r="BJ38" s="2" t="inlineStr"/>
+      <c r="BJ38" s="2" t="inlineStr">
+        <is>
+          <t>Editorial (no statistics). Synthesizes a 7-article Frontiers Research Topic on inclusion of young children with social-emotional or behavioral needs in early childhood education across diverse contexts (ADHD-type behaviours in Hungary/Romania/Slovakia; educator professional development in Quebec; stigma/systemic inequities for neurodiverse learners in Bangladesh). | Cross-cutting themes: inclusion as a process and outcome of empowerment; co-construction and shared expertise; and the centrality of educator learning and reflective practice — inclusion must be achieved WITH communities, not for them.</t>
+        </is>
+      </c>
       <c r="BK38" s="2" t="inlineStr"/>
       <c r="BL38" s="2" t="inlineStr"/>
       <c r="BM38" s="2" t="inlineStr"/>
@@ -9564,7 +9684,11 @@
       <c r="BG39" s="2" t="inlineStr"/>
       <c r="BH39" s="2" t="inlineStr"/>
       <c r="BI39" s="2" t="inlineStr"/>
-      <c r="BJ39" s="2" t="inlineStr"/>
+      <c r="BJ39" s="2" t="inlineStr">
+        <is>
+          <t>Quasi-experimental, rolling-cohort evaluation (559 children aged 5–6; 4 Crescendo vs 4 matched control schools; Year 1 of 7). Significant positive effects across all outcome domains, with moderate effects on behavioural self-regulation (Cohen's d=0.29, p&lt;.01) and reaction to music (d=0.21, p&lt;0.1). | Suggests orchestra–educator collaboration can support young children's musical and SEL development in resource-constrained settings; clearly defined program models aid replication/scalability.</t>
+        </is>
+      </c>
       <c r="BK39" s="2" t="inlineStr"/>
       <c r="BL39" s="2" t="inlineStr">
         <is>
@@ -9808,7 +9932,11 @@
       <c r="BG40" s="2" t="inlineStr"/>
       <c r="BH40" s="2" t="inlineStr"/>
       <c r="BI40" s="2" t="inlineStr"/>
-      <c r="BJ40" s="2" t="inlineStr"/>
+      <c r="BJ40" s="2" t="inlineStr">
+        <is>
+          <t>Methods chapter (no statistics). Documents adaptations to Sesame Workshop's formative research model for the Watch, Play, Learn early-learning videos supporting families affected by crisis and displacement across nine countries; COVID-19 movement restrictions prompted blending remote and in-person methods to assess content appeal, engagement, relevance and comprehensibility with young children and caregivers. | Offers approaches for conducting research with young children and lessons on remote data collection in emergency settings.</t>
+        </is>
+      </c>
       <c r="BK40" s="2" t="inlineStr"/>
       <c r="BL40" s="2" t="inlineStr"/>
       <c r="BM40" s="2" t="inlineStr"/>
@@ -10036,7 +10164,11 @@
       <c r="BG41" s="2" t="inlineStr"/>
       <c r="BH41" s="2" t="inlineStr"/>
       <c r="BI41" s="2" t="inlineStr"/>
-      <c r="BJ41" s="2" t="inlineStr"/>
+      <c r="BJ41" s="2" t="inlineStr">
+        <is>
+          <t>Practice/lessons-learned paper (no statistics). Describes three ways educational mass media and its diverse distribution platforms can support young children's understanding and use of COPING strategies amid adversity, using examples reaching refugee and migrant children in the US, Latin America and the Middle East. | Lessons: content curation/implementation, engagement of local and regional advisors, and the importance of a network of on-the-ground implementing partners.</t>
+        </is>
+      </c>
       <c r="BK41" s="2" t="inlineStr"/>
       <c r="BL41" s="2" t="inlineStr">
         <is>
@@ -10284,7 +10416,11 @@
       <c r="BG42" s="2" t="inlineStr"/>
       <c r="BH42" s="2" t="inlineStr"/>
       <c r="BI42" s="2" t="inlineStr"/>
-      <c r="BJ42" s="2" t="inlineStr"/>
+      <c r="BJ42" s="2" t="inlineStr">
+        <is>
+          <t>Pilot pre-post evaluation of the Huckepack summer programme (no control group; 2020 and 2022 cohorts; T1/T2 self-report on tablets). On average pupils held positive expectations of the primary-to-secondary transition; at the 2020 closing session 91.1% (41/45) agreed/strongly agreed that Huckepack adults were responsive to their needs. | In 2020 pupils reported higher perceived academic challenges at T2 than T1 (looking forward to new demands); in 2022 none of the six outcomes changed significantly from T1 to T2, and outcomes were uncorrelated with pupils' age. Self-esteem, social awareness and well-being (positively correlated with transition expectations) are flagged as promising entry points; an RCT is needed for causal evidence.</t>
+        </is>
+      </c>
       <c r="BK42" s="2" t="inlineStr"/>
       <c r="BL42" s="2" t="inlineStr"/>
       <c r="BM42" s="2" t="inlineStr"/>
@@ -10532,7 +10668,11 @@
       <c r="BG43" s="2" t="inlineStr"/>
       <c r="BH43" s="2" t="inlineStr"/>
       <c r="BI43" s="2" t="inlineStr"/>
-      <c r="BJ43" s="2" t="inlineStr"/>
+      <c r="BJ43" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-methods study (36 educators: survey + focus groups pre-transition, female n=32/male n=4; 116 newly-migrated Arab parents post-transition: female n=55, male n=61, M age 38.49, SD=10.96). Specific transition activities — communication and collaboration between educators and parents — took place and were valued as important, but specific challenges (e.g., language barriers impeding parental involvement) hindered their implementation. | Argues kindergarten-to-primary school-transition policies should center the views of migrant families and the educators who work with them.</t>
+        </is>
+      </c>
       <c r="BK43" s="2" t="inlineStr"/>
       <c r="BL43" s="2" t="inlineStr">
         <is>
@@ -10768,7 +10908,11 @@
       <c r="BG44" s="2" t="inlineStr"/>
       <c r="BH44" s="2" t="inlineStr"/>
       <c r="BI44" s="2" t="inlineStr"/>
-      <c r="BJ44" s="2" t="inlineStr"/>
+      <c r="BJ44" s="2" t="inlineStr">
+        <is>
+          <t>Pilot pre-post evaluation (135 Arab refugee/migrant caregivers in Berlin). Small, statistically NON-significant changes in most outcomes over time. | The only statistically significant finding: female participants reported a decrease in parental stress over time, whereas male participants on average reported an increase. Increases in perceived social support over time were associated with reductions in parental stress and distress and with increases in sensitive parenting, paternal engagement and co-parenting — implying parenting programs with Arab families should be tailored to the needs of male vs female caregivers.</t>
+        </is>
+      </c>
       <c r="BK44" s="2" t="inlineStr"/>
       <c r="BL44" s="2" t="inlineStr">
         <is>
@@ -11032,7 +11176,11 @@
       <c r="BG45" s="2" t="inlineStr"/>
       <c r="BH45" s="2" t="inlineStr"/>
       <c r="BI45" s="2" t="inlineStr"/>
-      <c r="BJ45" s="2" t="inlineStr"/>
+      <c r="BJ45" s="2" t="inlineStr">
+        <is>
+          <t>Implementation evaluation of the Arab Resource Collective's multi-sectoral responsive-caregiving/positive-parenting program (three delivery modalities — adapted face-to-face and a new post-COVID online modality; one Mount Lebanon village + two refugee camps in Lebanon and Jordan). Parent knowledge/attitude/behaviour surveys found high stress and harsh responses: about a third of families did not feel they could control themselves, and 54% of those reported resorting to violence or shouting at children/in the home; 38% reported further difficulties. | High 3-month follow-up retention (98% Group 1, 94.4% Group 2, 86% Group 3). The master-trainer-led face-to-face modality had a 25% dropout but improved parents' psychosocial well-being and stress more than the online program. Reports lessons for adapting parenting support in other crisis contexts.</t>
+        </is>
+      </c>
       <c r="BK45" s="2" t="inlineStr"/>
       <c r="BL45" s="2" t="inlineStr">
         <is>
@@ -11268,7 +11416,11 @@
       <c r="BG46" s="2" t="inlineStr"/>
       <c r="BH46" s="2" t="inlineStr"/>
       <c r="BI46" s="2" t="inlineStr"/>
-      <c r="BJ46" s="2" t="inlineStr"/>
+      <c r="BJ46" s="2" t="inlineStr">
+        <is>
+          <t>Pre-registered scoping review (systematic search to Sept 2022, k=6,843 records). Only 6 relevant studies identified (1 on war-affected, 5 on disaster-affected youth); experts (GROW Network) nominated 35 additional potentially relevant interventions spanning universal prevention to specialist-guided treatment — mostly self-guided and targeting young people and caregivers, with about a quarter tested via RCTs. | Less than 10% of the interventions were developed in LMICs where war/displacement typically occurs, and most were not culturally/linguistically adapted, leaving implementation potential unclear. Concludes evidence is very limited and offers a framework to guide development of new interventions.</t>
+        </is>
+      </c>
       <c r="BK46" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -11508,7 +11660,11 @@
       <c r="BG47" s="2" t="inlineStr"/>
       <c r="BH47" s="2" t="inlineStr"/>
       <c r="BI47" s="2" t="inlineStr"/>
-      <c r="BJ47" s="2" t="inlineStr"/>
+      <c r="BJ47" s="2" t="inlineStr">
+        <is>
+          <t>Prospective multinational pilot (18 in-country facilitators trained 236 frontline health-care workers at 8 sites in Nigeria &amp; Bangladesh, incl. 1 humanitarian setting; ENC online course + low-dose high-frequency manikin practice; remote vs in-person facilitation). All sites showed significant improvement in pass rates from baseline to post-training on the ENC knowledge check and bag-mask-ventilation skills (e.g., Damaturu, Nigeria: 43% → 100%). | NeoNatalie Live manikin pass rates generally improved from post-training to endline; OSCE A pass rates ranged 48–100% post-training and were largely maintained at endline (44–100%; 1 site declined). Concludes ENC online materials + LDHF practice can augment knowledge/skills and offer a flexible remote or in-person training option.</t>
+        </is>
+      </c>
       <c r="BK47" s="2" t="inlineStr"/>
       <c r="BL47" s="2" t="inlineStr">
         <is>
@@ -11740,7 +11896,11 @@
       <c r="BG48" s="2" t="inlineStr"/>
       <c r="BH48" s="2" t="inlineStr"/>
       <c r="BI48" s="2" t="inlineStr"/>
-      <c r="BJ48" s="2" t="inlineStr"/>
+      <c r="BJ48" s="2" t="inlineStr">
+        <is>
+          <t>Qualitative pilot study (25 SEL stakeholders: K-12 educators, administrators, district staff, policymakers, parents, researchers/advocates; grounded-theory; ≥20-interviewee target). SEL research evidence currently lacks accessibility for policymakers, leaders and practitioners and is hard to translate into practice; stakeholders access evidence diversely, mostly via news and education media. | SEL misinformation/disinformation may be MORE accessible to decision-makers than the supportive evidence, risking exclusionary policies; discusses implications for producing, disseminating and using SEL research amid a polarized US socio-political climate.</t>
+        </is>
+      </c>
       <c r="BK48" s="2" t="inlineStr"/>
       <c r="BL48" s="2" t="inlineStr">
         <is>
@@ -11960,7 +12120,11 @@
       <c r="BG49" s="2" t="inlineStr"/>
       <c r="BH49" s="2" t="inlineStr"/>
       <c r="BI49" s="2" t="inlineStr"/>
-      <c r="BJ49" s="2" t="inlineStr"/>
+      <c r="BJ49" s="2" t="inlineStr">
+        <is>
+          <t>Protocol (no findings). Sets out the methods for a live, searchable evidence and gap map (EGM) to identify and map all primary studies (including randomized and cluster-randomized trials) and systematic reviews on universal, school-based social and emotional learning programmes for young children aged 3–11 years.</t>
+        </is>
+      </c>
       <c r="BK49" s="2" t="inlineStr"/>
       <c r="BL49" s="2" t="inlineStr"/>
       <c r="BM49" s="2" t="inlineStr"/>
@@ -12216,7 +12380,11 @@
       <c r="BG50" s="2" t="inlineStr"/>
       <c r="BH50" s="2" t="inlineStr"/>
       <c r="BI50" s="2" t="inlineStr"/>
-      <c r="BJ50" s="2" t="inlineStr"/>
+      <c r="BJ50" s="2" t="inlineStr">
+        <is>
+          <t>Quasi-experimental pre/post evaluation (LINKS study; 607 children from 33 pre-schools; 508 post-tested after ~9 months — retention 83.7%, control 75.4% / intervention 87.9%; East-Asia Pacific Early Childhood Development Scales). At baseline the public pre-school group significantly out-performed the CBAP group on all EAP-ECDS domains. | Despite differences in time-in-pre-school and infrastructure, CBAP attendance appeared to CLOSE the baseline developmental gap between the two school types — underscoring the importance of pre-school access for children at highest risk of not reaching their developmental potential, and pointing to the need to scale and rigorously (experimentally) evaluate the programme.</t>
+        </is>
+      </c>
       <c r="BK50" s="2" t="inlineStr"/>
       <c r="BL50" s="2" t="inlineStr">
         <is>
@@ -12476,7 +12644,11 @@
       <c r="BG51" s="2" t="inlineStr"/>
       <c r="BH51" s="2" t="inlineStr"/>
       <c r="BI51" s="2" t="inlineStr"/>
-      <c r="BJ51" s="2" t="inlineStr"/>
+      <c r="BJ51" s="2" t="inlineStr">
+        <is>
+          <t>Prospective study (Syrian refugee father–mother–child triads, n=160 T1 / 105 T2; children 4–8). Syrian fathers rated themselves as highly involved — 13% MORE involved than mothers reported them to be (and indicated 17.6% more time with children, ~0.6 more days/week, than mothers reported). Levels of father involvement were largely UNRELATED to child outcomes. | Spousal DISAGREEMENT about father involvement was negatively associated with relationship quality, mother mental health and child social-emotional learning (SEL): in the most discordant families, child SEL was more than 1 SD (43%) below the most concordant families — distinguishing levels of involvement from father–mother agreement.</t>
+        </is>
+      </c>
       <c r="BK51" s="2" t="inlineStr"/>
       <c r="BL51" s="2" t="inlineStr"/>
       <c r="BM51" s="2" t="inlineStr">
@@ -12700,7 +12872,11 @@
           <t>Yes (toxic stress / war-related adversity)</t>
         </is>
       </c>
-      <c r="BJ52" s="2" t="inlineStr"/>
+      <c r="BJ52" s="2" t="inlineStr">
+        <is>
+          <t>Comprehensive review (37 publications since 2000; most refugees relocated in Europe and the Middle East; 24 of 37 studied adults rather than youth/children). Cross-sectional, observational and experimental studies show heterogeneous physiological and genomic (DNA methylation, MAOA, 5-HTT, COMT) responses to war-related adversity and their links to health — e.g., higher BDNF/NGF associated with worse PTSD, depression and anxiety scores when controlling for pre-displacement exposures. | Concludes with four observations: why genomic/physiological biomarkers are valuable; which study designs advance causal/intervention understanding; how to prepare for ethical challenges; and why theoretical frameworks and research procedures need more detailed consideration.</t>
+        </is>
+      </c>
       <c r="BK52" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -12948,7 +13124,11 @@
           <t>cortisol</t>
         </is>
       </c>
-      <c r="BJ53" s="2" t="inlineStr"/>
+      <c r="BJ53" s="2" t="inlineStr">
+        <is>
+          <t>Multivariable regression of diurnal salivary cortisol among adolescent mothers (14–19) and infants in São Paulo (saliva from n=23 mothers, n=32 infants at 12 months postpartum; adjusting for intervention group, infant sex, maternal age, medication and sample timing). Higher-than-average LIFETIME trauma exposure was associated with maternal EVENING cortisol (b=0.472, p=.028); lifetime assaultive-violence exposure likewise (b=0.196, p=.02); and maternal trauma during PREGNANCY was positively associated with INFANT bedtime cortisol (b=0.21, p=.01). | Trauma variables were not associated with maternal or infant morning cortisol — consistent with fetal-programming models of intergenerational trauma transmission.</t>
+        </is>
+      </c>
       <c r="BK53" s="2" t="inlineStr"/>
       <c r="BL53" s="2" t="inlineStr"/>
       <c r="BM53" s="2" t="inlineStr">
@@ -13200,7 +13380,11 @@
           <t>epigenetics</t>
         </is>
       </c>
-      <c r="BJ54" s="2" t="inlineStr"/>
+      <c r="BJ54" s="2" t="inlineStr">
+        <is>
+          <t>Epigenome-wide association study across three generations of Syrian refugees (buccal swabs + survey from mothers and 1–2 children in each of 48 families; n=131 participants). Identified differentially methylated regions: 14 associated with germline and 21 with direct exposure to violence; most DMPs showed the SAME directionality of DNAm change across germline, prenatal and direct exposures, suggesting a common epigenetic response to violence. | Also identified epigenetic age acceleration associated with PRENATAL exposure to violence in children — the first reported intergenerational epigenetic signature of violence, with important implications for understanding the inheritance of trauma.</t>
+        </is>
+      </c>
       <c r="BK54" s="2" t="inlineStr"/>
       <c r="BL54" s="2" t="inlineStr"/>
       <c r="BM54" s="2" t="inlineStr"/>
@@ -13424,7 +13608,11 @@
       <c r="BG55" s="2" t="inlineStr"/>
       <c r="BH55" s="2" t="inlineStr"/>
       <c r="BI55" s="2" t="inlineStr"/>
-      <c r="BJ55" s="2" t="inlineStr"/>
+      <c r="BJ55" s="2" t="inlineStr">
+        <is>
+          <t>Review (no primary statistics; ~50 million children under 18 forcibly displaced). More than 50% of forcibly displaced children in highly adverse contexts experience mental health problems — over four times the 13% global estimate for non-displaced children — yet up to 90% in LMICs never receive appropriate care (only ~25% resettle in high-income countries; ~69% settle in directly bordering countries). | Synthesizes prevalence, individual differences in response, and existing MHPSS approaches; some interventions have positively influenced displaced children's mental health, but more culturally/contextually relevant, accessible services that also address family and community factors — and links to strategies targeting structural barriers — are needed (socio-ecological framework).</t>
+        </is>
+      </c>
       <c r="BK55" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -13640,7 +13828,11 @@
       <c r="BG56" s="2" t="inlineStr"/>
       <c r="BH56" s="2" t="inlineStr"/>
       <c r="BI56" s="2" t="inlineStr"/>
-      <c r="BJ56" s="2" t="inlineStr"/>
+      <c r="BJ56" s="2" t="inlineStr">
+        <is>
+          <t>Cohort study (1,133 caregivers, 87.6% female, mean age 29.39; 14 Colombian municipalities; child SEC for ages 21–53 months; resilience subsample n=487). Caregivers reported substantial psychopathology: 12.84% elevated anxiety, 24.5% above the PTSD cutoff, and 44.7% screened positive for depression (among displaced children 13.2% high PTSD vs 6.6% non-displaced). | Child SEC–caregiver psychopathology correlations r=0.15–0.33; the caregiver-depression↔child-SEC association was stronger for boys (B=0.56) than girls (B=0.22); girls whose caregivers reported elevated psychopathology AND low resilience received the highest caregiver-reported SEC ratings. Underscores caregiver–child resilience-focused psychosocial support.</t>
+        </is>
+      </c>
       <c r="BK56" s="2" t="inlineStr"/>
       <c r="BL56" s="2" t="inlineStr"/>
       <c r="BM56" s="2" t="inlineStr"/>
@@ -13896,7 +14088,11 @@
       <c r="BG57" s="2" t="inlineStr"/>
       <c r="BH57" s="2" t="inlineStr"/>
       <c r="BI57" s="2" t="inlineStr"/>
-      <c r="BJ57" s="2" t="inlineStr"/>
+      <c r="BJ57" s="2" t="inlineStr">
+        <is>
+          <t>Cluster-RCT (3,858 children, n=3,852 with complete IDELA, across four survey rounds Jan 2019–Mar 2021; LEAPS implemented in 91 of 99 villages). LEAPS significantly increased children's school readiness vs control (IDELA overall SMD=0.30, 95% CI 0.20–0.40, p&lt;0.0001). | Among executive-function skills only cognitive flexibility improved (dimensional change card sort SMD=0.22, 95% CI 0.12–0.33, p&lt;0.0001); the effect on total IDELA was larger in round 2, before COVID-19 (SMD=0.37, 95% CI 0.22–0.52). Offers a scalable youth-led model to expand high-quality ECCE and school readiness while creating employment for female youth.</t>
+        </is>
+      </c>
       <c r="BK57" s="2" t="inlineStr"/>
       <c r="BL57" s="2" t="inlineStr">
         <is>
@@ -14116,7 +14312,11 @@
       <c r="BG58" s="2" t="inlineStr"/>
       <c r="BH58" s="2" t="inlineStr"/>
       <c r="BI58" s="2" t="inlineStr"/>
-      <c r="BJ58" s="2" t="inlineStr"/>
+      <c r="BJ58" s="2" t="inlineStr">
+        <is>
+          <t>Conceptual review (no statistics; Cowan, Cowan, M.K. Pruett &amp; K.D. Pruett). Examines the gap between CORRELATIONAL and INTERVENTION studies of fatherhood and children's development through a family-systems ecological perspective. | Synthesizes how father involvement relates to child outcomes and how randomized father/couple intervention studies can establish causal pathways, emphasizing coparenting, the couple relationship and the wider family system rather than father involvement in isolation.</t>
+        </is>
+      </c>
       <c r="BK58" s="2" t="inlineStr"/>
       <c r="BL58" s="2" t="inlineStr"/>
       <c r="BM58" s="2" t="inlineStr"/>
@@ -14328,7 +14528,11 @@
       <c r="BG59" s="2" t="inlineStr"/>
       <c r="BH59" s="2" t="inlineStr"/>
       <c r="BI59" s="2" t="inlineStr"/>
-      <c r="BJ59" s="2" t="inlineStr"/>
+      <c r="BJ59" s="2" t="inlineStr">
+        <is>
+          <t>Meta-analysis of Early Childhood Development Index data (UNICEF MICS + DHS, 2010–2019; n=226,980 children aged 36–59 months, 49% female, across 71 LMICs). In about half of LMICs, odds of being developmentally on track did not differ significantly by gender; where they did, girls were more likely on track than boys (overall pooled OR=1.21, 95% CI 1.18–1.24, p&lt;.001), with the largest difference in the social-emotional domain (OR=1.27, 95% CI 1.24–1.30) and a smaller literacy-numeracy advantage (OR=1.13, 95% CI 1.10–1.17); no gender differences in the physical-health domain. | Country-level significant ORs ranged from 1.12 (Nigeria) to 2.51 (North Macedonia); meta-regression on the Gender Development Index explained substantial between-country heterogeneity — girls' advantage was larger in countries with greater gender equality.</t>
+        </is>
+      </c>
       <c r="BK59" s="2" t="inlineStr"/>
       <c r="BL59" s="2" t="inlineStr"/>
       <c r="BM59" s="2" t="inlineStr"/>
@@ -14568,7 +14772,11 @@
       <c r="BG60" s="2" t="inlineStr"/>
       <c r="BH60" s="2" t="inlineStr"/>
       <c r="BI60" s="2" t="inlineStr"/>
-      <c r="BJ60" s="2" t="inlineStr"/>
+      <c r="BJ60" s="2" t="inlineStr">
+        <is>
+          <t>Longitudinal study (N=1,240 Russian first-graders, 49.5% female). Confirmed the gendered pattern over the first-grade year (girls ahead in language, boys in math): significant gender×time interactions for literacy (F(1,1236)=5.63, p=.02, d=0.07) and math (F=7.97, p=.005, d=0.08). | Parents produced more input in literacy than math (domain main effect d=0.27) and gave gender-differentiated input (domain×gender F(1,1237)=130.49, p&lt;.001, d=0.33 — more literacy activities with girls, more math with boys); parent education predicted input (d=0.22). Changes in gender differences in children's language and math skills were MEDIATED by language and math parental input, respectively.</t>
+        </is>
+      </c>
       <c r="BK60" s="2" t="inlineStr"/>
       <c r="BL60" s="2" t="inlineStr"/>
       <c r="BM60" s="2" t="inlineStr">
@@ -14828,7 +15036,11 @@
       <c r="BG61" s="2" t="inlineStr"/>
       <c r="BH61" s="2" t="inlineStr"/>
       <c r="BI61" s="2" t="inlineStr"/>
-      <c r="BJ61" s="2" t="inlineStr"/>
+      <c r="BJ61" s="2" t="inlineStr">
+        <is>
+          <t>Primary-data SEM (267 parents; child M age 13.66 months, 52% girls; Bogotá &amp; Soacha). Most parents reported ≥1 symptom of distress (M=1.88, SD=0.50). The partially-mediated model fit well (RMSEA=0.04, CFI=0.91, SRMR=0.05) and was favored over the fully-mediated alternative (Δχ²(4)=18.30, p=.001). | Positive parental beliefs about violence were linked to reduced engagement in stimulating activities, predicting lower child effortful control and positive affectivity; parental psychological distress was associated with greater use of violent punishment, predicting lower effortful control and higher negative affectivity. Underscores addressing parental beliefs and well-being to support positive parenting in LMICs.</t>
+        </is>
+      </c>
       <c r="BK61" s="2" t="inlineStr"/>
       <c r="BL61" s="2" t="inlineStr">
         <is>
@@ -15092,7 +15304,11 @@
       <c r="BG62" s="2" t="inlineStr"/>
       <c r="BH62" s="2" t="inlineStr"/>
       <c r="BI62" s="2" t="inlineStr"/>
-      <c r="BJ62" s="2" t="inlineStr"/>
+      <c r="BJ62" s="2" t="inlineStr">
+        <is>
+          <t>Mixed-methods pilot (convergent parallel; difference-in-differences + thematic analysis; N=267 caregivers — 134 Apapacho, 133 comparison; 99.3% female, mean age 28.9, 97.4% mothers; qualitative N=22; baseline &amp; 1-month follow-up). Apapacho was associated with short-term improvements in beliefs about responsive caregiving (β=0.17), increased stimulation (β=0.19), increased use of non-violent discipline (β=0.12) and reduced approval of violent discipline (β=0.12). | Qualitative findings: better caregiver–child relationships, greater understanding of children's needs, increased emotional awareness/self-regulation and more non-violent discipline — a promising strategy for positive parenting and violence prevention, integrated into Colombia's national Modalidad Familiar service.</t>
+        </is>
+      </c>
       <c r="BK62" s="2" t="inlineStr"/>
       <c r="BL62" s="2" t="inlineStr">
         <is>
@@ -15336,7 +15552,11 @@
       <c r="BG63" s="2" t="inlineStr"/>
       <c r="BH63" s="2" t="inlineStr"/>
       <c r="BI63" s="2" t="inlineStr"/>
-      <c r="BJ63" s="2" t="inlineStr"/>
+      <c r="BJ63" s="2" t="inlineStr">
+        <is>
+          <t>Quasi-experimental two-generation study (CareerAdvance + Head Start, 3 years). CareerAdvance promoted low-income parents' EDUCATIONAL advancement, with weaker evidence of career-progress and psychological-wellbeing benefits and NO evidence of economic gains. | Psychological wellbeing: immediate (Year 1) increase in optimism (ES=0.305, p=.088), sustained to end of Year 2 (ES=0.312, p=.066); parents WITH postsecondary credentials at baseline continued to show increased optimism through Year 3 (ES=0.291, p=.069). Educational/career advancement was greater for parents without baseline credentials.</t>
+        </is>
+      </c>
       <c r="BK63" s="2" t="inlineStr"/>
       <c r="BL63" s="2" t="inlineStr">
         <is>
@@ -15592,7 +15812,11 @@
       <c r="BG64" s="2" t="inlineStr"/>
       <c r="BH64" s="2" t="inlineStr"/>
       <c r="BI64" s="2" t="inlineStr"/>
-      <c r="BJ64" s="2" t="inlineStr"/>
+      <c r="BJ64" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT ($333 vs $20/month, 3 years; 1,000 dyads, 857 across all 3 waves; majority Black 42% and Hispanic 41%). NO statistically detectable differences between high- and low-cash groups in maternal assessments of children's health/medical care, sleep disturbances, or healthy/unhealthy food consumption (effect sizes 0.01–0.08). | Infants were of normal birthweight (mean 7.11 lb) and born at term.</t>
+        </is>
+      </c>
       <c r="BK64" s="2" t="inlineStr"/>
       <c r="BL64" s="2" t="inlineStr"/>
       <c r="BM64" s="2" t="inlineStr">
@@ -15852,7 +16076,11 @@
       <c r="BG65" s="2" t="inlineStr"/>
       <c r="BH65" s="2" t="inlineStr"/>
       <c r="BI65" s="2" t="inlineStr"/>
-      <c r="BJ65" s="2" t="inlineStr"/>
+      <c r="BJ65" s="2" t="inlineStr">
+        <is>
+          <t>Two-year experimental mixed-methods evaluation of a Two-Generation ESL program (189 Latinx &amp; Zomi immigrant parents; 67 in focus groups). Treatment parents reported significantly higher English writing skills — the 1-year positive effect was sustained and grew after 2 years (B=0.36, SE=0.14, p=.009) — higher self-esteem, and significantly less language brokering (B=−0.29, SE=0.14, p=.049) and material hardship. | NO significant effect on positive parenting skills and NO significant differences in children's outcomes; qualitative data identified explanatory mechanisms across contexts.</t>
+        </is>
+      </c>
       <c r="BK65" s="2" t="inlineStr"/>
       <c r="BL65" s="2" t="inlineStr"/>
       <c r="BM65" s="2" t="inlineStr">
@@ -16080,7 +16308,11 @@
       <c r="BG66" s="2" t="inlineStr"/>
       <c r="BH66" s="2" t="inlineStr"/>
       <c r="BI66" s="2" t="inlineStr"/>
-      <c r="BJ66" s="2" t="inlineStr"/>
+      <c r="BJ66" s="2" t="inlineStr">
+        <is>
+          <t>Conceptual review (no statistics). Argues that, globally, two-generation approaches (harnessing synergies between children's development and caregivers' education/livelihood/well-being) are likely more effective than single-generation approaches against poverty. | Identifies five program models across regions grouped as quality child care; ECD + nonformal parent education; and cash transfers + parenting — calling for more research on two-generation programs and policies globally.</t>
+        </is>
+      </c>
       <c r="BK66" s="2" t="inlineStr"/>
       <c r="BL66" s="2" t="inlineStr"/>
       <c r="BM66" s="2" t="inlineStr"/>
@@ -16328,7 +16560,11 @@
       <c r="BG67" s="2" t="inlineStr"/>
       <c r="BH67" s="2" t="inlineStr"/>
       <c r="BI67" s="2" t="inlineStr"/>
-      <c r="BJ67" s="2" t="inlineStr"/>
+      <c r="BJ67" s="2" t="inlineStr">
+        <is>
+          <t>Experimental analysis of the Baby's First Years RCT ($333 vs $20/month) of poverty-reduction impacts on maternal well-being and family processes among ~1,000 low-income US mothers of young children (food-insecurity α=.85–.87; PHQ-8 depression α=.84; detectable effect size ≈.195 SD). | Experimentally analyzes impacts of monthly unconditional cash transfers on maternal well-being and family processes.</t>
+        </is>
+      </c>
       <c r="BK67" s="2" t="inlineStr"/>
       <c r="BL67" s="2" t="inlineStr"/>
       <c r="BM67" s="2" t="inlineStr">
@@ -16580,7 +16816,11 @@
       <c r="BG68" s="2" t="inlineStr"/>
       <c r="BH68" s="2" t="inlineStr"/>
       <c r="BI68" s="2" t="inlineStr"/>
-      <c r="BJ68" s="2" t="inlineStr"/>
+      <c r="BJ68" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT analysis (N=563 mothers and their 1-year-olds; 48% girls; 2019–2020). Monthly unconditional cash transfers did NOT impact mothers' child-directed speech during a 10-min at-home play session (effect sizes range −.08 to .02), though within-sample variability was wide. | Consistent with related findings that maternal stress was not associated with SES and did not mediate SES–language-input associations.</t>
+        </is>
+      </c>
       <c r="BK68" s="2" t="inlineStr"/>
       <c r="BL68" s="2" t="inlineStr"/>
       <c r="BM68" s="2" t="inlineStr">
@@ -16840,7 +17080,11 @@
       <c r="BG69" s="2" t="inlineStr"/>
       <c r="BH69" s="2" t="inlineStr"/>
       <c r="BI69" s="2" t="inlineStr"/>
-      <c r="BJ69" s="2" t="inlineStr"/>
+      <c r="BJ69" s="2" t="inlineStr">
+        <is>
+          <t>Cluster-RCT (99 community health volunteers; 2,298 caregivers; Syrian &amp; Jordanian families, phone-delivered). Exposure to the parenting + caregiver-support condition produced a small but statistically significant reduction in caregivers' depressive symptoms (β=−0.06, p=0.021; adjusted p=0.044; ES=−0.11), robust to multiple-comparison adjustment. | NO significant impacts on caregiver anxiety, parenting stress, harsh discipline, parent–child learning activities, or parenting self-efficacy, and no significant effects on child development (BITSEA, ASQ) or implementation outcomes; no moderation by household nationality, child gender, or child age.</t>
+        </is>
+      </c>
       <c r="BK69" s="2" t="inlineStr"/>
       <c r="BL69" s="2" t="inlineStr">
         <is>
@@ -17108,7 +17352,11 @@
       <c r="BG70" s="2" t="inlineStr"/>
       <c r="BH70" s="2" t="inlineStr"/>
       <c r="BI70" s="2" t="inlineStr"/>
-      <c r="BJ70" s="2" t="inlineStr"/>
+      <c r="BJ70" s="2" t="inlineStr">
+        <is>
+          <t>Quasi-experimental study (147 CareerAdvance + 139 matched comparison children; n=286; M age 3.6, 47% female; 3 years). The effect of adding parent education/workforce training (CareerAdvance) to Head Start on children's academic, language, math and inhibitory-control outcomes was neither greater nor less than Head Start alone. | Subgroup: among low-parent-education families the treatment effect was nonsignificant though positive (β=.309, SE=0.387, p=.431) — children's developmental outcomes did not worsen or improve in the short term when parents returned to school.</t>
+        </is>
+      </c>
       <c r="BK70" s="2" t="inlineStr"/>
       <c r="BL70" s="2" t="inlineStr"/>
       <c r="BM70" s="2" t="inlineStr">
@@ -17356,7 +17604,11 @@
       <c r="BG71" s="2" t="inlineStr"/>
       <c r="BH71" s="2" t="inlineStr"/>
       <c r="BI71" s="2" t="inlineStr"/>
-      <c r="BJ71" s="2" t="inlineStr"/>
+      <c r="BJ71" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT (N=828; preregistered intent-to-treat, wave-4 maternal MEFS analytic sample). NO differences in low-income US mothers' cognitive bandwidth after receiving a high-cash ($333/month) vs low-cash ($20/month) gift for 48 months after childbirth — contrary to scarcity-theory predictions.</t>
+        </is>
+      </c>
       <c r="BK71" s="2" t="inlineStr"/>
       <c r="BL71" s="2" t="inlineStr"/>
       <c r="BM71" s="2" t="inlineStr">
@@ -17572,7 +17824,11 @@
       <c r="BG72" s="2" t="inlineStr"/>
       <c r="BH72" s="2" t="inlineStr"/>
       <c r="BI72" s="2" t="inlineStr"/>
-      <c r="BJ72" s="2" t="inlineStr"/>
+      <c r="BJ72" s="2" t="inlineStr">
+        <is>
+          <t>Conceptual framework (no statistics; bioecological &amp; dynamic-systems perspectives). Presents a framework for how the distinctive dual time frame of acute (extreme weather events) and chronic (ecological degradation) climate-change risks, experienced prenatally and early in life across ecological contexts, can threaten human development. | Calls on developmental researchers, practitioners and policymakers to address the climate crisis's developmental consequences.</t>
+        </is>
+      </c>
       <c r="BK72" s="2" t="inlineStr"/>
       <c r="BL72" s="2" t="inlineStr"/>
       <c r="BM72" s="2" t="inlineStr"/>
@@ -17820,7 +18076,11 @@
       <c r="BG73" s="2" t="inlineStr"/>
       <c r="BH73" s="2" t="inlineStr"/>
       <c r="BI73" s="2" t="inlineStr"/>
-      <c r="BJ73" s="2" t="inlineStr"/>
+      <c r="BJ73" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years registered report (1,000 racially/ethnically diverse US mothers in poverty; 40% high-cash n=400 / 60% low-cash n=600; maternal reports at ages 1, 2, 3). NO statistically detectable impacts of the high-cash gift ($333 vs $20/month) on maternal reports of children's early language and socioemotional development, concerns for developmental delay, or enrollment in early-intervention services across ages 1–3.</t>
+        </is>
+      </c>
       <c r="BK73" s="2" t="inlineStr"/>
       <c r="BL73" s="2" t="inlineStr"/>
       <c r="BM73" s="2" t="inlineStr">
@@ -18076,7 +18336,11 @@
       <c r="BG74" s="2" t="inlineStr"/>
       <c r="BH74" s="2" t="inlineStr"/>
       <c r="BI74" s="2" t="inlineStr"/>
-      <c r="BJ74" s="2" t="inlineStr"/>
+      <c r="BJ74" s="2" t="inlineStr">
+        <is>
+          <t>Research brief (descriptive; Baby's First Years, $333 vs $20/month; 1,000 mothers near/below poverty + newborns, recruited 2018–19 from 12 hospitals in 4 US communities). Reports three-year follow-up findings on food security, household spending and consumption, situating cash transfers alongside SNAP and WIC in reducing child poverty and hunger and supporting child development (noting persistent inequities such as food deserts).</t>
+        </is>
+      </c>
       <c r="BK74" s="2" t="inlineStr"/>
       <c r="BL74" s="2" t="inlineStr"/>
       <c r="BM74" s="2" t="inlineStr">
@@ -18328,7 +18592,11 @@
       <c r="BG75" s="2" t="inlineStr"/>
       <c r="BH75" s="2" t="inlineStr"/>
       <c r="BI75" s="2" t="inlineStr"/>
-      <c r="BJ75" s="2" t="inlineStr"/>
+      <c r="BJ75" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT (1,000 low-income US mothers, infant's first year). The likelihood and length of breastfeeding, use of nonparental child care, and maternal employment did NOT statistically differ between high- ($333) and low-cash ($20) groups. | However, the higher gift DELAYED the starting age of child care by almost 1 month (low-cash infants entered home-/center-based care 1 month sooner, p&lt;.01) and increased mothers' ability to meet their birth-stated breastfeeding intentions; the high-cash effect in New York differed statistically from other sites (p&lt;.10).</t>
+        </is>
+      </c>
       <c r="BK75" s="2" t="inlineStr"/>
       <c r="BL75" s="2" t="inlineStr"/>
       <c r="BM75" s="2" t="inlineStr">
@@ -18592,7 +18860,11 @@
       <c r="BG76" s="2" t="inlineStr"/>
       <c r="BH76" s="2" t="inlineStr"/>
       <c r="BI76" s="2" t="inlineStr"/>
-      <c r="BJ76" s="2" t="inlineStr"/>
+      <c r="BJ76" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT after 4 years of monthly cash ($333 vs $20; data from 891 of 1,000 dyads; mean maternal age 27.0). NO statistically detectable group differences in maternal depressive symptoms (ES=0.04, 95% CI −0.08 to 0.17, p=.51), anxiety (ES=0.12, p=.09), or BMI (ES=−0.06, p=.42), nor in child BMI percentile or maternal-reported child health. | Designed to detect an effect size of ~0.20 SD after expected 20% attrition.</t>
+        </is>
+      </c>
       <c r="BK76" s="2" t="inlineStr"/>
       <c r="BL76" s="2" t="inlineStr"/>
       <c r="BM76" s="2" t="inlineStr">
@@ -18836,7 +19108,11 @@
       <c r="BG77" s="2" t="inlineStr"/>
       <c r="BH77" s="2" t="inlineStr"/>
       <c r="BI77" s="2" t="inlineStr"/>
-      <c r="BJ77" s="2" t="inlineStr"/>
+      <c r="BJ77" s="2" t="inlineStr">
+        <is>
+          <t>Cohort profile (descriptive; first large prenatal birth-cohort study in a refugee context in an LMIC; Cox's Bazar, N=2,888, 80% Rohingya, recruited over 12 months). Rohingya women were substantially less literate, married/had children younger, lived in more crowded/resource-limited households, and had higher rates of clinically significant PTSD and anxiety than host-community women. | A fifth wave (children 6 months) was completed April 2025; the next follow-up is planned at child age 36 months (from March 2026).</t>
+        </is>
+      </c>
       <c r="BK77" s="2" t="inlineStr"/>
       <c r="BL77" s="2" t="inlineStr">
         <is>
@@ -19084,7 +19360,11 @@
       <c r="BG78" s="2" t="inlineStr"/>
       <c r="BH78" s="2" t="inlineStr"/>
       <c r="BI78" s="2" t="inlineStr"/>
-      <c r="BJ78" s="2" t="inlineStr"/>
+      <c r="BJ78" s="2" t="inlineStr">
+        <is>
+          <t>9-year prospective Chinese cohort (N=356 middle-class families, 48.9% female; maternal sensitivity observed at 14 &amp; 24 months, child attachment via the Attachment Script Assessment at age 10). Early maternal sensitivity positively predicted children's attachment representations at age 10 (β=0.20, p&lt;0.01), supporting the cross-cultural universality of the sensitivity→attachment-security hypothesis outside Western contexts. | (Meta-analytic benchmark for the sensitivity–attachment link r=0.25.)</t>
+        </is>
+      </c>
       <c r="BK78" s="2" t="inlineStr"/>
       <c r="BL78" s="2" t="inlineStr"/>
       <c r="BM78" s="2" t="inlineStr">
@@ -19360,7 +19640,11 @@
           <t>EEG (brain activity)</t>
         </is>
       </c>
-      <c r="BJ79" s="2" t="inlineStr"/>
+      <c r="BJ79" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT after 4 years of monthly cash ($333 vs $20; n=891; valid observations 637–886 across outcomes). NO statistically significant impacts on four preregistered primary outcomes (language, executive function, social-emotional problems, high-frequency brain activity) nor on three secondary outcomes (visual processing/spatial perception, pre-literacy, maternal reports of developmental diagnoses). | Designed to detect an effect size of ~0.20 SD after expected 20% attrition.</t>
+        </is>
+      </c>
       <c r="BK79" s="2" t="inlineStr"/>
       <c r="BL79" s="2" t="inlineStr"/>
       <c r="BM79" s="2" t="inlineStr">
@@ -19612,7 +19896,11 @@
       <c r="BG80" s="2" t="inlineStr"/>
       <c r="BH80" s="2" t="inlineStr"/>
       <c r="BI80" s="2" t="inlineStr"/>
-      <c r="BJ80" s="2" t="inlineStr"/>
+      <c r="BJ80" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years subgroup analysis of Latina families (~36 months of cash-gift receipt; spending descriptives from 4MyBaby debit-card transactions, n=363 Latina of 900 overall; survey N=392 Latina). High-cash households spent MORE on child-specific goods and MORE time on child-specific early-learning activities than low-cash households, and reported lower public-benefit receipt and less residence in poverty.</t>
+        </is>
+      </c>
       <c r="BK80" s="2" t="inlineStr"/>
       <c r="BL80" s="2" t="inlineStr"/>
       <c r="BM80" s="2" t="inlineStr">
@@ -19876,7 +20164,11 @@
       <c r="BG81" s="2" t="inlineStr"/>
       <c r="BH81" s="2" t="inlineStr"/>
       <c r="BI81" s="2" t="inlineStr"/>
-      <c r="BJ81" s="2" t="inlineStr"/>
+      <c r="BJ81" s="2" t="inlineStr">
+        <is>
+          <t>Cluster-RCT (N=2,002 fathers — 786 Rohingya camps, 1,216 host; minimum detectable ES 0.17). The 6-month father-engagement intervention (added to a mother-focused ECD program) positively impacted fathers' parenting (father-reported) and family engagement (father- and mother-reported) and father-reported child social-emotional development vs the mother-only program. | NO main effect on directly-assessed child development; baseline mother-reported stimulation and mother health moderated father-reported child SEL impacts in camps; child gender and baseline stimulation moderated multiple mother-reported child outcomes (treatment effects negative for boys, weakly positive for girls). (CREDI subscale correlations 0.88–0.96.)</t>
+        </is>
+      </c>
       <c r="BK81" s="2" t="inlineStr"/>
       <c r="BL81" s="2" t="inlineStr"/>
       <c r="BM81" s="2" t="inlineStr">
@@ -20132,7 +20424,11 @@
       <c r="BG82" s="2" t="inlineStr"/>
       <c r="BH82" s="2" t="inlineStr"/>
       <c r="BI82" s="2" t="inlineStr"/>
-      <c r="BJ82" s="2" t="inlineStr"/>
+      <c r="BJ82" s="2" t="inlineStr">
+        <is>
+          <t>Qualitative interview study (no statistics; 25 Rohingya fathers aged 23–48, each with a child in BRAC's 0–6 range; Cox's Bazar). Examines fathers' perceptions of children's play in structured (Humanitarian Play Labs) and unstructured (home/surrounding) settings, addressing a gap in heavily-Western, individualistic father-engagement research by examining play, discipline/behavior management and child participation in collective-care, forced-displacement contexts.</t>
+        </is>
+      </c>
       <c r="BK82" s="2" t="inlineStr"/>
       <c r="BL82" s="2" t="inlineStr"/>
       <c r="BM82" s="2" t="inlineStr"/>
@@ -20380,7 +20676,11 @@
           <t>EEG (brain activity)</t>
         </is>
       </c>
-      <c r="BJ83" s="2" t="inlineStr"/>
+      <c r="BJ83" s="2" t="inlineStr">
+        <is>
+          <t>Baby's First Years EEG study (Age-4 wave, mean 4.03 years, SD=0.19; intent-to-treat). Four years of monthly cash ($333 vs $20) produced NO impact on the primary preregistered outcome (aggregated mid-to-high-frequency brain activity) or the secondary outcome frontal gamma power (ES=−.09, p=.266); no significant theta-band effects. | Exploratory preregistered analyses found higher ALPHA power in the high-cash group (no differences in theta, beta or gamma) — suggesting a possible but unconfirmed effect on preschoolers' alpha power that needs replication. (Age-1 EEG sample was limited to N=435 assessed pre-COVID.)</t>
+        </is>
+      </c>
       <c r="BK83" s="2" t="inlineStr"/>
       <c r="BL83" s="2" t="inlineStr"/>
       <c r="BM83" s="2" t="inlineStr">
@@ -20648,7 +20948,11 @@
       <c r="BG84" s="2" t="inlineStr"/>
       <c r="BH84" s="2" t="inlineStr"/>
       <c r="BI84" s="2" t="inlineStr"/>
-      <c r="BJ84" s="2" t="inlineStr"/>
+      <c r="BJ84" s="2" t="inlineStr">
+        <is>
+          <t>Cycle 1 (Mindfulness, 11 weeks) vs HCT-only: significant reduction in sadness dysregulation (ES=-0.30, p=.003) and marginal reduction in reactive aggression (ES=-0.29, p=.029); no impacts on school-related stress, other social-context regulation, behavioral regulation, executive function, social-emotional functioning, or academics. Cycle 1+2 (Mindfulness+Brain Games, 22 weeks): NO overall impacts on any proximal or distal outcome. | Moderation (exploratory, p&lt;.05, unadjusted): Nigerian refugees improved more than Nigerien peers in cognitive inhibitory control from Mindfulness (ES=0.46, p=.017); girls showed steeper declines than boys in school-related stress (ES=-0.31, p=.020), sadness dysregulation (ES=-0.31, p=.002) and reactive aggression (ES=-0.47, p&lt;.001), and greater working-memory gains from full-year SEL (ES=0.22, p=.014). | Baseline disadvantages: refugees &lt; Nigerien children in working memory (b=-0.21, p=.026), social functioning (b=-0.16, p=.038), French literacy (b=-0.25, p=.005) and higher emotional/behavioral problems (b=0.20, p=.007); girls behind boys in working memory (b=-0.16, p=.016) and French literacy (b=-0.13, p=.013).</t>
+        </is>
+      </c>
       <c r="BK84" s="2" t="inlineStr"/>
       <c r="BL84" s="2" t="inlineStr">
         <is>
@@ -20916,7 +21220,11 @@
       <c r="BG85" s="2" t="inlineStr"/>
       <c r="BH85" s="2" t="inlineStr"/>
       <c r="BI85" s="2" t="inlineStr"/>
-      <c r="BJ85" s="2" t="inlineStr"/>
+      <c r="BJ85" s="2" t="inlineStr">
+        <is>
+          <t>Vs 10 weeks, 26 weeks (2 cycles) of HCT marginally improved literacy (adjusted ES=0.04, p=.097, q=.051) and showed no impact on numeracy, but significantly improved externally-observed behavioral regulation (ES=0.31, p&lt;.001, q=.001). | However, 26-week students reported LESS positive perceptions of their public school — less caring/supportive teachers (adjusted ES=-0.89, p&lt;.001), less engaging/motivating climate (ES=-0.83), less respectful/inclusive schools (ES=-0.87) — and of their remedial site (less positive climate ES=-0.24; less engaging/safe ES=-0.15). | Adding skill-targeted SEL activities to 26 weeks increased student-reported school-related stress (ES=0.21; marginal, q=.09 after FDR correction), with marginal trends toward decreased aggressive reaction and higher teacher-reported externalizing, and no impacts on literacy or numeracy.</t>
+        </is>
+      </c>
       <c r="BK85" s="2" t="inlineStr"/>
       <c r="BL85" s="2" t="inlineStr">
         <is>
@@ -21156,7 +21464,11 @@
       <c r="BG86" s="2" t="inlineStr"/>
       <c r="BH86" s="2" t="inlineStr"/>
       <c r="BI86" s="2" t="inlineStr"/>
-      <c r="BJ86" s="2" t="inlineStr"/>
+      <c r="BJ86" s="2" t="inlineStr">
+        <is>
+          <t>Narrative review (no new statistics). Synthesizes evidence largely from the authors' Global TIES for Children / IRC programs — Learning to Read in a Healing Classroom (DR Congo) and Healing Classroom Tutoring + skill-targeted SEL (Lebanon, Niger): SEL-infused remedial programming improved children's learning and some SEL/self-regulation outcomes but often showed NO impact on mental health, a critical distal outcome. | Situates evidence against ~1 in 5 children globally living in conflict-affected areas (≥224 million school-age children affected in 2023) and argues SEL measurement in CAC contexts is hampered by reliance on measures developed in stable, high-income, Western settings — calling for psychometric validation/contextualization and a common mapping framework (the Taxonomy Project).</t>
+        </is>
+      </c>
       <c r="BK86" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -21372,7 +21684,11 @@
       <c r="BG87" s="2" t="inlineStr"/>
       <c r="BH87" s="2" t="inlineStr"/>
       <c r="BI87" s="2" t="inlineStr"/>
-      <c r="BJ87" s="2" t="inlineStr"/>
+      <c r="BJ87" s="2" t="inlineStr">
+        <is>
+          <t>Rapid review (no primary statistics; &gt;42 studies of children &lt;18 across 64 LMICs). Reviewed studies consistently show corporal punishment is associated with negative cognitive and social-emotional outcomes, with NO evidence of any positive developmental outcome; two of three children under five in LMICs are exposed to corporal punishment. | Internal/external validity limitations are common, so stronger multi-site designs are warranted, but current evidence indicates corporal punishment likely increases the risk of detrimental child outcomes in LMICs.</t>
+        </is>
+      </c>
       <c r="BK87" s="2" t="inlineStr"/>
       <c r="BL87" s="2" t="inlineStr">
         <is>
@@ -21620,7 +21936,11 @@
       <c r="BG88" s="2" t="inlineStr"/>
       <c r="BH88" s="2" t="inlineStr"/>
       <c r="BI88" s="2" t="inlineStr"/>
-      <c r="BJ88" s="2" t="inlineStr"/>
+      <c r="BJ88" s="2" t="inlineStr">
+        <is>
+          <t>Cluster-RCT in rural Peru (2,461 caregiver–child dyads). Relative to control, home visits (HVs) increased directly-assessed child development by 0.17 SD (95% CI 0.03–0.30) and the AI-supported digital intervention (DI) by 0.11 SD (95% CI 0.02–0.19) at ~2.5 years; similar magnitudes for caregiver-reported development (HV 0.10 SD; DI 0.12 SD). | HVs increased caregiver-reported stimulation by 0.29 SD and DI by 0.09 SD. At 1/15 of the cost of in-person support, the digital intervention yielded superior cost-effectiveness — suggesting digital platforms are a viable, scalable alternative in resource-constrained settings.</t>
+        </is>
+      </c>
       <c r="BK88" s="2" t="inlineStr"/>
       <c r="BL88" s="2" t="inlineStr"/>
       <c r="BM88" s="2" t="inlineStr"/>
@@ -21828,7 +22148,11 @@
       <c r="BG89" s="2" t="inlineStr"/>
       <c r="BH89" s="2" t="inlineStr"/>
       <c r="BI89" s="2" t="inlineStr"/>
-      <c r="BJ89" s="2" t="inlineStr"/>
+      <c r="BJ89" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review (no primary statistics). Synthesizes evidence on prenatal and early-childhood ambient heat exposure and developmental outcomes, situated in a growing literature linking excessive heat to harms to physical health, mental health, behavior (e.g., violence) and learning (e.g., test-score declines). | Examines how extreme heat during sensitive prenatal and early-childhood periods relates to children's developmental outcomes and identifies evidence gaps and directions for research and policy.</t>
+        </is>
+      </c>
       <c r="BK89" s="2" t="inlineStr"/>
       <c r="BL89" s="2" t="inlineStr"/>
       <c r="BM89" s="2" t="inlineStr"/>
@@ -22056,7 +22380,11 @@
       <c r="BG90" s="2" t="inlineStr"/>
       <c r="BH90" s="2" t="inlineStr"/>
       <c r="BI90" s="2" t="inlineStr"/>
-      <c r="BJ90" s="2" t="inlineStr"/>
+      <c r="BJ90" s="2" t="inlineStr">
+        <is>
+          <t>Across five LMIC longitudinal studies, random-effects and conservative child-fixed-effects models showed family stimulation (caregivers' engagement in nine activities, e.g., reading, playing, singing) predicted increments in children's development: a 1 SD increment in family stimulation related to increments of 0.05 SD (executive function) to 0.08 SD (numeracy, literacy, social-emotional skills). | Study-specific models showed variability, with null associations in two of the five studies — indicating a need for more research on culturally specific caregiver-stimulation practices.</t>
+        </is>
+      </c>
       <c r="BK90" s="2" t="inlineStr"/>
       <c r="BL90" s="2" t="inlineStr"/>
       <c r="BM90" s="2" t="inlineStr">
@@ -22304,7 +22632,11 @@
       <c r="BG91" s="2" t="inlineStr"/>
       <c r="BH91" s="2" t="inlineStr"/>
       <c r="BI91" s="2" t="inlineStr"/>
-      <c r="BJ91" s="2" t="inlineStr"/>
+      <c r="BJ91" s="2" t="inlineStr">
+        <is>
+          <t>Quasi-experimental study leveraging natural variation in timing/location of community homicides (N=3,241 São Paulo 3-year-olds; M age 41 months, 53% female). Recent exposure to community homicides was associated with lower effortful control, higher behavior problems and lower overall developmental performance (d=.05–.20 SD; p=ns–&lt;.001). | Effects were consistent across sociodemographic subgroups but generally largest when violence was geographically proximal (within 600 m of home) and recent (within 2 weeks prior to assessment).</t>
+        </is>
+      </c>
       <c r="BK91" s="2" t="inlineStr"/>
       <c r="BL91" s="2" t="inlineStr"/>
       <c r="BM91" s="2" t="inlineStr">
@@ -22564,7 +22896,11 @@
       <c r="BG92" s="2" t="inlineStr"/>
       <c r="BH92" s="2" t="inlineStr"/>
       <c r="BI92" s="2" t="inlineStr"/>
-      <c r="BJ92" s="2" t="inlineStr"/>
+      <c r="BJ92" s="2" t="inlineStr">
+        <is>
+          <t>Five-year RCT (424 parent–child pairs; outcomes at &lt;12 months, age 3, age 5). Compared with controls, Lifestart parents reported greater knowledge of their child's development (ES=.277, p=.016), higher parenting confidence/self-efficacy (ES=.213, p=.047), and lower parenting-related stress (ES=−.220, p=.045). | NO evidence of change in child development outcomes (cognitive, behavioural, social or emotional) and no consistent differential effects by gender, first-time motherhood, high pre-test anxiety, or low maternal education — consistent with the programme's hypothesized theory of change.</t>
+        </is>
+      </c>
       <c r="BK92" s="2" t="inlineStr"/>
       <c r="BL92" s="2" t="inlineStr">
         <is>
@@ -22776,7 +23112,11 @@
       <c r="BG93" s="2" t="inlineStr"/>
       <c r="BH93" s="2" t="inlineStr"/>
       <c r="BI93" s="2" t="inlineStr"/>
-      <c r="BJ93" s="2" t="inlineStr"/>
+      <c r="BJ93" s="2" t="inlineStr">
+        <is>
+          <t>Commentary (no statistics). Argues decades of evidence show MHPSS interventions can reduce mental distress even in active fragile and conflict-affected settings, yet they remain confined to short-term, externally managed pilots rather than sustainable systems; calls for implementation science and systems strengthening to integrate MHPSS across health, education, and social-protection platforms. (Maria Alejandra Gutierrez-Torres is a co-author.)</t>
+        </is>
+      </c>
       <c r="BK93" s="2" t="inlineStr"/>
       <c r="BL93" s="2" t="inlineStr"/>
       <c r="BM93" s="2" t="inlineStr"/>
@@ -23000,7 +23340,11 @@
       <c r="BG94" s="2" t="inlineStr"/>
       <c r="BH94" s="2" t="inlineStr"/>
       <c r="BI94" s="2" t="inlineStr"/>
-      <c r="BJ94" s="2" t="inlineStr"/>
+      <c r="BJ94" s="2" t="inlineStr">
+        <is>
+          <t>Policy brief (no statistics; Yale Jackson School of Global Affairs). Argues Early Childhood Development is a catalyst for intergenerational peacebuilding and community stability; ECD interventions encompassing learning, stimulation and social cohesion foster skills for peaceful societies, with NUTRITION proposed as a critical entry point. | Synthesizes evidence and offers policy directions for putting children first in peacebuilding and recovery agendas.</t>
+        </is>
+      </c>
       <c r="BK94" s="2" t="inlineStr"/>
       <c r="BL94" s="2" t="inlineStr"/>
       <c r="BM94" s="2" t="inlineStr"/>
@@ -23208,7 +23552,11 @@
       <c r="BG95" s="2" t="inlineStr"/>
       <c r="BH95" s="2" t="inlineStr"/>
       <c r="BI95" s="2" t="inlineStr"/>
-      <c r="BJ95" s="2" t="inlineStr"/>
+      <c r="BJ95" s="2" t="inlineStr">
+        <is>
+          <t>Psychometric evaluation of Save the Children's Remote Assessment of Learning (ReAL) for 5–14-year-olds across six low-resource/crisis-affected countries (N=4,840; ~equal male/female within each country). Assessed inter-rater reliability, factor structure, item slope/difficulty, criterion validity and test–retest reliability. | Moderate evidence that ReAL is valid and reliable for literacy and numeracy (weaker for social-emotional skills); the alpha pilot showed high internal consistency (literacy Cronbach's α≥.86, numeracy α≥.78, SEL α≥.90) — supporting feasible, contextually appropriate remote learning assessment in low-resource and crisis contexts.</t>
+        </is>
+      </c>
       <c r="BK95" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -23432,7 +23780,11 @@
       <c r="BG96" s="2" t="inlineStr"/>
       <c r="BH96" s="2" t="inlineStr"/>
       <c r="BI96" s="2" t="inlineStr"/>
-      <c r="BJ96" s="2" t="inlineStr"/>
+      <c r="BJ96" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; meta-analysis updating Durlak et al. (2011): 424 studies from 53 countries (2008–2020), 252 discrete universal school-based (USB) SEL interventions, 575,361 K-12 students. Compared with controls, students in USB SEL interventions experienced significantly improved skills, attitudes, behaviors, school climate and safety, peer relationships, school functioning, and academic achievement. | Significant heterogeneity in SEL content, intervention features, context and implementation quality moderated student outcomes — calling for a more nuanced, equity-focused understanding of for whom and under what conditions SEL works.</t>
+        </is>
+      </c>
       <c r="BK96" s="2" t="inlineStr"/>
       <c r="BL96" s="2" t="inlineStr">
         <is>
@@ -23644,7 +23996,11 @@
       <c r="BG97" s="2" t="inlineStr"/>
       <c r="BH97" s="2" t="inlineStr"/>
       <c r="BI97" s="2" t="inlineStr"/>
-      <c r="BJ97" s="2" t="inlineStr"/>
+      <c r="BJ97" s="2" t="inlineStr">
+        <is>
+          <t>Perspectives article (no new meta-analytic statistics) drawing on the authors' 13-year systematic review/meta-analysis of universal school-based SEL for K-12 students. Argues the field knows a great deal about variation in SEL program effects but very little about the experiences of students with marginalized and minoritized identities within them. | Details key findings and critical future directions to make SEL genuinely inclusive for gender-, racially-, ethnically-, linguistically-, and ability-minoritized youth.</t>
+        </is>
+      </c>
       <c r="BK97" s="2" t="inlineStr"/>
       <c r="BL97" s="2" t="inlineStr">
         <is>
@@ -23864,7 +24220,11 @@
       <c r="BG98" s="2" t="inlineStr"/>
       <c r="BH98" s="2" t="inlineStr"/>
       <c r="BI98" s="2" t="inlineStr"/>
-      <c r="BJ98" s="2" t="inlineStr"/>
+      <c r="BJ98" s="2" t="inlineStr">
+        <is>
+          <t>US-specific systematic review &amp; meta-analysis (90 studies, 47 discrete programs, 20,626 K-12 students, 2008–2020). Students who participated in universal school-based SEL experienced significantly improved academic achievement, school functioning, and social-emotional outcomes, including significant reductions in emotional distress and externalizing behaviors. | Programs benefited elementary and secondary students equally and had the strongest outcomes when teachers were the implementers; provides nation-specific trends and recommendations for marginalized students (minority gender, racial-ethnic, linguistic, and disability identities).</t>
+        </is>
+      </c>
       <c r="BK98" s="2" t="inlineStr"/>
       <c r="BL98" s="2" t="inlineStr">
         <is>
@@ -24009,7 +24369,7 @@
       <c r="P99" s="2" t="inlineStr"/>
       <c r="Q99" s="2" t="inlineStr">
         <is>
-          <t>258 universal K-12 SEL studies (from 382 screened)</t>
+          <t>40 empirical studies (33,737 students; 76 academic-achievement effect sizes) analyzed, narrowed from 258 screened universal K-12 SEL studies (~9,745 records de-duplicated), grades 1–12, 2008–2020</t>
         </is>
       </c>
       <c r="R99" s="2" t="inlineStr">
@@ -24080,7 +24440,11 @@
       <c r="BG99" s="2" t="inlineStr"/>
       <c r="BH99" s="2" t="inlineStr"/>
       <c r="BI99" s="2" t="inlineStr"/>
-      <c r="BJ99" s="2" t="inlineStr"/>
+      <c r="BJ99" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; meta-analysis (Review of Educational Research): from ~9,745 de-duplicated records and 258 screened universal K-12 SEL studies, the academic-achievement meta-analysis analyzed 40 empirical studies (2008–2020), 33,737 students and 76 effect sizes. | Students in grades 1–12 who participated in universal school-based SEL programs showed significantly better academic achievement than non-participants (g=.101), with significant improvements in BOTH literacy and math across grades — indicating SEL's impact spans academic domains.</t>
+        </is>
+      </c>
       <c r="BK99" s="2" t="inlineStr"/>
       <c r="BL99" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Pruett 2023 row (flagged attribution) + accuracy fixes
- Add fully-coded "Early parenting interventions...network meta-analysis"
  (Costantini et al. 2023, BMJ Mental Health; 59 RCTs, 18,349 participants)
  per user request, filed under Pruett with a prominent ⚠ Notes flag: no
  Kyle Pruett / Yale authorship appears in the paper (14 UK-based authors).
- Accuracy fixes verified against PDFs:
  * EEG paper corrected to its published version — journal Developmental
    Cognitive Neuroscience, DOI 10.1016/j.dcn.2026.101673 (was "PsyArXiv").
  * Added DOI 10.1111/jcpp.13799 (Cuartas/McCoy Brazil community violence).
  * Added DOI 10.1111/cdev.13968 (McCarthy "state of evidence" meta-analysis).
- Now 92 papers; review Excel regenerated (137 verify-flags). Refreshed
  062226ECPCRR.csv.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF99"/>
+  <dimension ref="A1:DF100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -20765,10 +20765,14 @@
       </c>
       <c r="DA83" s="2" t="inlineStr">
         <is>
-          <t>PsyArXiv (OSF Preprints)</t>
-        </is>
-      </c>
-      <c r="DB83" s="3" t="inlineStr"/>
+          <t>Developmental Cognitive Neuroscience</t>
+        </is>
+      </c>
+      <c r="DB83" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.dcn.2026.101673</t>
+        </is>
+      </c>
       <c r="DC83" s="2" t="inlineStr">
         <is>
           <t>https://osf.io/dw2em</t>
@@ -22728,7 +22732,11 @@
           <t>Journal of Child Psychology and Psychiatry</t>
         </is>
       </c>
-      <c r="DB91" s="3" t="inlineStr"/>
+      <c r="DB91" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcpp.13799</t>
+        </is>
+      </c>
       <c r="DC91" s="2" t="inlineStr"/>
       <c r="DD91" s="2" t="inlineStr"/>
       <c r="DE91" s="2" t="inlineStr"/>
@@ -23876,7 +23884,11 @@
           <t>Child Development</t>
         </is>
       </c>
-      <c r="DB96" s="3" t="inlineStr"/>
+      <c r="DB96" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/cdev.13968</t>
+        </is>
+      </c>
       <c r="DC96" s="2" t="inlineStr"/>
       <c r="DD96" s="2" t="inlineStr"/>
       <c r="DE96" s="2" t="inlineStr"/>
@@ -24546,6 +24558,262 @@
         </is>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>Pruett, Kyle — 2023 — Early parenting interventions to prevent internalising problems in children and adolescents: a global systematic review and network meta-analysis</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr"/>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Global (international)</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; network meta-analysis of RCTs (parenting interventions, children &lt;4)</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; network meta-analysis of RCTs (random-effects NMA; a priori taxonomy of parenting interventions; SMDs with 95% credible intervals)</t>
+        </is>
+      </c>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>quantitative</t>
+        </is>
+      </c>
+      <c r="K100" s="2" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>not applicable</t>
+        </is>
+      </c>
+      <c r="O100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr"/>
+      <c r="Q100" s="2" t="inlineStr">
+        <is>
+          <t>59 RCTs (18,349 participants); children younger than 4 years; screened from 20,520 citations (searched to 1 Oct 2022)</t>
+        </is>
+      </c>
+      <c r="R100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (parents/caregivers)</t>
+        </is>
+      </c>
+      <c r="U100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V100" s="2" t="inlineStr"/>
+      <c r="W100" s="2" t="inlineStr">
+        <is>
+          <t>Children younger than 4 years and their parents/caregivers across 59 RCTs (18,349 participants) globally; excluded children born preterm or with intellectual disabilities and families receiving support for current abuse, neglect, or substance misuse</t>
+        </is>
+      </c>
+      <c r="X100" s="2" t="inlineStr"/>
+      <c r="Y100" s="2" t="inlineStr"/>
+      <c r="Z100" s="2" t="inlineStr"/>
+      <c r="AA100" s="2" t="inlineStr"/>
+      <c r="AB100" s="2" t="inlineStr"/>
+      <c r="AC100" s="2" t="inlineStr"/>
+      <c r="AD100" s="2" t="inlineStr"/>
+      <c r="AE100" s="2" t="inlineStr"/>
+      <c r="AF100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (internalising — primary)</t>
+        </is>
+      </c>
+      <c r="AG100" s="2" t="inlineStr"/>
+      <c r="AH100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (internalising problems — primary outcome)</t>
+        </is>
+      </c>
+      <c r="AI100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (externalising problems)</t>
+        </is>
+      </c>
+      <c r="AJ100" s="2" t="inlineStr"/>
+      <c r="AK100" s="2" t="inlineStr"/>
+      <c r="AL100" s="2" t="inlineStr"/>
+      <c r="AM100" s="2" t="inlineStr"/>
+      <c r="AN100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (parental depressive symptoms)</t>
+        </is>
+      </c>
+      <c r="AO100" s="2" t="inlineStr"/>
+      <c r="AP100" s="2" t="inlineStr"/>
+      <c r="AQ100" s="2" t="inlineStr"/>
+      <c r="AR100" s="2" t="inlineStr"/>
+      <c r="AS100" s="2" t="inlineStr"/>
+      <c r="AT100" s="2" t="inlineStr"/>
+      <c r="AU100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (parental sense of self-efficacy)</t>
+        </is>
+      </c>
+      <c r="AV100" s="2" t="inlineStr"/>
+      <c r="AW100" s="2" t="inlineStr"/>
+      <c r="AX100" s="2" t="inlineStr"/>
+      <c r="AY100" s="2" t="inlineStr"/>
+      <c r="AZ100" s="2" t="inlineStr"/>
+      <c r="BA100" s="2" t="inlineStr"/>
+      <c r="BB100" s="2" t="inlineStr"/>
+      <c r="BC100" s="2" t="inlineStr"/>
+      <c r="BD100" s="2" t="inlineStr"/>
+      <c r="BE100" s="2" t="inlineStr"/>
+      <c r="BF100" s="2" t="inlineStr"/>
+      <c r="BG100" s="2" t="inlineStr"/>
+      <c r="BH100" s="2" t="inlineStr"/>
+      <c r="BI100" s="2" t="inlineStr"/>
+      <c r="BJ100" s="2" t="inlineStr">
+        <is>
+          <t>Network meta-analysis of 59 RCTs (18,349 participants; children &lt;4 years; screened from 20,520 citations; random-effects NMA estimating SMDs with 95% credible intervals). Parenting interventions focusing on the dyadic relationship (SMD=−0.26, 95% CrI −0.43 to −0.08) and those with mixed focus (SMD=−0.09, −0.17 to −0.02) were more effective than treatment-as-usual (TAU) at reducing child internalising problems at the first time point available. | All interventions were more effective than waitlist, which itself INCREASED internalising risk vs TAU (SMD=0.36, 95% CrI 0.19 to 0.52). Weak evidence that all parenting interventions improved parental self-efficacy and that home-visiting reduced parental depressive symptoms; no moderators or intervention components affecting effectiveness were identified. Most studies were rated 'high risk' or 'some concerns' for bias — findings should be interpreted with caution.</t>
+        </is>
+      </c>
+      <c r="BK100" s="2" t="inlineStr"/>
+      <c r="BL100" s="2" t="inlineStr"/>
+      <c r="BM100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BN100" s="2" t="inlineStr"/>
+      <c r="BO100" s="2" t="inlineStr"/>
+      <c r="BP100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (tested moderators/components — none identified)</t>
+        </is>
+      </c>
+      <c r="BQ100" s="2" t="inlineStr"/>
+      <c r="BR100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (network meta-analysis of intervention effects)</t>
+        </is>
+      </c>
+      <c r="BS100" s="2" t="inlineStr"/>
+      <c r="BT100" s="2" t="inlineStr"/>
+      <c r="BU100" s="2" t="inlineStr"/>
+      <c r="BV100" s="2" t="inlineStr"/>
+      <c r="BW100" s="2" t="inlineStr"/>
+      <c r="BX100" s="2" t="inlineStr"/>
+      <c r="BY100" s="2" t="inlineStr"/>
+      <c r="BZ100" s="2" t="inlineStr"/>
+      <c r="CA100" s="2" t="inlineStr"/>
+      <c r="CB100" s="2" t="inlineStr"/>
+      <c r="CC100" s="2" t="inlineStr"/>
+      <c r="CD100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (parental depressive symptoms)</t>
+        </is>
+      </c>
+      <c r="CE100" s="2" t="inlineStr"/>
+      <c r="CF100" s="2" t="inlineStr"/>
+      <c r="CG100" s="2" t="inlineStr"/>
+      <c r="CH100" s="2" t="inlineStr"/>
+      <c r="CI100" s="2" t="inlineStr"/>
+      <c r="CJ100" s="2" t="inlineStr"/>
+      <c r="CK100" s="2" t="inlineStr"/>
+      <c r="CL100" s="2" t="inlineStr"/>
+      <c r="CM100" s="2" t="inlineStr"/>
+      <c r="CN100" s="2" t="inlineStr"/>
+      <c r="CO100" s="2" t="inlineStr"/>
+      <c r="CP100" s="2" t="inlineStr"/>
+      <c r="CQ100" s="2" t="inlineStr"/>
+      <c r="CR100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (network diagrams / forest plots)</t>
+        </is>
+      </c>
+      <c r="CS100" s="2" t="inlineStr">
+        <is>
+          <t>Yes (a priori taxonomy of parenting interventions)</t>
+        </is>
+      </c>
+      <c r="CT100" s="3" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; network meta-analysis (BMJ Mental Health) comparing types of early parenting intervention (a priori taxonomy) for preventing child internalising problems; 59 RCTs, 18,349 participants. Relationship-focused and mixed interventions reduced internalising problems vs TAU; the waitlist comparator increased risk, with implications for referral-to-support waiting times. ⚠ ATTRIBUTION TO VERIFY: No author named Kyle Pruett (and no Yale affiliation) appears anywhere in this paper. Authors are Costantini, López-López, Caldwell, Campbell, Hadjipanayi, Cantrell, Thomas, Badmann, Paul, James, Cordero, Jewell, Evans &amp; Pearson (UCL/Bristol/Manchester Met). Filed under Pruett per user request; ECPC member connection needs confirming.</t>
+        </is>
+      </c>
+      <c r="CU100" s="2" t="inlineStr"/>
+      <c r="CV100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW100" s="2" t="inlineStr">
+        <is>
+          <t>Pruett, Kyle</t>
+        </is>
+      </c>
+      <c r="CX100" s="2" t="inlineStr">
+        <is>
+          <t>Yale Child Study Center</t>
+        </is>
+      </c>
+      <c r="CY100" s="2" t="inlineStr">
+        <is>
+          <t>Ilaria Costantini, José A López-López, Deborah Caldwell, Amy Campbell, Veronica Hadjipanayi, Sarah J Cantrell, Tallulah Thomas, Nathan Badmann, Elise Paul, Deborah M James, Miguel Cordero, Tom Jewell, Jonathan Evans, Rebecca M Pearson</t>
+        </is>
+      </c>
+      <c r="CZ100" s="2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="DA100" s="2" t="inlineStr">
+        <is>
+          <t>BMJ Mental Health</t>
+        </is>
+      </c>
+      <c r="DB100" s="2" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/bmjment-2023-300811</t>
+        </is>
+      </c>
+      <c r="DC100" s="2" t="inlineStr">
+        <is>
+          <t>https://mentalhealth.bmj.com/content/26/1/e300811.full.pdf</t>
+        </is>
+      </c>
+      <c r="DD100" s="2" t="inlineStr"/>
+      <c r="DE100" s="2" t="inlineStr"/>
+      <c r="DF100" s="2" t="inlineStr">
+        <is>
+          <t>Question: We compared the effectiveness of different types of parenting interventions based on an a priori taxonomy, and the impact of waitlists versus treatment as usual (TAU), in reducing child internalising problems. Study selection and analysis: Systematic review and network meta-analysis of published and unpublished randomised controlled trials (RCTs) until 1 October 2022 that investigated parenting interventions with children younger than 4 years; excluded children born preterm or with intellectual disabilities and families receiving support for current abuse, neglect, and substance misuse. Random-effects network meta-analysis estimated standardised mean differences (SMDs) with 95% credible intervals (CrIs). Findings: Of 20,520 citations identified, 59 RCTs (18,349 participants) were eligible. Parenting interventions focusing on the dyadic relationship (SMD: −0.26, 95% CrI: −0.43 to −0.08) and those with mixed focus (−0.09, −0.17 to −0.02) were more effective in reducing internalising problems than TAU at the first time point; all interventions were more effective than waitlist, which increased the risk of internalising problems compared with TAU (0.36, 0.19 to 0.52). There was weak evidence that all parenting interventions improved self-efficacy and that home visiting reduced parental depressive symptoms. Most studies were rated 'high risk' or 'some concerns' for bias. Conclusions: Preliminary evidence that relationship-focused and mixed parenting interventions reduced child internalising problems, and the waitlist comparator increased internalising problems with implications for waiting times between referral and support. Given the high risk of bias of most included studies, findings should be interpreted with caution.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Complete: stage 103-paper data, review Excel, new PDFs; drop stray backups
Fixes the prior commit that only captured the CSV rename. Stages the actual
103-paper dataset (ecpc_unga_FILLED.csv + 07072026ECPCRR.csv), regenerated
review Excel, and the new backing PDFs (Foundations for a Peaceful World book
+ Feder/Fitzpatrick/Vasic chapters, UNICEF Power of Play). Removes accidental
.bak/.bak2 working backups from version control.

Note: a stray duplicate pdfs/Aber/Salah/UNICEF-The-Power-of-Play_June-2026.pdf
was left untracked (identical to pdfs/Salah/ copy) pending user decision.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF107"/>
+  <dimension ref="A1:DF111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -26362,6 +26362,898 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Feder, Joshua — 2025 — The Early Years Media Initiative for Children – Revised Toddler Module: Building Social-Emotional Resilience (in 'Foundations for a Peaceful World', Ch. 5)</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr"/>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom (Northern Ireland); scaling nationally &amp; internationally</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Early-years settings; Media Initiative for Children – toddler module</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>-5.9</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter (programme description; reports a controlled trial of the Revised Toddler Module)</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr"/>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>Early Years Media Initiative for Children – Revised Toddler Module (Building Social-Emotional Resilience)</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (controlled trial)</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="O108" s="2" t="inlineStr"/>
+      <c r="P108" s="2" t="inlineStr"/>
+      <c r="Q108" s="2" t="inlineStr">
+        <is>
+          <t>Toddlers, early-years staff and parents in the Media Initiative toddler module; a controlled trial is referenced (programme now scaling nationally/internationally)</t>
+        </is>
+      </c>
+      <c r="R108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S108" s="2" t="inlineStr"/>
+      <c r="T108" s="2" t="inlineStr"/>
+      <c r="U108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W108" s="2" t="inlineStr">
+        <is>
+          <t>Toddlers, early-years staff, and parents participating in the Media Initiative for Children Revised Toddler Module (Northern Ireland; scaling nationally and internationally)</t>
+        </is>
+      </c>
+      <c r="X108" s="2" t="inlineStr"/>
+      <c r="Y108" s="2" t="inlineStr"/>
+      <c r="Z108" s="2" t="inlineStr"/>
+      <c r="AA108" s="2" t="inlineStr"/>
+      <c r="AB108" s="2" t="inlineStr"/>
+      <c r="AC108" s="2" t="inlineStr"/>
+      <c r="AD108" s="2" t="inlineStr"/>
+      <c r="AE108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (children's social-emotional functioning)</t>
+        </is>
+      </c>
+      <c r="AF108" s="2" t="inlineStr"/>
+      <c r="AG108" s="2" t="inlineStr"/>
+      <c r="AH108" s="2" t="inlineStr"/>
+      <c r="AI108" s="2" t="inlineStr"/>
+      <c r="AJ108" s="2" t="inlineStr"/>
+      <c r="AK108" s="2" t="inlineStr"/>
+      <c r="AL108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (self-regulation / co-regulation; problem-solving resilience)</t>
+        </is>
+      </c>
+      <c r="AM108" s="2" t="inlineStr"/>
+      <c r="AN108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (decreased parent stress)</t>
+        </is>
+      </c>
+      <c r="AO108" s="2" t="inlineStr"/>
+      <c r="AP108" s="2" t="inlineStr"/>
+      <c r="AQ108" s="2" t="inlineStr"/>
+      <c r="AR108" s="2" t="inlineStr"/>
+      <c r="AS108" s="2" t="inlineStr"/>
+      <c r="AT108" s="2" t="inlineStr"/>
+      <c r="AU108" s="2" t="inlineStr"/>
+      <c r="AV108" s="2" t="inlineStr"/>
+      <c r="AW108" s="2" t="inlineStr"/>
+      <c r="AX108" s="2" t="inlineStr"/>
+      <c r="AY108" s="2" t="inlineStr"/>
+      <c r="AZ108" s="2" t="inlineStr"/>
+      <c r="BA108" s="2" t="inlineStr"/>
+      <c r="BB108" s="2" t="inlineStr"/>
+      <c r="BC108" s="2" t="inlineStr"/>
+      <c r="BD108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (decreased staff stress)</t>
+        </is>
+      </c>
+      <c r="BE108" s="2" t="inlineStr"/>
+      <c r="BF108" s="2" t="inlineStr"/>
+      <c r="BG108" s="2" t="inlineStr"/>
+      <c r="BH108" s="2" t="inlineStr"/>
+      <c r="BI108" s="2" t="inlineStr"/>
+      <c r="BJ108" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter describing the Early Years Media Initiative for Children Revised Toddler Module (a 2.5-hour start-of-year staff training covering 12 topics with 12 micro-training videos; co-regulation techniques for managing tantrums; a 'Building Problem-Solving Resilience' section). | A controlled trial demonstrated marked improvements in children's social-emotional functioning and decreased stress among staff and parents; the programme is now being scaled nationwide and internationally.</t>
+        </is>
+      </c>
+      <c r="BK108" s="2" t="inlineStr"/>
+      <c r="BL108" s="2" t="inlineStr"/>
+      <c r="BM108" s="2" t="inlineStr"/>
+      <c r="BN108" s="2" t="inlineStr"/>
+      <c r="BO108" s="2" t="inlineStr"/>
+      <c r="BP108" s="2" t="inlineStr"/>
+      <c r="BQ108" s="2" t="inlineStr"/>
+      <c r="BR108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BS108" s="2" t="inlineStr"/>
+      <c r="BT108" s="2" t="inlineStr"/>
+      <c r="BU108" s="2" t="inlineStr"/>
+      <c r="BV108" s="2" t="inlineStr"/>
+      <c r="BW108" s="2" t="inlineStr"/>
+      <c r="BX108" s="2" t="inlineStr"/>
+      <c r="BY108" s="2" t="inlineStr"/>
+      <c r="BZ108" s="2" t="inlineStr"/>
+      <c r="CA108" s="2" t="inlineStr"/>
+      <c r="CB108" s="2" t="inlineStr"/>
+      <c r="CC108" s="2" t="inlineStr"/>
+      <c r="CD108" s="2" t="inlineStr"/>
+      <c r="CE108" s="2" t="inlineStr"/>
+      <c r="CF108" s="2" t="inlineStr"/>
+      <c r="CG108" s="2" t="inlineStr"/>
+      <c r="CH108" s="2" t="inlineStr"/>
+      <c r="CI108" s="2" t="inlineStr"/>
+      <c r="CJ108" s="2" t="inlineStr"/>
+      <c r="CK108" s="2" t="inlineStr"/>
+      <c r="CL108" s="2" t="inlineStr"/>
+      <c r="CM108" s="2" t="inlineStr"/>
+      <c r="CN108" s="2" t="inlineStr"/>
+      <c r="CO108" s="2" t="inlineStr"/>
+      <c r="CP108" s="2" t="inlineStr"/>
+      <c r="CQ108" s="2" t="inlineStr"/>
+      <c r="CR108" s="2" t="inlineStr"/>
+      <c r="CS108" s="2" t="inlineStr">
+        <is>
+          <t>Yes (programme model)</t>
+        </is>
+      </c>
+      <c r="CT108" s="2" t="inlineStr">
+        <is>
+          <t>Chapter 5 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation. Chapter authors: Joshua D. Feder, Z. Kernohan-Neely, Zach Davis.</t>
+        </is>
+      </c>
+      <c r="CU108" s="2" t="inlineStr"/>
+      <c r="CV108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW108" s="2" t="inlineStr">
+        <is>
+          <t>Feder, Joshua</t>
+        </is>
+      </c>
+      <c r="CX108" s="2" t="inlineStr">
+        <is>
+          <t>Media Initiative for Children / ECPC (book co-editor)</t>
+        </is>
+      </c>
+      <c r="CY108" s="2" t="inlineStr">
+        <is>
+          <t>Joshua D. Feder, Z. Kernohan-Neely, Zach Davis</t>
+        </is>
+      </c>
+      <c r="CZ108" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="DA108" s="2" t="inlineStr">
+        <is>
+          <t>Foundations for a Peaceful World (book chapter) — Early Years / ACEV</t>
+        </is>
+      </c>
+      <c r="DB108" s="3" t="inlineStr"/>
+      <c r="DC108" s="2" t="inlineStr"/>
+      <c r="DD108" s="2" t="inlineStr"/>
+      <c r="DE108" s="2" t="inlineStr"/>
+      <c r="DF108" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter presenting the Early Years Media Initiative for Children Revised Toddler Module, which builds toddlers' social-emotional resilience through staff training (12 topics, micro-training videos), co-regulation techniques, and problem-solving activities. A controlled trial showed marked improvements in children's social-emotional functioning and reduced stress among staff and parents; the programme is being scaled nationally and internationally.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>Fitzpatrick, Siobhan — 2025 — Developing a culture of respecting difference with young children, their families and communities in Northern Ireland (in 'Foundations for a Peaceful World', Ch. 1)</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr"/>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom (Northern Ireland)</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>Early Years NI; Media Initiative for Children – Respecting Difference programme</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>-5.9</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter (programme description; references a large RCT and qualitative evaluations)</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr"/>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>Media Initiative for Children – Respecting Difference Programme (Early Years, Northern Ireland)</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr"/>
+      <c r="N109" s="2" t="inlineStr"/>
+      <c r="O109" s="2" t="inlineStr"/>
+      <c r="P109" s="2" t="inlineStr"/>
+      <c r="Q109" s="2" t="inlineStr">
+        <is>
+          <t>Young children, their families and communities in Northern Ireland engaged in the Respecting Difference programme; a large RCT and qualitative evaluations are referenced</t>
+        </is>
+      </c>
+      <c r="R109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S109" s="2" t="inlineStr"/>
+      <c r="T109" s="2" t="inlineStr"/>
+      <c r="U109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W109" s="2" t="inlineStr">
+        <is>
+          <t>Young children and their families and communities in (divided) Northern Ireland engaged in the Early Years Respecting Difference programme</t>
+        </is>
+      </c>
+      <c r="X109" s="2" t="inlineStr"/>
+      <c r="Y109" s="2" t="inlineStr"/>
+      <c r="Z109" s="2" t="inlineStr"/>
+      <c r="AA109" s="2" t="inlineStr"/>
+      <c r="AB109" s="2" t="inlineStr"/>
+      <c r="AC109" s="2" t="inlineStr"/>
+      <c r="AD109" s="2" t="inlineStr"/>
+      <c r="AE109" s="2" t="inlineStr">
+        <is>
+          <t>Yes (respect for difference / social-emotional)</t>
+        </is>
+      </c>
+      <c r="AF109" s="2" t="inlineStr"/>
+      <c r="AG109" s="2" t="inlineStr"/>
+      <c r="AH109" s="2" t="inlineStr"/>
+      <c r="AI109" s="2" t="inlineStr"/>
+      <c r="AJ109" s="2" t="inlineStr"/>
+      <c r="AK109" s="2" t="inlineStr"/>
+      <c r="AL109" s="2" t="inlineStr"/>
+      <c r="AM109" s="2" t="inlineStr"/>
+      <c r="AN109" s="2" t="inlineStr"/>
+      <c r="AO109" s="2" t="inlineStr">
+        <is>
+          <t>Yes (respect for diversity)</t>
+        </is>
+      </c>
+      <c r="AP109" s="2" t="inlineStr"/>
+      <c r="AQ109" s="2" t="inlineStr"/>
+      <c r="AR109" s="2" t="inlineStr"/>
+      <c r="AS109" s="2" t="inlineStr"/>
+      <c r="AT109" s="2" t="inlineStr"/>
+      <c r="AU109" s="2" t="inlineStr"/>
+      <c r="AV109" s="2" t="inlineStr"/>
+      <c r="AW109" s="2" t="inlineStr"/>
+      <c r="AX109" s="2" t="inlineStr"/>
+      <c r="AY109" s="2" t="inlineStr"/>
+      <c r="AZ109" s="2" t="inlineStr"/>
+      <c r="BA109" s="2" t="inlineStr"/>
+      <c r="BB109" s="2" t="inlineStr"/>
+      <c r="BC109" s="2" t="inlineStr"/>
+      <c r="BD109" s="2" t="inlineStr"/>
+      <c r="BE109" s="2" t="inlineStr"/>
+      <c r="BF109" s="2" t="inlineStr"/>
+      <c r="BG109" s="2" t="inlineStr"/>
+      <c r="BH109" s="2" t="inlineStr"/>
+      <c r="BI109" s="2" t="inlineStr"/>
+      <c r="BJ109" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter describing how Early Years – the organisation for young children in Northern Ireland – pioneered a culture of respect for difference among young children, their families and communities through its Media Initiative for Children / Respecting Difference programme in a historically divided society. | The approach has been subjected to rigorous independent research and evaluation, including a large randomised controlled trial and a range of qualitative evaluations. (Author Siobhan Fitzpatrick is a founder member and vice-chairperson of the Early Childhood Peace Consortium and of the International Network on Peacebuilding with Young Children.)</t>
+        </is>
+      </c>
+      <c r="BK109" s="2" t="inlineStr"/>
+      <c r="BL109" s="2" t="inlineStr"/>
+      <c r="BM109" s="2" t="inlineStr"/>
+      <c r="BN109" s="2" t="inlineStr"/>
+      <c r="BO109" s="2" t="inlineStr"/>
+      <c r="BP109" s="2" t="inlineStr"/>
+      <c r="BQ109" s="2" t="inlineStr"/>
+      <c r="BR109" s="2" t="inlineStr"/>
+      <c r="BS109" s="2" t="inlineStr"/>
+      <c r="BT109" s="2" t="inlineStr"/>
+      <c r="BU109" s="2" t="inlineStr"/>
+      <c r="BV109" s="2" t="inlineStr"/>
+      <c r="BW109" s="2" t="inlineStr"/>
+      <c r="BX109" s="2" t="inlineStr"/>
+      <c r="BY109" s="2" t="inlineStr"/>
+      <c r="BZ109" s="2" t="inlineStr"/>
+      <c r="CA109" s="2" t="inlineStr"/>
+      <c r="CB109" s="2" t="inlineStr"/>
+      <c r="CC109" s="2" t="inlineStr"/>
+      <c r="CD109" s="2" t="inlineStr"/>
+      <c r="CE109" s="2" t="inlineStr"/>
+      <c r="CF109" s="2" t="inlineStr"/>
+      <c r="CG109" s="2" t="inlineStr"/>
+      <c r="CH109" s="2" t="inlineStr"/>
+      <c r="CI109" s="2" t="inlineStr"/>
+      <c r="CJ109" s="2" t="inlineStr"/>
+      <c r="CK109" s="2" t="inlineStr"/>
+      <c r="CL109" s="2" t="inlineStr"/>
+      <c r="CM109" s="2" t="inlineStr"/>
+      <c r="CN109" s="2" t="inlineStr"/>
+      <c r="CO109" s="2" t="inlineStr"/>
+      <c r="CP109" s="2" t="inlineStr"/>
+      <c r="CQ109" s="2" t="inlineStr"/>
+      <c r="CR109" s="2" t="inlineStr"/>
+      <c r="CS109" s="2" t="inlineStr">
+        <is>
+          <t>Yes (Respecting Difference approach)</t>
+        </is>
+      </c>
+      <c r="CT109" s="2" t="inlineStr">
+        <is>
+          <t>Chapter 1 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation.</t>
+        </is>
+      </c>
+      <c r="CU109" s="2" t="inlineStr"/>
+      <c r="CV109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW109" s="2" t="inlineStr">
+        <is>
+          <t>Fitzpatrick, Siobhan</t>
+        </is>
+      </c>
+      <c r="CX109" s="2" t="inlineStr">
+        <is>
+          <t>Early Years – the organisation for young children (Northern Ireland); ECPC</t>
+        </is>
+      </c>
+      <c r="CY109" s="2" t="inlineStr">
+        <is>
+          <t>Siobhan Fitzpatrick</t>
+        </is>
+      </c>
+      <c r="CZ109" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="DA109" s="2" t="inlineStr">
+        <is>
+          <t>Foundations for a Peaceful World (book chapter) — Early Years / ACEV</t>
+        </is>
+      </c>
+      <c r="DB109" s="3" t="inlineStr"/>
+      <c r="DC109" s="2" t="inlineStr"/>
+      <c r="DD109" s="2" t="inlineStr"/>
+      <c r="DE109" s="2" t="inlineStr"/>
+      <c r="DF109" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter describing how Early Years (Northern Ireland) pioneered a culture of respecting difference with young children, their families and communities through the Media Initiative for Children / Respecting Difference programme. The approach has been evaluated with rigorous independent research, including a large randomised controlled trial and qualitative evaluations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>Vasic, Ljiljana — 2025 — Active Development of Respect for Diversity from Early Years in Serbia and the Western Balkans (in 'Foundations for a Peaceful World', Ch. 7)</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr"/>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Serbia (and the Western Balkans)</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Pomoć deci (Children &amp; Youth Support Organisation); Media Initiative adaptation</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>44.79</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>20.45</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter (programme description; cross-context adaptation/scale-up narrative)</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr"/>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>qualitative</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>Media Initiative for Children adapted in Serbia/Western Balkans (Pomoć deci)</t>
+        </is>
+      </c>
+      <c r="M110" s="2" t="inlineStr"/>
+      <c r="N110" s="2" t="inlineStr"/>
+      <c r="O110" s="2" t="inlineStr"/>
+      <c r="P110" s="2" t="inlineStr"/>
+      <c r="Q110" s="2" t="inlineStr">
+        <is>
+          <t>Young children in divided communities across Serbia and the Western Balkans (ethnic, religious, economic and language divisions), including children with multiple/intersecting differences</t>
+        </is>
+      </c>
+      <c r="R110" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S110" s="2" t="inlineStr"/>
+      <c r="T110" s="2" t="inlineStr"/>
+      <c r="U110" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V110" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W110" s="2" t="inlineStr">
+        <is>
+          <t>Young children (including those with multiple/intersecting differences, and children of displaced families) in divided communities across Serbia and the Western Balkans</t>
+        </is>
+      </c>
+      <c r="X110" s="2" t="inlineStr"/>
+      <c r="Y110" s="2" t="inlineStr"/>
+      <c r="Z110" s="2" t="inlineStr"/>
+      <c r="AA110" s="2" t="inlineStr"/>
+      <c r="AB110" s="2" t="inlineStr"/>
+      <c r="AC110" s="2" t="inlineStr"/>
+      <c r="AD110" s="2" t="inlineStr"/>
+      <c r="AE110" s="2" t="inlineStr">
+        <is>
+          <t>Yes (respect for diversity / social-emotional)</t>
+        </is>
+      </c>
+      <c r="AF110" s="2" t="inlineStr"/>
+      <c r="AG110" s="2" t="inlineStr"/>
+      <c r="AH110" s="2" t="inlineStr"/>
+      <c r="AI110" s="2" t="inlineStr"/>
+      <c r="AJ110" s="2" t="inlineStr"/>
+      <c r="AK110" s="2" t="inlineStr"/>
+      <c r="AL110" s="2" t="inlineStr"/>
+      <c r="AM110" s="2" t="inlineStr"/>
+      <c r="AN110" s="2" t="inlineStr"/>
+      <c r="AO110" s="2" t="inlineStr">
+        <is>
+          <t>Yes (respect for diversity)</t>
+        </is>
+      </c>
+      <c r="AP110" s="2" t="inlineStr"/>
+      <c r="AQ110" s="2" t="inlineStr"/>
+      <c r="AR110" s="2" t="inlineStr"/>
+      <c r="AS110" s="2" t="inlineStr"/>
+      <c r="AT110" s="2" t="inlineStr"/>
+      <c r="AU110" s="2" t="inlineStr"/>
+      <c r="AV110" s="2" t="inlineStr"/>
+      <c r="AW110" s="2" t="inlineStr"/>
+      <c r="AX110" s="2" t="inlineStr"/>
+      <c r="AY110" s="2" t="inlineStr"/>
+      <c r="AZ110" s="2" t="inlineStr"/>
+      <c r="BA110" s="2" t="inlineStr"/>
+      <c r="BB110" s="2" t="inlineStr"/>
+      <c r="BC110" s="2" t="inlineStr"/>
+      <c r="BD110" s="2" t="inlineStr"/>
+      <c r="BE110" s="2" t="inlineStr"/>
+      <c r="BF110" s="2" t="inlineStr"/>
+      <c r="BG110" s="2" t="inlineStr"/>
+      <c r="BH110" s="2" t="inlineStr"/>
+      <c r="BI110" s="2" t="inlineStr"/>
+      <c r="BJ110" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter describing how the Media Initiative for Children (originating in divided Northern Ireland) inspired a strategic approach to actively developing respect for diversity from the early years in Serbia and the Western Balkans, implemented by Pomoć deci (Children &amp; Youth Support Organisation). | It addresses ethnic, religious, economic and language-based divisions—especially difficult for children with multiple/intersecting differences and for displaced families not accepted by local populations. (Author Ljiljana Vasic has led Pomoć deci for ~20 years and represents it in the International Network on Peacebuilding for Young Children and Eurochild.)</t>
+        </is>
+      </c>
+      <c r="BK110" s="2" t="inlineStr"/>
+      <c r="BL110" s="2" t="inlineStr"/>
+      <c r="BM110" s="2" t="inlineStr"/>
+      <c r="BN110" s="2" t="inlineStr"/>
+      <c r="BO110" s="2" t="inlineStr"/>
+      <c r="BP110" s="2" t="inlineStr"/>
+      <c r="BQ110" s="2" t="inlineStr"/>
+      <c r="BR110" s="2" t="inlineStr"/>
+      <c r="BS110" s="2" t="inlineStr"/>
+      <c r="BT110" s="2" t="inlineStr"/>
+      <c r="BU110" s="2" t="inlineStr"/>
+      <c r="BV110" s="2" t="inlineStr"/>
+      <c r="BW110" s="2" t="inlineStr"/>
+      <c r="BX110" s="2" t="inlineStr"/>
+      <c r="BY110" s="2" t="inlineStr"/>
+      <c r="BZ110" s="2" t="inlineStr"/>
+      <c r="CA110" s="2" t="inlineStr"/>
+      <c r="CB110" s="2" t="inlineStr"/>
+      <c r="CC110" s="2" t="inlineStr"/>
+      <c r="CD110" s="2" t="inlineStr"/>
+      <c r="CE110" s="2" t="inlineStr"/>
+      <c r="CF110" s="2" t="inlineStr"/>
+      <c r="CG110" s="2" t="inlineStr"/>
+      <c r="CH110" s="2" t="inlineStr"/>
+      <c r="CI110" s="2" t="inlineStr"/>
+      <c r="CJ110" s="2" t="inlineStr"/>
+      <c r="CK110" s="2" t="inlineStr"/>
+      <c r="CL110" s="2" t="inlineStr"/>
+      <c r="CM110" s="2" t="inlineStr"/>
+      <c r="CN110" s="2" t="inlineStr"/>
+      <c r="CO110" s="2" t="inlineStr"/>
+      <c r="CP110" s="2" t="inlineStr"/>
+      <c r="CQ110" s="2" t="inlineStr"/>
+      <c r="CR110" s="2" t="inlineStr"/>
+      <c r="CS110" s="2" t="inlineStr">
+        <is>
+          <t>Yes (adaptation/strategy model)</t>
+        </is>
+      </c>
+      <c r="CT110" s="2" t="inlineStr">
+        <is>
+          <t>Chapter 7 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation.</t>
+        </is>
+      </c>
+      <c r="CU110" s="2" t="inlineStr"/>
+      <c r="CV110" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW110" s="2" t="inlineStr">
+        <is>
+          <t>Vasic, Ljiljana</t>
+        </is>
+      </c>
+      <c r="CX110" s="2" t="inlineStr">
+        <is>
+          <t>Pomoć deci (Children &amp; Youth Support Organisation), Serbia; INPB</t>
+        </is>
+      </c>
+      <c r="CY110" s="2" t="inlineStr">
+        <is>
+          <t>Ljiljana Vasic</t>
+        </is>
+      </c>
+      <c r="CZ110" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="DA110" s="2" t="inlineStr">
+        <is>
+          <t>Foundations for a Peaceful World (book chapter) — Early Years / ACEV</t>
+        </is>
+      </c>
+      <c r="DB110" s="3" t="inlineStr"/>
+      <c r="DC110" s="2" t="inlineStr"/>
+      <c r="DD110" s="2" t="inlineStr"/>
+      <c r="DE110" s="2" t="inlineStr"/>
+      <c r="DF110" s="2" t="inlineStr">
+        <is>
+          <t>Book chapter describing how inspiration from the Media Initiative for Children in Northern Ireland developed into a strategic approach to actively develop respect for diversity from the early years in Serbia and the Western Balkans, led by Pomoć deci. It addresses ethnic, religious, economic and language divisions, particularly for children with multiple differences and displaced families.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>Salah — 2026 — The Power of Play: A Global Data Story (UNICEF Office of Strategy and Evidence – Innocenti)</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr"/>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Global (93 countries)</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>Cross-national analysis of children's play &amp; availability of playthings (MICS-based)</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr"/>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Global data story / descriptive cross-national analysis (internationally comparable MICS data; children aged 2–4)</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>quantitative</t>
+        </is>
+      </c>
+      <c r="K111" s="2" t="inlineStr">
+        <is>
+          <t>observational</t>
+        </is>
+      </c>
+      <c r="L111" s="2" t="inlineStr"/>
+      <c r="M111" s="2" t="inlineStr"/>
+      <c r="N111" s="2" t="inlineStr"/>
+      <c r="O111" s="2" t="inlineStr"/>
+      <c r="P111" s="2" t="inlineStr"/>
+      <c r="Q111" s="2" t="inlineStr">
+        <is>
+          <t>Estimates based on data collected 2010–2024 for 93 countries covering ~60% of the global under-5 population; internationally comparable play data available for children aged 2–4</t>
+        </is>
+      </c>
+      <c r="R111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S111" s="2" t="inlineStr"/>
+      <c r="T111" s="2" t="inlineStr"/>
+      <c r="U111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V111" s="2" t="inlineStr"/>
+      <c r="W111" s="2" t="inlineStr">
+        <is>
+          <t>Children under age 5 (internationally comparable play data for ages 2–4) and caregivers across 93 countries (MICS-based); regional population coverage &gt;50% for Eastern Europe/Central Asia and sub-Saharan Africa, 46% for Latin America &amp; the Caribbean</t>
+        </is>
+      </c>
+      <c r="X111" s="2" t="inlineStr"/>
+      <c r="Y111" s="2" t="inlineStr"/>
+      <c r="Z111" s="2" t="inlineStr"/>
+      <c r="AA111" s="2" t="inlineStr">
+        <is>
+          <t>Yes (cognitive development via play)</t>
+        </is>
+      </c>
+      <c r="AB111" s="2" t="inlineStr"/>
+      <c r="AC111" s="2" t="inlineStr"/>
+      <c r="AD111" s="2" t="inlineStr"/>
+      <c r="AE111" s="2" t="inlineStr">
+        <is>
+          <t>Yes (social-emotional development via play)</t>
+        </is>
+      </c>
+      <c r="AF111" s="2" t="inlineStr"/>
+      <c r="AG111" s="2" t="inlineStr"/>
+      <c r="AH111" s="2" t="inlineStr"/>
+      <c r="AI111" s="2" t="inlineStr"/>
+      <c r="AJ111" s="2" t="inlineStr"/>
+      <c r="AK111" s="2" t="inlineStr"/>
+      <c r="AL111" s="2" t="inlineStr"/>
+      <c r="AM111" s="2" t="inlineStr"/>
+      <c r="AN111" s="2" t="inlineStr"/>
+      <c r="AO111" s="2" t="inlineStr"/>
+      <c r="AP111" s="2" t="inlineStr"/>
+      <c r="AQ111" s="2" t="inlineStr"/>
+      <c r="AR111" s="2" t="inlineStr">
+        <is>
+          <t>Yes (caregiver play / availability of playthings at home)</t>
+        </is>
+      </c>
+      <c r="AS111" s="2" t="inlineStr"/>
+      <c r="AT111" s="2" t="inlineStr"/>
+      <c r="AU111" s="2" t="inlineStr"/>
+      <c r="AV111" s="2" t="inlineStr"/>
+      <c r="AW111" s="2" t="inlineStr"/>
+      <c r="AX111" s="2" t="inlineStr"/>
+      <c r="AY111" s="2" t="inlineStr"/>
+      <c r="AZ111" s="2" t="inlineStr"/>
+      <c r="BA111" s="2" t="inlineStr"/>
+      <c r="BB111" s="2" t="inlineStr"/>
+      <c r="BC111" s="2" t="inlineStr"/>
+      <c r="BD111" s="2" t="inlineStr"/>
+      <c r="BE111" s="2" t="inlineStr"/>
+      <c r="BF111" s="2" t="inlineStr"/>
+      <c r="BG111" s="2" t="inlineStr"/>
+      <c r="BH111" s="2" t="inlineStr"/>
+      <c r="BI111" s="2" t="inlineStr"/>
+      <c r="BJ111" s="2" t="inlineStr">
+        <is>
+          <t>UNICEF Innocenti global data story on children's play, drawing on internationally comparable data (MICS) collected 2010–2024 across 93 countries (~60% of the global under-5 population; comparable play data available only for ages 2–4). | Documents the developmental importance of play (meaningful play supports cognitive and social-emotional growth; missing it can hinder development of the brain's 'control centre'); age patterns (0–3 play alone or with caregivers; 3–5 more parallel and pretend play); six drivers of children's digital play; and UNICEF's effort to refine/expand MICS questions on play and availability of playthings at home. Regional population coverage was above 50% for Eastern Europe/Central Asia and sub-Saharan Africa and 46% for Latin America &amp; the Caribbean (caution urged where coverage &lt;50%).</t>
+        </is>
+      </c>
+      <c r="BK111" s="2" t="inlineStr"/>
+      <c r="BL111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="BM111" s="2" t="inlineStr"/>
+      <c r="BN111" s="2" t="inlineStr"/>
+      <c r="BO111" s="2" t="inlineStr"/>
+      <c r="BP111" s="2" t="inlineStr"/>
+      <c r="BQ111" s="2" t="inlineStr"/>
+      <c r="BR111" s="2" t="inlineStr"/>
+      <c r="BS111" s="2" t="inlineStr"/>
+      <c r="BT111" s="2" t="inlineStr"/>
+      <c r="BU111" s="2" t="inlineStr"/>
+      <c r="BV111" s="2" t="inlineStr"/>
+      <c r="BW111" s="2" t="inlineStr"/>
+      <c r="BX111" s="2" t="inlineStr"/>
+      <c r="BY111" s="2" t="inlineStr"/>
+      <c r="BZ111" s="2" t="inlineStr"/>
+      <c r="CA111" s="2" t="inlineStr"/>
+      <c r="CB111" s="2" t="inlineStr"/>
+      <c r="CC111" s="2" t="inlineStr"/>
+      <c r="CD111" s="2" t="inlineStr"/>
+      <c r="CE111" s="2" t="inlineStr"/>
+      <c r="CF111" s="2" t="inlineStr"/>
+      <c r="CG111" s="2" t="inlineStr"/>
+      <c r="CH111" s="2" t="inlineStr"/>
+      <c r="CI111" s="2" t="inlineStr"/>
+      <c r="CJ111" s="2" t="inlineStr"/>
+      <c r="CK111" s="2" t="inlineStr"/>
+      <c r="CL111" s="2" t="inlineStr"/>
+      <c r="CM111" s="2" t="inlineStr"/>
+      <c r="CN111" s="2" t="inlineStr"/>
+      <c r="CO111" s="2" t="inlineStr"/>
+      <c r="CP111" s="2" t="inlineStr"/>
+      <c r="CQ111" s="2" t="inlineStr"/>
+      <c r="CR111" s="2" t="inlineStr">
+        <is>
+          <t>Yes (global data charts)</t>
+        </is>
+      </c>
+      <c r="CS111" s="2" t="inlineStr"/>
+      <c r="CT111" s="3" t="inlineStr">
+        <is>
+          <t>Grey literature — UNICEF Office of Strategy and Evidence – Innocenti global data story (Florence, June 2026). ⚠ ATTRIBUTION TO VERIFY: the name 'Salah' does not appear in the report; it is an institutional UNICEF publication whose preparation was led by Claudia Cappa and Nicole Petrowski. Suggested citation: 'United Nations Children's Fund, The Power of Play: A global data story, UNICEF, Florence, June 2026.' Filed under Salah per upload; ECPC member's first name and connection need confirming.</t>
+        </is>
+      </c>
+      <c r="CU111" s="2" t="inlineStr"/>
+      <c r="CV111" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="CW111" s="2" t="inlineStr">
+        <is>
+          <t>Salah</t>
+        </is>
+      </c>
+      <c r="CX111" s="2" t="inlineStr">
+        <is>
+          <t>UNICEF Office of Strategy and Evidence – Innocenti</t>
+        </is>
+      </c>
+      <c r="CY111" s="2" t="inlineStr">
+        <is>
+          <t>United Nations Children's Fund (UNICEF Innocenti; preparation led by Claudia Cappa &amp; Nicole Petrowski)</t>
+        </is>
+      </c>
+      <c r="CZ111" s="2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="DA111" s="2" t="inlineStr">
+        <is>
+          <t>UNICEF Innocenti (global data story / report)</t>
+        </is>
+      </c>
+      <c r="DB111" s="3" t="inlineStr"/>
+      <c r="DC111" s="2" t="inlineStr"/>
+      <c r="DD111" s="2" t="inlineStr"/>
+      <c r="DE111" s="2" t="inlineStr"/>
+      <c r="DF111" s="2" t="inlineStr">
+        <is>
+          <t>A UNICEF Office of Strategy and Evidence – Innocenti global data story on children's play, using internationally comparable data (2010–2024; 93 countries, ~60% of the global under-5 population; comparable play data for ages 2–4). It documents the developmental importance of play, age-based play patterns, drivers of digital play, and gaps in globally comparable data, and describes UNICEF's work to expand MICS measurement of play and playthings.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Apply corrections: book year 2023, Rima Salah attribution, Seri figures
- Book "Foundations for a Peaceful World" chapters (Feder, Fitzpatrick,
  Vasic) corrected to 2023 (title + Year column).
- UNICEF "Power of Play" re-attributed: member = Salah, Rima (Chair, ECPC);
  Notes state it was submitted by Rima Salah and is an institutional UNICEF
  publication (led by Cappa & Petrowski) — removed the ⚠ verify flag.
- Seri / Telefono Azzurro dossier enriched with concrete figures: main
  areas of need (mental health 35.3%, relational difficulties 28.5%,
  abuse/violence 18.2%, digital 6.1%); within relational, parents 61.0%,
  peers 21.8%. Added abuse/violence outcome marker.
- Removed stray duplicate pdfs/Aber/Salah/ (user-authorized).
- Accuracy audit: 103 papers, all 110 cols, KF 103/103, no duplicate
  titles, no year mismatches. Old dated CSVs kept. Excel regenerated
  (162 flags).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -26243,7 +26243,11 @@
       <c r="AH107" s="2" t="inlineStr"/>
       <c r="AI107" s="2" t="inlineStr"/>
       <c r="AJ107" s="2" t="inlineStr"/>
-      <c r="AK107" s="2" t="inlineStr"/>
+      <c r="AK107" s="2" t="inlineStr">
+        <is>
+          <t>Yes (abuse and violence — 18.2% of cases)</t>
+        </is>
+      </c>
       <c r="AL107" s="2" t="inlineStr"/>
       <c r="AM107" s="2" t="inlineStr"/>
       <c r="AN107" s="2" t="inlineStr"/>
@@ -26270,7 +26274,7 @@
       <c r="BI107" s="2" t="inlineStr"/>
       <c r="BJ107" s="2" t="inlineStr">
         <is>
-          <t>Descriptive analysis of cases recorded by Telefono Azzurro's free 24/7 phone-and-chat Listening Service 1.96.96 during 01/01/2025–01/01/2026 in Italy. A clear preference for chat over the telephone emerged from Line 1.96.96, interpreted as more than a generational trait. | Situates listening needs against WHO estimates (about 1 in 7 adolescents aged 10–19 lives with a mental disorder; suicide is the third leading cause of death among people aged 15–29) and maps the main areas of need, how needs overlap, and multidimensional situations that surface through the helpline. (Specific case counts and top need-category percentages to be verified from the dossier's tables/figures.)</t>
+          <t>Descriptive analysis of cases recorded by Telefono Azzurro's free 24/7 phone-and-chat Listening Service 1.96.96 during 01/01/2025–01/01/2026 in Italy; a clear preference for chat over the telephone emerged. | Main areas of need (share of cases): mental health 35.3% (most frequent), relational difficulties 28.5%, abuse and violence 18.2%, digital 6.1%, and other areas 11.9%. Within relational difficulties, difficulties with parents accounted for 61.0% of cases, with peers 21.8%, a partner 9.3%, siblings 2.6% and teachers/educators 2.6%; eating disorders represented 6.6%. Situates these needs against WHO estimates (about 1 in 7 adolescents aged 10–19 lives with a mental disorder; suicide is the third leading cause of death among those aged 15–29).</t>
         </is>
       </c>
       <c r="BK107" s="2" t="inlineStr"/>
@@ -26365,7 +26369,7 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Feder, Joshua — 2025 — The Early Years Media Initiative for Children – Revised Toddler Module: Building Social-Emotional Resilience (in 'Foundations for a Peaceful World', Ch. 5)</t>
+          <t>Feder, Joshua — 2023 — The Early Years Media Initiative for Children – Revised Toddler Module: Building Social-Emotional Resilience (in 'Foundations for a Peaceful World', Ch. 5)</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr"/>
@@ -26558,7 +26562,7 @@
       </c>
       <c r="CT108" s="2" t="inlineStr">
         <is>
-          <t>Chapter 5 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation. Chapter authors: Joshua D. Feder, Z. Kernohan-Neely, Zach Davis.</t>
+          <t>Chapter 5 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Published 2023. Chapter authors: Joshua D. Feder, Z. Kernohan-Neely, Zach Davis.</t>
         </is>
       </c>
       <c r="CU108" s="2" t="inlineStr"/>
@@ -26584,7 +26588,7 @@
       </c>
       <c r="CZ108" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="DA108" s="2" t="inlineStr">
@@ -26605,7 +26609,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Fitzpatrick, Siobhan — 2025 — Developing a culture of respecting difference with young children, their families and communities in Northern Ireland (in 'Foundations for a Peaceful World', Ch. 1)</t>
+          <t>Fitzpatrick, Siobhan — 2023 — Developing a culture of respecting difference with young children, their families and communities in Northern Ireland (in 'Foundations for a Peaceful World', Ch. 1)</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr"/>
@@ -26778,7 +26782,7 @@
       </c>
       <c r="CT109" s="2" t="inlineStr">
         <is>
-          <t>Chapter 1 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation.</t>
+          <t>Chapter 1 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Published 2023.</t>
         </is>
       </c>
       <c r="CU109" s="2" t="inlineStr"/>
@@ -26804,7 +26808,7 @@
       </c>
       <c r="CZ109" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="DA109" s="2" t="inlineStr">
@@ -26825,7 +26829,7 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Vasic, Ljiljana — 2025 — Active Development of Respect for Diversity from Early Years in Serbia and the Western Balkans (in 'Foundations for a Peaceful World', Ch. 7)</t>
+          <t>Vasic, Ljiljana — 2023 — Active Development of Respect for Diversity from Early Years in Serbia and the Western Balkans (in 'Foundations for a Peaceful World', Ch. 7)</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr"/>
@@ -26998,7 +27002,7 @@
       </c>
       <c r="CT110" s="2" t="inlineStr">
         <is>
-          <t>Chapter 7 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Book publication year is not printed in the PDF (references run to 2024); listed as 2025 pending confirmation.</t>
+          <t>Chapter 7 in Foundations for a Peaceful World: The Transformative Power of Early Childhood Education to Promote Peace and Social Cohesion (eds. J.D. Feder, S. Fitzpatrick &amp; M. Ziv; Early Years / ACEV). Published 2023.</t>
         </is>
       </c>
       <c r="CU110" s="2" t="inlineStr"/>
@@ -27024,7 +27028,7 @@
       </c>
       <c r="CZ110" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="DA110" s="2" t="inlineStr">
@@ -27045,7 +27049,7 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Salah — 2026 — The Power of Play: A Global Data Story (UNICEF Office of Strategy and Evidence – Innocenti)</t>
+          <t>Salah, Rima — 2026 — The Power of Play: A Global Data Story (UNICEF Office of Strategy and Evidence – Innocenti)</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr"/>
@@ -27208,9 +27212,9 @@
         </is>
       </c>
       <c r="CS111" s="2" t="inlineStr"/>
-      <c r="CT111" s="3" t="inlineStr">
-        <is>
-          <t>Grey literature — UNICEF Office of Strategy and Evidence – Innocenti global data story (Florence, June 2026). ⚠ ATTRIBUTION TO VERIFY: the name 'Salah' does not appear in the report; it is an institutional UNICEF publication whose preparation was led by Claudia Cappa and Nicole Petrowski. Suggested citation: 'United Nations Children's Fund, The Power of Play: A global data story, UNICEF, Florence, June 2026.' Filed under Salah per upload; ECPC member's first name and connection need confirming.</t>
+      <c r="CT111" s="2" t="inlineStr">
+        <is>
+          <t>Grey literature — UNICEF Office of Strategy and Evidence – Innocenti global data story (Florence, June 2026); preparation was led by Claudia Cappa and Nicole Petrowski. Submitted to the ECPC repository by Rima Salah (Chair of the ECPC); she is not a named author of this institutional UNICEF publication. Suggested citation: 'United Nations Children's Fund, The Power of Play: A global data story, UNICEF, Florence, June 2026.'</t>
         </is>
       </c>
       <c r="CU111" s="2" t="inlineStr"/>
@@ -27221,12 +27225,12 @@
       </c>
       <c r="CW111" s="2" t="inlineStr">
         <is>
-          <t>Salah</t>
+          <t>Salah, Rima</t>
         </is>
       </c>
       <c r="CX111" s="2" t="inlineStr">
         <is>
-          <t>UNICEF Office of Strategy and Evidence – Innocenti</t>
+          <t>Yale Child Study Center; Chair, Early Childhood Peace Consortium</t>
         </is>
       </c>
       <c r="CY111" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add advocacy relevance ranking columns (ECPC ToC-aligned)
Appends 5 columns (110->115) ranking all 103 papers for the ECPC
"Peacebuilding through ECD" advocacy brief, per user's priorities:
1) Theme fit — alignment with the background paper's Theory of Change
   outcomes (child dev, caregiver practices/MH, social cohesion/intergroup,
   violence prevention, resilience, economic/governance) + crisis-context
   factors (conflict/displacement/refugee/toxic stress). Weight 50%.
2) Evidence rigour — RCT>quasi-exp>longitudinal>cross-sectional>qual;
   meta-analyses/reviews NOT penalised for lacking original data. Weight 30%.
3) Citations — "Cited by" among white literature; grey lit neutralised. 20%.
Columns: Advocacy relevance rank (1=highest), Relevance score, Theme fit,
Evidence rigour, Citations percentile. Excel + 07072026ECPCRR.csv regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF111"/>
+  <dimension ref="A1:DK111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -548,6 +548,11 @@
     <col width="12" customWidth="1" min="108" max="108"/>
     <col width="12" customWidth="1" min="109" max="109"/>
     <col width="70" customWidth="1" min="110" max="110"/>
+    <col width="16" customWidth="1" min="111" max="111"/>
+    <col width="14" customWidth="1" min="112" max="112"/>
+    <col width="16" customWidth="1" min="113" max="113"/>
+    <col width="14" customWidth="1" min="114" max="114"/>
+    <col width="16" customWidth="1" min="115" max="115"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -737,6 +742,15 @@
           <t>Abstract</t>
         </is>
       </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>ADVOCACY PRIORITIZATION (added: ranks papers for the ECPC "Peacebuilding through ECD" brief)</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr"/>
+      <c r="DI1" s="1" t="inlineStr"/>
+      <c r="DJ1" s="1" t="inlineStr"/>
+      <c r="DK1" s="1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -881,6 +895,11 @@
       <c r="DD2" s="1" t="inlineStr"/>
       <c r="DE2" s="1" t="inlineStr"/>
       <c r="DF2" s="1" t="inlineStr"/>
+      <c r="DG2" s="1" t="inlineStr"/>
+      <c r="DH2" s="1" t="inlineStr"/>
+      <c r="DI2" s="1" t="inlineStr"/>
+      <c r="DJ2" s="1" t="inlineStr"/>
+      <c r="DK2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -1025,6 +1044,11 @@
       <c r="DD3" s="1" t="inlineStr"/>
       <c r="DE3" s="1" t="inlineStr"/>
       <c r="DF3" s="1" t="inlineStr"/>
+      <c r="DG3" s="1" t="inlineStr"/>
+      <c r="DH3" s="1" t="inlineStr"/>
+      <c r="DI3" s="1" t="inlineStr"/>
+      <c r="DJ3" s="1" t="inlineStr"/>
+      <c r="DK3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -1145,6 +1169,11 @@
       <c r="DD4" s="1" t="inlineStr"/>
       <c r="DE4" s="1" t="inlineStr"/>
       <c r="DF4" s="1" t="inlineStr"/>
+      <c r="DG4" s="1" t="inlineStr"/>
+      <c r="DH4" s="1" t="inlineStr"/>
+      <c r="DI4" s="1" t="inlineStr"/>
+      <c r="DJ4" s="1" t="inlineStr"/>
+      <c r="DK4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr"/>
@@ -1369,6 +1398,31 @@
       <c r="DD5" s="1" t="inlineStr"/>
       <c r="DE5" s="1" t="inlineStr"/>
       <c r="DF5" s="1" t="inlineStr"/>
+      <c r="DG5" s="1" t="inlineStr">
+        <is>
+          <t>Advocacy relevance rank (1=highest)</t>
+        </is>
+      </c>
+      <c r="DH5" s="1" t="inlineStr">
+        <is>
+          <t>Relevance score (0-100)</t>
+        </is>
+      </c>
+      <c r="DI5" s="1" t="inlineStr">
+        <is>
+          <t>Theme fit: ToC outcomes + crisis context (0-100)</t>
+        </is>
+      </c>
+      <c r="DJ5" s="1" t="inlineStr">
+        <is>
+          <t>Evidence rigour (0-100)</t>
+        </is>
+      </c>
+      <c r="DK5" s="1" t="inlineStr">
+        <is>
+          <t>Citations percentile (white lit, 0-100)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr"/>
@@ -1661,6 +1715,11 @@
       <c r="DD6" s="1" t="inlineStr"/>
       <c r="DE6" s="1" t="inlineStr"/>
       <c r="DF6" s="1" t="inlineStr"/>
+      <c r="DG6" s="1" t="inlineStr"/>
+      <c r="DH6" s="1" t="inlineStr"/>
+      <c r="DI6" s="1" t="inlineStr"/>
+      <c r="DJ6" s="1" t="inlineStr"/>
+      <c r="DK6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr"/>
@@ -1845,6 +1904,11 @@
       <c r="DD7" s="1" t="inlineStr"/>
       <c r="DE7" s="1" t="inlineStr"/>
       <c r="DF7" s="1" t="inlineStr"/>
+      <c r="DG7" s="1" t="inlineStr"/>
+      <c r="DH7" s="1" t="inlineStr"/>
+      <c r="DI7" s="1" t="inlineStr"/>
+      <c r="DJ7" s="1" t="inlineStr"/>
+      <c r="DK7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr"/>
@@ -1977,6 +2041,11 @@
       <c r="DD8" s="1" t="inlineStr"/>
       <c r="DE8" s="1" t="inlineStr"/>
       <c r="DF8" s="1" t="inlineStr"/>
+      <c r="DG8" s="1" t="inlineStr"/>
+      <c r="DH8" s="1" t="inlineStr"/>
+      <c r="DI8" s="1" t="inlineStr"/>
+      <c r="DJ8" s="1" t="inlineStr"/>
+      <c r="DK8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2251,6 +2320,31 @@
       <c r="DF9" s="2" t="inlineStr">
         <is>
           <t>This study explores patterns of self-regulation and emotional well-being among Syrian refugee children in Lebanon, employing a person-centered approach, responding to theoretical challenges articulated by Dante Cicchetti and other psychologists. Using latent profile analysis with data from 2,132 children, we identified seven distinct profiles across cognitive regulation, emotional-behavioral regulation, interpersonal regulation, and emotional well-being. These profiles showed significant heterogeneity in patterns of self-regulation across domains and emotional well-being among Syrian children. Some profiles consistently exhibited either positive ("Well-regulated and Adjusted") or negative ("Moody and Frustrated") functioning across all domains, while others revealed domain-specific challenges, e.g., particularly sensitive to interpersonal conflict. This heterogeneity in the organization of self-regulatory skill and emotional well-being challenges the traditional homogeneous view of child development in conflict settings. The study also underscores the profiles' differential associations with demographic characteristics and experiences, with school-related experiences being particularly salient. We discuss the implications of these findings for future research in developmental psychopathology on self-regulation and emotional well-being in conflict-affected contexts. In addition, we advocate for tailored interventions to meet the diverse needs of children affected by conflict.</t>
+        </is>
+      </c>
+      <c r="DG9" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="DH9" s="2" t="inlineStr">
+        <is>
+          <t>55.2</t>
+        </is>
+      </c>
+      <c r="DI9" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="DJ9" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK9" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -2525,6 +2619,31 @@
           <t>Abstract This chapter critically reviews opportunities and challenges in designing and conducting actionable research on improving preprimary school quality and children’s learning and development, with a case study in Ghana. We describe the development of a research–practice partnership among university-based researchers, a local research organization, and Ghana’s Ministry of Education. The partnership developed and evaluated an in-service teacher training and a parental awareness program. Both programs pursued the same goals of increasing child-centered and play-based learning and improving children’s school readiness. We discuss the successes and challenges of scaling-up a successful teacher in-service training program. In addition, we describe unexpected findings of the parental awareness program that pose several new research questions. Implications for future research on measuring and improving preprimary educational quality through similar research–practice partnerships are discussed.</t>
         </is>
       </c>
+      <c r="DG10" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="DH10" s="2" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="DI10" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="DJ10" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="DK10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2819,6 +2938,31 @@
       <c r="DF11" s="2" t="inlineStr">
         <is>
           <t>This study investigates bidirectional relationships between Syrian refugee children’s social and emotional learning (SEL) skills and academic performance in an education support program in Lebanon. Using data from a cluster randomized control trial with 2,757 students who completed performance-based academic assessments and reports of their SEL skills from 131 teachers, we examine bidirectional associations between academic and five teacher-observable SEL skills/behaviors: Working Memory Functioning, Inhibitory Control Functioning, Prosocial Behavior, Hyperactivity &amp;amp; Externalizing Behavior, and Emotional Distress &amp;amp; Internalizing Behavior. Controlling for child-, teacher-, household risk-, and site-level covariates, multilevel modeling revealed that Working Memory Functioning uniquely stood apart from other SEL domains: start-of-year teacher-reported Working Memory Functioning predicted end-of-year academic performance, and start-of-year academic performance predicted end-of-year teacher-reported Working Memory Functioning. No other SEL skills demonstrated such bidirectional associations. Start-of-year academic performance also negatively predicted end-of-year teacher-reported Emotional Distress. Findings highlight the distinct and central role of Working Memory Functioning in academic learning, suggesting that easier-to-collect academic performance data may serve as an indicator of SEL skills that may be difficult to assess sans strong teacher–student relationships. Further, they highlight the utility of teacher-reported SEL assessments in resource-constrained contexts, calling attention to bidirectional developmental pathways when supporting children’s holistic well-being.</t>
+        </is>
+      </c>
+      <c r="DG11" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DH11" s="2" t="inlineStr">
+        <is>
+          <t>54.0</t>
+        </is>
+      </c>
+      <c r="DI11" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ11" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -3069,6 +3213,31 @@
           <t>Two case studies of parenting programs, aiming to improve parenting practices and child development outcomes, and implemented by Save the Children/Ministry of Health/Khesar Gyalpo University in Bhutan and Boston College/University of Rwanda/FXB in Rwanda, respectively called Prescription to Play and Sugira Muryango, were conducted by an independent research and learning group. Implementation research focused on the workforce, a crucial but little-studied element determining the success of programs going to scale. Mixed methods were used to examine their training, workload, challenges, and quality of delivery. Health assistants in Bhutan and volunteers in Rwanda were trained for 10-11 days using demonstrations, role plays, and manuals outlining activities to deliver to groups of parents (Bhutan) or during home visits (Rwanda). Workers' own assessments of their delivery quality, their confidence, and their motivations revealed that duty, confidence, and community respect were strong motivators. According to independent observations, the quality of their delivery was generally good, with an overall mean rating on 10 items of 2.36 (Bhutan) and 2.44 (Rwanda) out of 3. The facilitators of scaling for Bhutan included institutionalizing training and a knowledgeable workforce; the barrier was an overworked workforce. The facilitators of scaling for Rwanda included strong follow-up supervision; the barriers included high attrition among a volunteer workforce.</t>
         </is>
       </c>
+      <c r="DG12" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="DH12" s="2" t="inlineStr">
+        <is>
+          <t>47.0</t>
+        </is>
+      </c>
+      <c r="DI12" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ12" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="DK12" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -3327,6 +3496,31 @@
       <c r="DF13" s="2" t="inlineStr">
         <is>
           <t>Early childhood development (ECD) programmes are heralded as a way to improve children's health and educational outcomes. However, few studies in developing countries calculate the effectiveness of quality early childhood interventions. This study estimates the cost and cost-effectiveness of the Sugira Muryango (SM) trial, a home-visiting intervention to improve ECD outcomes through positive parent-child relationships. Cost-effectiveness analysis of ECD interventions is challenging given their potential to have multiple benefits. We propose a cost-effectiveness method using a single outcome, in this case the improvement in cognitive development per home-visit session, as an indication of efficiency comparable across similar interventions. The trial intervention cost US$456 per family. This cost will likely fall below US$200 if the intervention is scaled through government systems. The cost-effectiveness analysis suggests that while SM generated a relatively small impact on markers of early development, it did so efficiently. The observed improvements in cognitive development per home-visit are similar to other home-visiting interventions of longer duration. SM by focusing on the family had benefits beyond ECD, including reductions in violence against children and intermate partner violence, further analysis is needed to include these returns in the economic evaluation.</t>
+        </is>
+      </c>
+      <c r="DG13" s="2" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="DH13" s="2" t="inlineStr">
+        <is>
+          <t>54.1</t>
+        </is>
+      </c>
+      <c r="DI13" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ13" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK13" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -3605,6 +3799,31 @@
           <t>Evidence linking maternal subjective wellbeing (SWB) to early childhood development (ECD) is scarce. SWB measures an individual’s negative and positive affect, life satisfaction, and optimism. Using structural equation modeling and a nationally representative sample of Nigerian women 15–24 and their focal child 3–4 years old (N=3,176), this study examined associations of maternal/caregiver SWB with child literacy, cognitive, and socioemotional indices. Women reported average-to-high SWB. The SWB construct had a weak, inverse association with child outcomes; the weak direct path did not change when standardized or mediated by family investments such as early education, children’s books, or stimulating activities (total effects −0.04). Family investments showed a strong, robust association with child outcomes (total effects 0.79, p&lt;0.001). Findings suggest SWB is a weak proxy for mental health and underscore the need to invest in child development, child engagement, and family-strengthening programs.</t>
         </is>
       </c>
+      <c r="DG14" s="2" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
+      <c r="DH14" s="2" t="inlineStr">
+        <is>
+          <t>41.1</t>
+        </is>
+      </c>
+      <c r="DI14" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ14" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK14" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -3847,6 +4066,31 @@
       <c r="DF15" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: Given the protective effect of nurturing caregivers and families for child and adolescent mental health, there is a need to review and synthesize research evidence regarding the effectiveness of parenting and family interventions in low and middle-income countries, including humanitarian settings. To advance practice, further understanding of the active ingredients of such interventions and implementation factors that lead to effectiveness are essential. METHOD: This systematic review, an update from a previous review, included studies on any parenting or family intervention for children and adolescents aged 0-24, living in a low- or middle-income country, that quantitatively measured child or adolescent mental health outcomes. We searched Global Health, PubMed, PsychINFO, PILOTS and the Cochrane Library databases on the 9th July 2020, and updated on the 12th August 2022. Risk of bias was assessed using an adapted version of the NIH Quality Assessment Tool. We extracted data on: effectiveness outcomes, practice elements included in effective interventions, and implementation challenges and successes. MAIN FINDINGS: We found a total of 80 studies (n = 18,193 participants) representing 64 different family or parenting interventions, 43 of which had evidence of effect for a child or adolescent mental health outcome. Only 3 studies found no effect on child, adolescent or caregiver outcomes. The most common practice elements delivered in effective interventions included caregiver psychoeducation, communication skills, and differential reinforcement. Key implementation strategies and lessons learned included non-specialist delivery, the engagement of fathers, and integrated or multi-sector care to holistically address family needs. PRELIMINARY CONCLUSIONS: Despite a high level of heterogeneity, preliminary findings from the review are promising and support the use of parenting and family interventions to address the wider social ecology of children in low reso</t>
+        </is>
+      </c>
+      <c r="DG15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="DH15" s="2" t="inlineStr">
+        <is>
+          <t>77.2</t>
+        </is>
+      </c>
+      <c r="DI15" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DJ15" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="DK15" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -4069,6 +4313,31 @@
           <t>zeena khazendar, bassam marshoud, and eve puffer Palestinian children today are the fifth generation to have lived under Israeli occupation, characterized by violence, restricted movement, and displacement.Children in Gaza, referred to as the world's largest "openair prison" by Human Rights Watch, have been suffering from a decades-long land, air, and sea blockade.In the first</t>
         </is>
       </c>
+      <c r="DG16" s="2" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
+      <c r="DH16" s="2" t="inlineStr">
+        <is>
+          <t>40.6</t>
+        </is>
+      </c>
+      <c r="DI16" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="DJ16" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK16" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4351,6 +4620,31 @@
       <c r="DF17" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: The prevalence of household violence in low- and middle-income countries (LMICs) is high, and exposure to violence has significant adverse effects on both mental health and child development across generations. Evidence-based services to improve parenting practices and reduce household violence in LMICs are scarce, particularly across rural regions of West Africa. This study explored the feasibility, acceptability, and potential benefits of an evidence-based home-visiting intervention to promote early childhood development and reduce household violence-the Family Strengthening Intervention for Early Childhood Development and Violence-Prevention (FSI-ECD + VP)-among vulnerable families in rural regions of Sierra Leone. METHODS: Eighty dual-caregiver households in the Makeni region of Sierra Leone were included in the study (N = 160 caregivers; 73% female). Eligibility criteria included having at least one child aged 6-36 months and elevated scores (&gt; 62.5) on the Difficulties in Emotion Regulation Scale (DERS). Community Health Workers (CHWs) employed in the Makeni region completed a 3-week FSI-ECD + VP training. Families were randomized to receive either the FSI-ECD + VP or treatment as usual (TAU). Research assistants blinded to treatment assignment assessed caregiver mental health, caregiver-child interactions, and household violence at baseline, post-intervention, and 3-month follow-up time points. RESULTS: Triangulation of quantitative and qualitative data showed that caregivers, CHWs, and supervisors generally perceived the intervention as beneficial, feasible, and acceptable. Mixed effects models showed that caregivers who received the FSI-ECD + VP had significantly improved caregiver-child relationship outcomes compared to TAU as assessed by the Home Observation for Measurement of the Environment and the Observation of Caregiver-Child Interactions at post-intervention. Preliminary data also suggests that caregivers receiving the FSI-ECD + VP were</t>
+        </is>
+      </c>
+      <c r="DG17" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="DH17" s="2" t="inlineStr">
+        <is>
+          <t>71.7</t>
+        </is>
+      </c>
+      <c r="DI17" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="DJ17" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="DK17" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -4621,6 +4915,31 @@
           <t>INTRODUCTION: Early childhood is a critical period for development, yet families in low-resource settings often face barriers that compromise effective caregiving. Research evidence shows that parenting interventions can improve child growth and development. Given the unique challenges faced by single-headed households, this study examined whether caregiver household type modified the effects of Sugira Muryango, an evidence-based home-visiting program in Rwanda. Specifically, it assessed whether changes in child growth and development, dietary diversity, and healthcare-seeking behaviors over time differed between children from single versus dual caregiver households in the Sugira Muryango cluster randomized controlled trial (cRCT). METHODS: A total of 1,049 households were enrolled in the Sugira Muryango cRCT, with 508 households assigned to the control group and 541 to the intervention group. The analytic sample included 959 children from 959 households. Of these, 498 were from single caregiver households and 461 from dual caregiver households. Baseline and follow-up data collected 12 months post-intervention were analyzed. Linear mixed-effects models (LMMs) were used to analyze continuous outcomes, accounting for children nested within households and clusters. Models included fixed effects for timepoint, treatment group, caregiver household type (single vs. dual), and their three-way interaction (timepoint × treatment group × caregiver household type). Random intercepts for households and clusters were included to account for the hierarchical data structure. Mixed-effects logistic regression models were used for binary outcomes. RESULTS: There was no evidence of effect modification by caregiver household type on any outcome. For child growth indicators, three-way interaction terms were not significant for weight-for-age z-score (WAZ) (β = 0.081, 95% CI: -0.077 to 0.239), height-for-age z-score (HAZ) (β = 0.013, 95% CI: -0.180 to 0.207), or weight-for-height z-scor</t>
         </is>
       </c>
+      <c r="DG18" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="DH18" s="2" t="inlineStr">
+        <is>
+          <t>32.0</t>
+        </is>
+      </c>
+      <c r="DI18" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ18" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -4903,6 +5222,31 @@
       <c r="DF19" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: Sugira Muryango (SM) is a home-visiting intervention designed to promote early childhood development (ECD) and prevent violence in families with young children living in extreme poverty in rural Rwanda. METHODS: We present 4-year follow-up data collected in 2022 in n=1009 households (93%) from a cluster randomised trial. We compare outcomes in SM and usual care (UC) families using mixed-effect models. Results are reported as the average difference in change over time in the SM versus UC group for longitudinal outcomes and the average difference in SM versus UC groups for new outcomes. RESULTS: Compared with UC caregivers, caregivers who participated in SM report engaging in more stimulating interaction with their children (b=0.531; 95% CI: 0.468, 0.594) and are less likely to report use of harsh discipline (b=-0.189; 95% CI: -0.292, -0.087). The SM caregivers also provide more learning materials (b=0.218; 95% CI: 0.0219, 0.414), language stimulation (b=0.159; 95% CI: 0.080, 0.240), more varied interactions (b=147; 95% CI: 0.030, 0.260), fathers are reported to be more engaged in play (b=0.253; 95% CI: 0.039, 0.467) and SM households have better hygiene practices (b=0.189; 95% CI: 0.052, 0.326) compared with UC households. We do not observe treatment effects on children's cognitive outcomes, self-regulation or behavioural problems. There is a small negative association between SM and height-for-age (b=-0.038; 95% CI: -0.062, -0.012). CONCLUSIONS: SM resulted in changes in caregivers' behaviours to support children's health and development. Despite positive caregiver effects, we did not observe effects on child development or behavioural outcomes. Programme updates may be required to support children's continued cognitive growth. TRIAL REGISTRATION NUMBER: NCT02510313.</t>
+        </is>
+      </c>
+      <c r="DG19" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="DH19" s="2" t="inlineStr">
+        <is>
+          <t>51.5</t>
+        </is>
+      </c>
+      <c r="DI19" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="DJ19" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK19" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -5121,6 +5465,31 @@
         </is>
       </c>
       <c r="DF20" s="2" t="inlineStr"/>
+      <c r="DG20" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DH20" s="2" t="inlineStr">
+        <is>
+          <t>50.8</t>
+        </is>
+      </c>
+      <c r="DI20" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DJ20" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DK20" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -5409,6 +5778,31 @@
           <t>BACKGROUND: Intervention effectiveness studies rarely empirically assess Theories of Change (ToC) to determine how an intervention worked. We examine the ToC underlying the Sugira Muryango (SM) parenting program in rural Rwanda to understand whether the intervention improved child development outcomes via changes in caregivers' behaviors to improve the home caregiving environment, as hypothesized. METHODS: SM uses coaching of parents to create a safe, affectionate, stimulating, and violence-free home environment. A cluster randomized trial enrolled 1049 families with young children. SM had immediate effects on caregiver behaviors, improving scores on the Home Observation for Measurement of the Environment (HOME), harsh discipline, caregiver emotion regulation, and provision of dietary diversity. We use structural equation modeling to examine whether change in caregivers' behaviors explains intervention-related improvements in child development (Ages and Stages Questionnaire) one year after the intervention ended. RESULTS: Improvements in positive caregiving practices, including stimulation and early language learning as captured by the HOME, explained some of the intervention-related changes in child development, including gross motor, communication, problem-solving, and personal-social development. Increased dietary diversity explained intervention-related change in gross motor, problem-solving, and personal-social development. Change in harsh discipline and caregiver emotion regulation did not explain child outcomes. CONCLUSIONS: Intervention-related changes related to constructs captured on the HOME and dietary diversity were associated with changes in child development scores, but violent discipline and caregiver emotion regulation were not. Future research should examine whether these components of the intervention can be strengthened and may influence child development via other pathways, for example, via caregiver mental health.</t>
         </is>
       </c>
+      <c r="DG21" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="DH21" s="2" t="inlineStr">
+        <is>
+          <t>52.1</t>
+        </is>
+      </c>
+      <c r="DI21" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DJ21" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK21" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5677,6 +6071,31 @@
           <t>BACKGROUND: Resettled refugee families face elevated mental health risks, compounded by structural and cultural barriers. The Family Strengthening Intervention for Resettlement (FSIR), co-developed with resettled refugee communities, aims to improve family functioning and child mental health. This study evaluated FSI-R in Somali Bantu and Bhutanese communities in New England during COVID-19 using a Hybrid Type II Implementation-Effectiveness Trial guided by the EPIS framework. METHODS: Linear mixed modeling assessed changes in family functioning and child mental health. A process evaluation identified implementation barriers and informed adaptations. Activities were registered under Clinical Registry #NCT03796065. RESULTS: Bhutanese families receiving FSI-R showed greater improvements in parental supervision compared to usual care. Process evaluation highlighted that responsiveness to community needs supported successful implementation despite pandemic stressors. Somali Bantu interventionists reported stronger emotional connection with families during in-person delivery. CONCLUSIONS: Findings support the utility of hybrid trials in assessing both effectiveness and implementation of preventive interventions with resettling families. Despite contextual disruptions, attention to community needs and delivery flexibility enabled successful implementation. This study underscores the importance of context-informed strategies to sustain core elements of evidence-based interventions in dynamic settings.</t>
         </is>
       </c>
+      <c r="DG22" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="DH22" s="2" t="inlineStr">
+        <is>
+          <t>60.8</t>
+        </is>
+      </c>
+      <c r="DI22" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DJ22" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -5955,6 +6374,31 @@
       <c r="DF23" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: Children in impoverished families-especially those affected by violence-face risks to healthy development. In the years of strong economic recovery since the 1994 Genocide Against the Tutsi, the Rwandan Government has invested in early child development, social and child protection and violence prevention, but few strategies for scaling evidence-based interventions (EBIs) in these areas have been studied. METHODS: We present a Hybrid Type-2 Implementation-Effectiveness study of the PLAY Collaborative implementation strategy to engage government and other stakeholders in scaling Sugira Muryango (SM, "Strong Family") to families eligible for social protection in three rural districts. SM promotes nurturing care of children under three while reducing family violence. We assessed delivery quality (fidelity, competence) and perceptions of the PLAY Collaborative (e.g, feasibility, leadership, organisation, sustainability). An embedded trial of 538 households (778 caregivers, 555 children) tested SM effectiveness when delivered by child protection volunteers. RESULTS: Child protection volunteers delivered SM with high fidelity and competence that improved with time and routine supervision. The PLAY Collaborative was rated moderately to highly across implementation outcomes. The embedded trial revealed improvements in children's stimulation at home (d = 0.20, 95% CI: 0.04-0.36) as caregivers involved them more in daily activities (d = 0.37, 95% CI: 0.18-0.57) and provided more learning materials (d = 0.37, 95% CI: 0.16-0.59). SM families increased stimulating care (e.g. singing, playing; d = 0.26, 95% CI: 0.07-0.46); involved fathers more in caregiving (IRR = 1.18, 95% CI: 1.03-1.37); reduced harsh discipline (OR = 0.34, 95% CI: 0.14-0.82); and increased dietary diversity (d = 0.25, 95% CI: 0.04-0.45). SM caregivers reported improved mental health (d = -0.13, 95% CI: -0.26 to -0.01). SM households increased safe water storage (OR = 3.14, 95% CI: 1.64-6.03) and w</t>
+        </is>
+      </c>
+      <c r="DG23" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="DH23" s="2" t="inlineStr">
+        <is>
+          <t>83.4</t>
+        </is>
+      </c>
+      <c r="DI23" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="DJ23" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK23" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -6181,6 +6625,31 @@
           <t>&lt;b&gt;Zulfiqar A Bhutta and colleagues&lt;/b&gt; argue that the response to children in fragile and conflict affected settings must move beyond event based framings to tackle cumulative and intergenerational adversity and contextually relevant opportunities for action</t>
         </is>
       </c>
+      <c r="DG24" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DH24" s="2" t="inlineStr">
+        <is>
+          <t>41.1</t>
+        </is>
+      </c>
+      <c r="DI24" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ24" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DK24" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6435,6 +6904,31 @@
       <c r="DF25" s="2" t="inlineStr">
         <is>
           <t>ABSTRACT As digital technologies have become increasingly embedded in daily family life, there has been a growing international concern about children's protection, provision and participation rights in a digital environment. Recognising this, the Committee on the Rights of the Child published General Comment No. 25 Children's Rights in Relation to the Digital Environment (CRC, 2021), giving detailed advice on implementation issues in this area and calling for up‐to‐date research about children's digital lives. This paper makes a significant contribution to that much‐needed knowledge base by reporting the findings of an online survey conducted with parents and legal guardians ( n = 1444) (hereafter parents) of children aged 0–36 months across socially and ethnically diverse families in the four UK nations. The survey represented phase one of a larger three‐phase project, ‘Toddlers, Tech and Talk’, funded by the Economic and Social Research Council, which aimed to build an empirically robust body of knowledge about how 0‐3‐year‐olds' lives intersect with digital technologies at home in socially and ethnically diverse families in inner‐city, urban and rural communities. The survey found that nearly all family homes have Wi‐Fi connection, that many homes have a wide range of digital devices and that very young children engage in a wide range of digital activities both with their parents and on their own. Parents' mediation practices are shaped by parental digital practices and attitudes, with concomitant implications for children's digital rights. Implications are highlighted.</t>
+        </is>
+      </c>
+      <c r="DG25" s="2" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="DH25" s="2" t="inlineStr">
+        <is>
+          <t>39.7</t>
+        </is>
+      </c>
+      <c r="DI25" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="DJ25" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK25" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -6691,6 +7185,31 @@
       <c r="DF26" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: This paper reports on the development and validation of the 15-item Parental Attitudes to Digital Technology Scale (PADTS), a brief, psychometrically validated measure assessing parents' beliefs confidence, and concerns about their very young children's use of digital technologies. METHOD: Developed as part of the UK-wide Toddlers, Tech and Talk (TTT) study, PADTS addresses a gap in existing research by focusing on children from birth to 3 years, a stage often overlooked in digital parenting literature. Co-developed with parents and early years experts, the scale was tested with a nationally balanced UK sample (N = 934). RESULTS: Exploratory and confirmatory factor analyses supported a four-factor structure: perceived risks, perceived learning benefits, parental confidence and technology-related anxiety. The PADTS showed strong model fit and measurement invariance across parent gender, ethnicity and region, with some variation by child age. Correlational analyses indicated that benefits, perceptions and confidence were associated with supportive digital parenting, while anxiety was more weakly linked. CONCLUSION: PADTS shows potential as a practical tool for researchers, practitioners and policy-makers and may support a more nuanced understanding of how parental attitudes shape early digital experiences.</t>
+        </is>
+      </c>
+      <c r="DG26" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="DH26" s="2" t="inlineStr">
+        <is>
+          <t>37.8</t>
+        </is>
+      </c>
+      <c r="DI26" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ26" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="DK26" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -6893,6 +7412,31 @@
         </is>
       </c>
       <c r="DF27" s="2" t="inlineStr"/>
+      <c r="DG27" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="DH27" s="2" t="inlineStr">
+        <is>
+          <t>50.5</t>
+        </is>
+      </c>
+      <c r="DI27" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="DJ27" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DK27" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -7145,6 +7689,31 @@
           <t>This cross-sectional study examines whether provision of nurturing care in 31 countries over 10 years was associated with improvements in countries’ child development outcomes.</t>
         </is>
       </c>
+      <c r="DG28" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="DH28" s="2" t="inlineStr">
+        <is>
+          <t>48.0</t>
+        </is>
+      </c>
+      <c r="DI28" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ28" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK28" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7385,6 +7954,31 @@
         </is>
       </c>
       <c r="DF29" s="2" t="inlineStr"/>
+      <c r="DG29" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DH29" s="2" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="DI29" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DJ29" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK29" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7629,6 +8223,31 @@
         </is>
       </c>
       <c r="DF30" s="2" t="inlineStr"/>
+      <c r="DG30" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="DH30" s="2" t="inlineStr">
+        <is>
+          <t>52.2</t>
+        </is>
+      </c>
+      <c r="DI30" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="DJ30" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="DK30" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7857,6 +8476,31 @@
           <t>INTRODUCTION: Low- and middle-income countries (LMICs) often dedicate limited domestic funds to expand quality early childhood care and education (ECCE), making complementary international donor support potentially important. However, research on the allocation of international development assistance for ECCE has been limited. METHODS: We analysed data from the Creditor Reporting System on aid projects to assess global development assistance for ECCE in 134 LMICs from 2007 to 2021. By employing keyword-searching and funding-allocation methods, we derived two estimates of ECCE aid: a lower-bound estimate comprising projects primarily focusing on ECCE and an upper-bound estimate comprising projects with both primary and partial ECCE focus, as well as those that could benefit ECCE but did not include ECCE keywords. We also assessed aid directed to conflict-affected countries and to ECCE projects integrating COVID-19-related activities. RESULTS: Between 2007 and 2021, the lower-bound ECCE aid totaled US$3646 million, comprising 1.7% of the total US$213 279 million allocated to education. The World Bank led in ECCE aid, contributing US$1944 million (53.3% out of total ECCE aid). Low-income countries received less ECCE aid per child before 2016, then started to catch up but experienced a decrease from US$0.8 (2020) per child to US$0.6 (2021) per child. Funding for ECCE projects with COVID-19 activities decreased from a total of US$50 million in 2020 to US$37 million in 2021, representing 11.4% and 6.6% of annual total ECCE aid, respectively. Over 15 years, conflict-affected countries received an average of US$0.3 per child, a quarter of the aid received by non-conflict-affected countries (US$1.2 per child). CONCLUSION: Although ECCE aid increased significantly between 2007 and 2021, its proportion of total educational aid fell short of UNICEF's suggested 10% minimum. Recommendations include increasing the share of ECCE aid in total educational aid, increasing aid to low-i</t>
         </is>
       </c>
+      <c r="DG31" s="2" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="DH31" s="2" t="inlineStr">
+        <is>
+          <t>36.9</t>
+        </is>
+      </c>
+      <c r="DI31" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="DJ31" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK31" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -8097,6 +8741,31 @@
         </is>
       </c>
       <c r="DF32" s="2" t="inlineStr"/>
+      <c r="DG32" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DH32" s="2" t="inlineStr">
+        <is>
+          <t>43.2</t>
+        </is>
+      </c>
+      <c r="DI32" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="DJ32" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK32" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -8351,6 +9020,31 @@
       <c r="DF33" s="2" t="inlineStr">
         <is>
           <t>OBJECTIVE: Violence against children (VAC) is a global public health and human rights issue that can lead to long-lasting negative consequences for individual and societal outcomes. While extensive evidence indicates that parenting programmes might be effective in preventing VAC, there are several unsolved questions on how to ensure interventions are acceptable, feasible, effective and sustainable, particularly in low- and- middle-income countries (LMICs). METHOD: In this study, we report findings from a qualitative examination of policymakers' (N = 10), early childhood and parenting programme facilitators' (N = 20) and parents' and other caregivers' (N = 38) perspectives on VAC prevention to examine the implementation ecosystem of parenting programmes in Colombia, including contextual risk and protection factors, features of existing programmes, and stakeholders' needs. We conducted interviews and focus groups using a semistructured format, along with a thematic approach, to analyse the data from each group of participants (i.e., policymakers, facilitators and caregivers) independently. RESULTS: Overall, the data revealed the critical role of intersecting and interacting factors at the micro (e.g., caregivers' capabilities and beliefs), meso (e.g., programme content and delivery approaches) and macro (e.g., policymakers' vision and existing infrastructure) levels in exacerbating risks/imposing barriers versus protecting/promoting VAC prevention. CONCLUSIONS: These findings provide evidence on the implementation ecosystem of prevention programmes to inform the design of novel strategies and programmes aimed at preventing violence and promoting families' well-being and young children's development.</t>
+        </is>
+      </c>
+      <c r="DG33" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="DH33" s="2" t="inlineStr">
+        <is>
+          <t>44.1</t>
+        </is>
+      </c>
+      <c r="DI33" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ33" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK33" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -8581,6 +9275,31 @@
         </is>
       </c>
       <c r="DF34" s="2" t="inlineStr"/>
+      <c r="DG34" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="DH34" s="2" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="DI34" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ34" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DK34" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -8831,6 +9550,31 @@
       <c r="DF35" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: Increasing evidence suggests that climate change, along with its cascading impacts on ecosystems, societies, and communities, has significant effects on both physical and mental health. However, less is known about how exposure to excessive heat early in life may influence the development of foundational skills that shape lifelong developmental trajectories. This study examined the effects of ambient heat on early childhood development across six countries, using geographic and time-stamped data on child development and ambient temperature. METHODS: Our primary outcome is the Early Childhood Development Index. We used linear probability models with geographic and seasonality fixed effects to account for baseline climatic conditions, as well as other individual and contextual covariates to address potential selection bias. The sample comprised 19,607 children aged three and four from Georgia, The Gambia, Madagascar, Malawi, Sierra Leone, and the State of Palestine, all participants in Multiple Indicators Cluster Surveys collected between 2017 and 2020. We merged these data with temperature data from the ERA5-Land Monthly Aggregated Climate Dataset, calculating the mean monthly maximum temperature children experienced from birth to interview. RESULTS: We found that children exposed to average maximum temperatures above 32°C were less likely to be developmentally on track compared to those exposed to cooler temperatures, even after accounting for baseline average climatic conditions and other covariates. Domain-specific models indicate that these effects were most pronounced in literacy and numeracy skills. Subgroup analyses revealed that the negative impacts were particularly severe for children in economically disadvantaged households and urban areas, and for those lacking access to adequate water and sanitation. CONCLUSIONS: This study highlights the potential impact of excessive heat on early childhood development, emphasizing the need for policies and</t>
+        </is>
+      </c>
+      <c r="DG35" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="DH35" s="2" t="inlineStr">
+        <is>
+          <t>45.0</t>
+        </is>
+      </c>
+      <c r="DI35" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="DJ35" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK35" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -9061,6 +9805,31 @@
         </is>
       </c>
       <c r="DF36" s="2" t="inlineStr"/>
+      <c r="DG36" s="2" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="DH36" s="2" t="inlineStr">
+        <is>
+          <t>39.6</t>
+        </is>
+      </c>
+      <c r="DI36" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="DJ36" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK36" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -9295,6 +10064,31 @@
       <c r="DF37" s="2" t="inlineStr">
         <is>
           <t>We examine empirical and conceptual considerations related to the role of nurturing care for protecting human capital formation in the context of climate change. Climate change is a pressing global challenge. Heatwaves, wildfires, storms, and floods are becoming more frequent and severe, and their direct impact and aftermath can have long-lasting negative effects on employment, education, healthcare, and access to essential services. Children are particularly vulnerable to these harms due to their developmental immaturity and limited capacity to mitigate and avoid risks [1,2]. Consequently, parents and other adult primary caregivers - such as grandparents, relatives, and foster parents (hereafter "caregivers") - provide the primary buffer between climate hazards and adverse developmental outcomes. They do this through nurturing care, defined as the provision of stable environments that promote children's health and nutrition, safety and security, opportunities for learning, and emotionally supportive relationships [3]. Despite the central role of nurturing care for children's life outcomes, it rarely appears in climate change research and policy discourse.</t>
+        </is>
+      </c>
+      <c r="DG37" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="DH37" s="2" t="inlineStr">
+        <is>
+          <t>50.1</t>
+        </is>
+      </c>
+      <c r="DI37" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ37" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DK37" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -9537,6 +10331,31 @@
           <t>The seven articles in this Research Topic advance a shared commitment to understanding and improving inclusion through diverse methodologies, geographical contexts, and theoretical lenses. Together, they illustrate how educators, researchers, and policymakers can build systems that are not only equitable but also responsive to the lived realities of children, families, and communities.A central contribution of this Research Topic is the emphasis on co-construction and shared expertise. In Inclusive early childhood education: exploring co-creation and the process of empowerment within participatory research and practice, Carr-Fanning and Rihtman (2025) investigate how participatory research can empower educators and community partners to develop culturally grounded inclusion programs for children with ADHD-type behaviours in Hungary, Romania, and Slovakia. Through collaborative curriculum design and co-created professional learning, they demonstrate how inclusion emerges as both a process and an outcome of empowerment. Their findings underscore that meaningful inclusion is contextually defined and must evolve through reflective partnerships that challenge traditional hierarchies of expertise This participatory ethos resonates across the Research Topic, that is, inclusion cannot be achieved for communities but must be achieved with them. Empowerment, in this sense, becomes both the method and measure of inclusive success.Several contributions highlight the centrality of educator learning and reflective practice in sustaining inclusion. Dionne et al. (2025), in Supporting the inclusion of young children in childcare settings through professional development: perceptions of educators and managers, illustrate how sustained coaching and leadership engagement in Quebec childcare centers enhance educators' competence, confidence, and responsiveness to children's diverse needs. Their findings emphasize that professional learning must be iterative, relational, and embedded wi</t>
         </is>
       </c>
+      <c r="DG38" s="2" t="inlineStr">
+        <is>
+          <t>103</t>
+        </is>
+      </c>
+      <c r="DH38" s="2" t="inlineStr">
+        <is>
+          <t>25.7</t>
+        </is>
+      </c>
+      <c r="DI38" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="DJ38" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK38" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -9799,6 +10618,31 @@
       <c r="DF39" s="2" t="inlineStr">
         <is>
           <t>Crescendo is a music-based social and emotional learning (SEL) programme designed for primary/elementary school children living in disadvantaged communities. It is a community-led, orchestra-delivered, and evidence-informed initiative aimed at improving children’s musical and SEL outcomes through sustained engagement. Children growing up in socioeconomically disadvantaged areas often experience challenges with SEL and limited access to orchestral music education. However, emerging research suggests a relationship between music participation and SEL development. This study evaluated the initial impact of Crescendo on 559 children aged 5–6 in their first year of participation (Year 1 of 7). A quasi-experimental, rolling cohort design compared pupils in four participating Crescendo schools with pupils in four matched control schools not receiving the programme. Outcome measures included music skills (beat, pitch, and reaction to music) and SEL (behavioural self-regulation). The findings indicated significant positive effects of the programme across all outcome domains, with moderate effects observed in self-regulation (Cohen’s d = 0.29) and reaction to music (Cohen’s d = 0.21) compared to control schools. These results suggest that collaboration between orchestral musicians and educators can positively influence young children’s musical and SEL development in resource-constrained settings. The findings also underscore the importance of clearly defined programme models to support replication and scalability.</t>
+        </is>
+      </c>
+      <c r="DG39" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DH39" s="2" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="DI39" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="DJ39" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK39" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -10037,6 +10881,31 @@
           <t>From broadcast television to community outreach initiatives, Sesame Workshop uses formative research to assess the appeal, engagement, relevance, and comprehensibility of its media content. Through this process, young children and caregivers become vital partners in the content creation process. As Sesame Workshop expands its scope to support the needs of children around the world, formative research continues to be the grounding force in creating culturally relevant educational media content (Foulds &amp; Bucuvalas, 2019; Kohn et al., 2021; Foulds et al., 2021). Before the pandemic, in-person data collection was a core component of the formative research process. However, COVID-19-related safety protocols and movement restrictions posed significant barriers to traditional methods, inspiring Sesame Workshop teams to develop new approaches, leveraging both in-person and remote methods. This chapter documents adaptations to Sesame Workshop’s formative research model, using Watch, Play, Learn videos, a series of early learning videos to support families affected by crisis and displacement in Bangladesh, Brazil, Colombia, India, Jordan, Lebanon, Mexico, Nigeria, and South Africa. These examples provide early childhood media content creators and researchers with multiple approaches to conducting research with young children and share initial lessons on remote data collection, which may be especially relevant in emergency settings.</t>
         </is>
       </c>
+      <c r="DG40" s="2" t="inlineStr">
+        <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="DH40" s="2" t="inlineStr">
+        <is>
+          <t>32.7</t>
+        </is>
+      </c>
+      <c r="DI40" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DJ40" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK40" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -10273,6 +11142,31 @@
           <t>Evidence firmly establishes the link between early childhood interventions and the mitigation of the effects of adverse childhood experiences (ACEs). Given the long-term effects of conflict and displacement on children's healthy development, educational mass media can offer critical learning opportunities to mitigate both the impact of learning disruption and the effects of ACEs. This paper will highlight three different ways media, and its diverse distribution platforms, can support young children's understanding and use of coping strategies in the face of significant adversity. Using examples of diverse distribution to reach refugee and migrant children in the United States and across Latin America and the Middle East, this paper will highlight the ways media can support children and families affected by displacement and conflict to develop critical coping strategies. Lessons learned in developing and adapting coping strategies for diverse contexts and platforms include learnings for content curation and implementation, engagement of local and regional advisors, and importance of a network of on-the-ground implementing partners. These findings offer guidance for those developing content and programs for children in conflict and crisis, in particular creators of children's media and outreach programs.</t>
         </is>
       </c>
+      <c r="DG41" s="2" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
+      <c r="DH41" s="2" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="DI41" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ41" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK41" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -10523,6 +11417,31 @@
       <c r="DF42" s="2" t="inlineStr">
         <is>
           <t>Since 2015,o vert wo million people have sought refuge and asylum in Germany.¹Between January and August of 2022,the total number of first-time asylum-seeker applicants included close to 50,000 children under 18 years of age, which constitutes 42.9%o ft he total number of applications submitted to the German Federal Office for Migration and Refugees [Bundesamtf ür Migration und Flüchtlinge].²About half of thosec hildren (21.6%)w ereu nder the ageo ff our.As ar esulto f the large scale of this migration, newcomer pupils have faced challenges in accessing quality educational services.There are no reliable estimates of how manynewcomer children and youth are enrolled in German schools.The Expert Council on Integration and Migration [Sachverständigenrat für Integrationund Migration] estimates that about130,000 refugeec hildren and youth entered theG erman school system between January 2015 and March2 018.³These newcomer pupils will continue to enter the schools ystem in the future, which will significantlyi mpact on the schools ystem'sr esources and infrastructure.R esearch has documentedc hallenges and needs related to providingq uality education to newcomer pupils in Germany.Differing language backgroundsand related communication difficulties, and the fluctuation of newcomer pupils duet of requent changes of residenceo r deportation, are challenges in establishingsupportive relationships with newcom-Note: We areg rateful to the pupilsa nd educators who participated in this project.The development and implementation of the Huckepack summer programme in 2020 wassupportedbythe UBS Optimus Foundation.The implementation in 2022 wass upported by the Auf!Leben program,</t>
+        </is>
+      </c>
+      <c r="DG42" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="DH42" s="2" t="inlineStr">
+        <is>
+          <t>42.6</t>
+        </is>
+      </c>
+      <c r="DI42" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="DJ42" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK42" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -10773,6 +11692,31 @@
         </is>
       </c>
       <c r="DF43" s="2" t="inlineStr"/>
+      <c r="DG43" s="2" t="inlineStr">
+        <is>
+          <t>99</t>
+        </is>
+      </c>
+      <c r="DH43" s="2" t="inlineStr">
+        <is>
+          <t>32.7</t>
+        </is>
+      </c>
+      <c r="DI43" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DJ43" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="DK43" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11027,6 +11971,31 @@
       <c r="DF44" s="2" t="inlineStr">
         <is>
           <t>We examined the impact of the program “Families Make the Difference” (FMD) on well-being, feelings of distress, parental stress, parenting, co-parenting, paternal engagement, and several exploratory outcomes of Arab families in Berlin, Germany. FMD is a parent support program designed to assist families with refugee and migration backgrounds as they navigate life in Germany, where they often face challenges such as uncertain residency status, economic hardship, and the loss of their social and familial networks. In addition to the main effects on key outcomes, we also hypothesized that the changes in social support relate to the changes in parent characteristics (e.g., parental stress) and parenting behaviors. One hundred thirty-five caregivers participated in FMD and completed questionnaires before and after the program. We found small but statistically non-significant changes in most outcome measures over time. The only statistically significant finding indicated that female participants reported a decrease in parental stress over time, whereas male participants, on average, reported an increase. The results also suggest that increases in the perceptions of social support over time were associated with reductions in parental stress and feelings of distress and with increases in sensitive parenting, a composite measure of responsive caregiving, paternal engagement with the child and his spouse, and co-parenting. The findings imply that parenting programs with Arab families should be tailored to the needs of male and female caregivers. Future studies should examine the role of social support as a contributing factor to the benefits of parenting programs.</t>
+        </is>
+      </c>
+      <c r="DG44" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DH44" s="2" t="inlineStr">
+        <is>
+          <t>44.7</t>
+        </is>
+      </c>
+      <c r="DI44" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ44" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK44" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -11287,6 +12256,31 @@
       <c r="DF45" s="2" t="inlineStr">
         <is>
           <t>Although the importance of early childhood development (ECD) is well understood, related programming is scarce, especially in vulnerable Arab communities facing multiple emergencies. In 2012, the Arab Resource Collective (ARC) and its partners developed and pilot-tested a multi-sectoral responsive caregiving program in Lebanon, Egypt, and Jordan, all countries facing climate and refugee crises, and soon the pandemic. The program aimed to improve parents’ well-being, reduce stress levels, and support positive discipline strategies. When COVID-19 impacted Lebanon and Jordan in 2020, the intervention was provided both through an adapted face-to-face model and a new online delivery modality. These new modalities were piloted in one village in Mount Lebanon and two refugee camps in Lebanon and Jordan. Beneficiaries included disadvantaged families in Lebanon and Jordan as well as Syrian and Palestinian refugees. This chapter describes the adaption process and findings from testing three implementation modalities on parents’ knowledge, attitudes, and behaviors. Additionally, the chapter provides lessons learned that can inform similar programs targeting parents of young children in other crisis contexts.</t>
+        </is>
+      </c>
+      <c r="DG45" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="DH45" s="2" t="inlineStr">
+        <is>
+          <t>53.3</t>
+        </is>
+      </c>
+      <c r="DI45" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DJ45" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK45" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -11533,6 +12527,31 @@
           <t>OBJECTIVE: More than 200 million children and adolescents live in countries affected by violent conflict, are likely to have complex mental health needs, and struggle to access traditional mental health services. Digital mental health interventions have the potential to overcome some of the barriers in accessing mental health support. We performed a scoping review to map existing digital mental health interventions relevant for children and adolescents affected by war, to examine the strength of the evidence base, and to inform the development of future interventions. METHOD: Based on a pre-registered strategy, we systematically searched MEDLINE, Embase, Global Health, APA PsychInfo, and Google Scholar from the creation of each database to September 30, 2022, identifying k = 6,843 studies. Our systematic search was complemented by extensive consultation with experts from the GROW Network. RESULTS: The systematic search identified 6 relevant studies: 1 study evaluating digital mental health interventions for children and adolescents affected by war, and 5 studies for those affected by disasters. Experts identified 35 interventions of possible relevance. The interventions spanned from universal prevention to specialist-guided treatment. Most interventions directly targeted young people and parents or carers/caregivers and were self-guided. A quarter of the interventions were tested through randomized controlled trials. Because most interventions were not culturally or linguistically adapted to relevant contexts, their implementation potential was unclear. CONCLUSION: There is very limited evidence for the use of digital mental health interventions for children and adolescents affected by war at present. The review provides a framework to inform the development of new interventions. PLAIN LANGUAGE SUMMARY: Digital mental health interventions have the potential to overcome some of the barriers in accessing mental health support for children and adolescents living in war</t>
         </is>
       </c>
+      <c r="DG46" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="DH46" s="2" t="inlineStr">
+        <is>
+          <t>71.9</t>
+        </is>
+      </c>
+      <c r="DI46" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DJ46" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="DK46" s="2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -11771,6 +12790,31 @@
       <c r="DF47" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND AND OBJECTIVES Essential Newborn Care (ENC) training improves neonatal outcomes, particularly in low-resource settings. The American Academy of Pediatrics and Laerdal Global Health developed an online platform, https://hmbs.org/, to facilitate training of health care workers (HCWs) in ENC. This study aims to examine the impact of training with the ENC course. We hypothesize that training with the ENC course, either with remote or in-person facilitation, and low-dose high-frequency (LDHF) practice improves HCW knowledge and skills. METHODS In this prospective educational intervention study, technical advisors remotely oriented in-country facilitators to ENC in Nigeria and Bangladesh. In-country facilitators then trained frontline HCWs, choosing between a remote or in-person approach based on the country context. ENC knowledge check, bag-mask ventilation (BMV) skills, and NeoNatalie Live (NNL) manikin feedback pass rates were assessed at baseline (BL), immediately posttraining (PT), and endline (EL). Objective structured clinical examination (OSCE) A and B scores were assessed at PT and EL. LDHF practice was implemented at all sites using the NNL manikin. RESULTS After remote orientation, 18 in-country facilitators trained 236 frontline HCWs at 8 sites, including 1 humanitarian setting. All sites showed significant improvement in pass rates from BL to PT in knowledge check and BMV skills. NNL pass rates generally improved from PT to EL. OSCE A and B pass rates were also generally high PT and maintained at EL. CONCLUSIONS ENC online materials coupled with LDHF practice can augment knowledge and skills in ENC and offer a flexible option for remote or in-person training.</t>
+        </is>
+      </c>
+      <c r="DG47" s="2" t="inlineStr">
+        <is>
+          <t>87</t>
+        </is>
+      </c>
+      <c r="DH47" s="2" t="inlineStr">
+        <is>
+          <t>37.8</t>
+        </is>
+      </c>
+      <c r="DI47" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DJ47" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK47" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -12007,6 +13051,31 @@
       <c r="DF48" s="2" t="inlineStr">
         <is>
           <t>An increasingly polarized socio-political climate is diminishing the public's confidence in the SEL research evidence. In some cases, producing misinformation – or false evidence- as well as disinformation – or intentionally false evidence. Both have the potential to contribute to exclusionary policies and inequitable social and emotional experiences for students in the United States. This manuscript explores whether and how SEL stakeholders ( n = 25) understand, access, and use evidence to inform SEL-related decisions across professions, including K-12 educators, school administrators, and district personnel as well as policymakers, parents, and SEL researchers and advocates. Results from this pilot study suggest that SEL research evidence currently lacks accessibility for policymakers, educational leaders, and practitioners, and that the evidence that is available is limited in how it can be translated to and used in practice. How stakeholders identify and use SEL evidence is diverse, and most stakeholders access SEL evidence via news and education media. Opportunities for improving SEL evidence understanding, access, and use in the current U.S. socio-political climate are discussed. Findings suggest that SEL misinformation is likely more accessible to decision makers than the evidence that illustrates the success and benefits of SEL programming. Without continued proof and confirmation about what SEL is and how SEL is benefiting the nation’s youth, false narrative surrounding SEL that is being advocated for by specific groups and politicians is likely to prevail, resulting in continued skepticism about the use of SEL approaches in classrooms. This policy analyses and research study yield significant implications for SEL researchers and other stakeholders interested in creating, disseminating, and using SEL research in practice.</t>
+        </is>
+      </c>
+      <c r="DG48" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="DH48" s="2" t="inlineStr">
+        <is>
+          <t>42.0</t>
+        </is>
+      </c>
+      <c r="DI48" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="DJ48" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK48" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -12229,6 +13298,31 @@
           <t>This is the protocol for an evidence and gap map. The objective of this EGM is to identify and map all primary studies (including randomised and cluster randomised trials) and systematic reviews on universal, school-based social and emotional learning programmes for young children (3-11 years) to create a live, searchable, and publicly available evidence and gap map.</t>
         </is>
       </c>
+      <c r="DG49" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="DH49" s="2" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="DI49" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ49" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK49" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -12499,6 +13593,31 @@
       <c r="DF50" s="2" t="inlineStr">
         <is>
           <t>There is a substantial body of evidence which indicates that early childhood programmes have a positive effect on children's school readiness, academic achievement, and social and emotional development. Indeed, these benefits can last into adulthood. Based on this evidence base, many countries that strive to build their early childhood education offer to enhance later chances of prosperity. LINKS is an NIHR-funded study, carried out by a team from Queen's University Belfast and Ulster University, with support from UNICEF. The project aims to explore the impact of early childhood development programmes on social cohesion/peacebuilding in six conflict-affected low- and middle-income countries (LMICs); Timor-Leste, Viet Nam, Mali, Egypt, Kyrgyzstan and Tajikistan. This paper will focus on research carried out as part of the LINKS study in Timor-Leste which aimed to evaluate the impact of UNICEF community-based alternative pre-schools (CBAPs) in Timor-Leste. This research, carried out in 2020, employed a quasi-experimental pre- post-test design with a public pre-school control group. A total of 607 children were recruited to participate from 33 pre-schools: 508 completed post-tests after nine months of pre-school exposure to the CBAP programme. The East-Asia Pacific Early Childhood Development Scales (EAP-ECDS) were used to assess the development of children in the current study. Results of the post-test suggest that despite differences in time children spend in pre-school and infrastructure between the school types, attendance at CBAPs appears to close the developmental gap seen at the pre-test (baseline) between children in the two groups. The findings underline the importance of pre-school access and early learning experiences to the development of children at the highest risk of not reaching their developmental potential. The results point to the need to scale the intervention and to carry out an experimental effectiveness evaluation of this promising programme.</t>
+        </is>
+      </c>
+      <c r="DG50" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="DH50" s="2" t="inlineStr">
+        <is>
+          <t>57.3</t>
+        </is>
+      </c>
+      <c r="DI50" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ50" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK50" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -12753,6 +13872,31 @@
         </is>
       </c>
       <c r="DF51" s="2" t="inlineStr"/>
+      <c r="DG51" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="DH51" s="2" t="inlineStr">
+        <is>
+          <t>73.2</t>
+        </is>
+      </c>
+      <c r="DI51" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="DJ51" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK51" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -12977,6 +14121,31 @@
         </is>
       </c>
       <c r="DF52" s="2" t="inlineStr"/>
+      <c r="DG52" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DH52" s="2" t="inlineStr">
+        <is>
+          <t>55.5</t>
+        </is>
+      </c>
+      <c r="DI52" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ52" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DK52" s="2" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -13235,6 +14404,31 @@
       <c r="DF53" s="2" t="inlineStr">
         <is>
           <t>INTRODUCTION: Interpersonal violence against women is a major global health problem that may have intergenerational effects. This study investigated associations between maternal experiences of interpersonal violence and other traumatic events and maternal and infant salivary diurnal cortisol in a cohort of adolescent mothers in São Paulo, Brazil. METHOD: Adolescent mothers (14-19 years) participating in a home-visiting intervention were interviewed retrospectively about lifetime and pregnancy violence and trauma exposure. Mothers collected saliva at waking and before bedtime from themselves (n = 23) and their infants (n = 32) at 12 months postpartum. Multivariable regression models were used to examine associations between trauma history variables and salivary diurnal cortisol. RESULTS: Adjusting for the intervention group, infant sex, maternal age, non-supplement medication use, and sample collection time, we found that higher-than-average lifetime trauma exposure was associated with maternal evening cortisol (b = 0.472, p-value = 0.028). Lifetime assaultive violence exposure was also associated with maternal evening cortisol (b = 0.196, p-value = 0.02). Maternal exposure to traumatic events in pregnancy was positively associated with bedtime cortisol levels of infants (b = 0.21, p = 0.01). Trauma variables were not associated with maternal or infant morning cortisol levels. CONCLUSION: Results suggest that maternal trauma history influences both maternal and infant postnatal cortisol regulation as indexed by evening cortisol levels. These results are consistent with models of fetal programming; however, future studies should investigate potential postnatal psychobiological pathways. Lifetime trauma exposure may also become embedded in the maternal hypothalamic-adrenal-pituitary axis regulation. Future studies are needed to consider other biological pathways in the intergenerational transmission of trauma.</t>
+        </is>
+      </c>
+      <c r="DG53" s="2" t="inlineStr">
+        <is>
+          <t>91</t>
+        </is>
+      </c>
+      <c r="DH53" s="2" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="DI53" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="DJ53" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK53" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -13483,6 +14677,31 @@
       <c r="DF54" s="2" t="inlineStr">
         <is>
           <t>Maternal trauma influences infant and adult health outcomes and may impact future generations through epigenetic modifications such as DNA methylation (DNAm). Research in humans on the intergenerational epigenetic transmission of trauma effects is limited. In this study, we assessed DNAm signatures of war-related violence by comparing germline, prenatal, and direct exposures to violence across three generations of Syrian refugees. We compared families in which a pregnant grandmother versus a pregnant mother was exposed to violence and included a control group with no exposure to war. We collected buccal swab samples and survey data from mothers and 1-2 children in each of 48 families (n = 131 participants). Based on an epigenome-wide association study (EWAS), we identified differentially methylated regions (DMPs): 14 were associated with germline and 21 with direct exposure to violence. Most DMPs showed the same directionality in DNAm change across germline, prenatal, and direct exposures, suggesting a common epigenetic response to violence. Additionally, we identified epigenetic age acceleration in association with prenatal exposure to violence in children, highlighting the critical period of in utero development. This is the first report of an intergenerational epigenetic signature of violence, which has important implications for understanding the inheritance of trauma.</t>
+        </is>
+      </c>
+      <c r="DG54" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="DH54" s="2" t="inlineStr">
+        <is>
+          <t>56.7</t>
+        </is>
+      </c>
+      <c r="DI54" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ54" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK54" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
         </is>
       </c>
     </row>
@@ -13713,6 +14932,31 @@
         </is>
       </c>
       <c r="DF55" s="2" t="inlineStr"/>
+      <c r="DG55" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="DH55" s="2" t="inlineStr">
+        <is>
+          <t>54.4</t>
+        </is>
+      </c>
+      <c r="DI55" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DJ55" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DK55" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -13931,6 +15175,31 @@
       <c r="DF56" s="2" t="inlineStr">
         <is>
           <t>We examined the social and emotional challenges (SEC) of young children and the mental health of their caregivers in areas affected by armed conflict and displacement in Colombia. Anxiety, depression, and PTSD symptoms were assessed in 1,133 caregivers. Caregivers also reported on the SEC of their children aged 21-53 months. A subsample of 487 caregivers (43%) completed a resilience self-report measure. Caregivers reported substantial levels of psychopathology ranging from 12.84% of caregivers with elevated anxiety levels, 24.5% who scored above the cutoff on the PTSD measure, and 44.7% who screened positive for depression. Correlations (r) between child SEC and caregiver psychopathology ranged from 0.15 to 0.33. The association between caregiver depression and child SEC was more substantial for boys (B = 0.56) than girls (B = 0.22). We also found that girls whose caregivers reported elevated levels of psychopathology and low levels of caregiver resilience received the highest ratings of caregiver-reported SEC. The importance of caregiver-child resilience-focused psychosocial support is discussed.</t>
+        </is>
+      </c>
+      <c r="DG56" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="DH56" s="2" t="inlineStr">
+        <is>
+          <t>59.7</t>
+        </is>
+      </c>
+      <c r="DI56" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ56" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK56" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -14197,6 +15466,31 @@
         </is>
       </c>
       <c r="DF57" s="2" t="inlineStr"/>
+      <c r="DG57" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="DH57" s="2" t="inlineStr">
+        <is>
+          <t>44.1</t>
+        </is>
+      </c>
+      <c r="DI57" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="DJ57" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK57" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -14417,6 +15711,31 @@
         </is>
       </c>
       <c r="DF58" s="2" t="inlineStr"/>
+      <c r="DG58" s="2" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="DH58" s="2" t="inlineStr">
+        <is>
+          <t>30.9</t>
+        </is>
+      </c>
+      <c r="DI58" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="DJ58" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DK58" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -14629,6 +15948,31 @@
           <t>Gender differences in early childhood development are under-researched in low- and middle-income countries (LMICs) where almost 90% of the world’s young children live. This study examines the direction, magnitude, and variation of gender similarities and differences in 3- and 4-year-olds’ early childhood development in 71 low- and middle-income countries (LMICs). Moreover, we explore whether country-level gender inequality correlates with gender differences in early development. We analyzed Early Childhood Development Index (ECDI) data from UNICEF’s Multiple Indicators Cluster Surveys and the Demographic and Health Surveys between 2010 and 2019 ( n = 226,980). Using logistic regression, we estimated children’s odds of being developmentally on track in literacy-numeracy, approaches to learning, social-emotional, and physical domains. We also used meta-analytic regression to examine associations between early childhood development and country-level indicators of gender inequality. In approximately one-half of LMICs, odds of being developmentally on track did not significantly differ for girls and boys; in countries with significant differences, girls were more likely to be on track than boys (odds ratio [OR] = 1.21, 95% confidence interval [CI] = [1.18–1.24], p &amp;lt;.001). Differences favoring girls were largest in the social-emotional domain (OR = 1.27, 95% CI = [1.24–1.30], p &amp;lt;.001). Country-level gender development index explained a substantial amount of variation in gender differences across countries. Overall, findings suggest that when gender differences exist, girls are more likely than boys to be developmentally on track, particularly in the social-emotional domain and in countries with greater gender equality.</t>
         </is>
       </c>
+      <c r="DG59" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="DH59" s="2" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="DI59" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="DJ59" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DK59" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -14885,6 +16229,31 @@
         </is>
       </c>
       <c r="DF60" s="2" t="inlineStr"/>
+      <c r="DG60" s="2" t="inlineStr">
+        <is>
+          <t>102</t>
+        </is>
+      </c>
+      <c r="DH60" s="2" t="inlineStr">
+        <is>
+          <t>30.3</t>
+        </is>
+      </c>
+      <c r="DI60" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="DJ60" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK60" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -15151,6 +16520,31 @@
       <c r="DF61" s="2" t="inlineStr">
         <is>
           <t>Parental engagement in stimulating activities and the use of different discipline behaviors play a significant role in young children's behavioral development. Psychological frameworks often posit that parental beliefs and psychological well-being are key drivers of these parental behaviors. However, the influence of parental beliefs and psychological well-being on these parenting behaviors, and consequently on children's behavioral outcomes, remains understudied, particularly in low- and middle-income countries (LMICs). We collected primary data from 267 parents of young children (Mage in months = 13.66; 52.06% girls) living in low-income households in Bogotá and Soacha, Colombia, and assessed how parental beliefs and psychological distress predict children's behaviors through parental engagement in stimulation activities and use of violent punishment. Structural equation modeling indicated that positive parental beliefs about violence were linked to reduced engagement in stimulating activities, predicting lower child effortful control and positive affectivity, while parental psychological distress was associated with greater use of violent punishment, predicting lower effortful control and higher negative affectivity in children. These results underscore the importance of addressing parental beliefs and psychological well-being to support positive parenting behaviors and promote healthy behavioral development in young children, particularly in LMIC contexts.</t>
+        </is>
+      </c>
+      <c r="DG61" s="2" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="DH61" s="2" t="inlineStr">
+        <is>
+          <t>40.7</t>
+        </is>
+      </c>
+      <c r="DI61" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ61" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK61" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -15405,6 +16799,31 @@
           <t>Background: Parenting programs are a promising approach to prevent violence against children and promote positive parenting. We tested whether Apapacho, a violence-prevention parenting program developed in a research-practice partnership, was associated with improvements in caregivers’ outcomes. Participants and setting: short-term outcomes of Apapacho in Bogotá and Soacha, Colombia, integrated into the Modalidad Familiar service; caregivers of children under five (N=267: 134 Apapacho, 133 comparison; qualitative N=22). Methods: convergent parallel mixed-methods; difference-in-differences and thematic analysis; outcomes included responsive caregiving and stimulation, mental health/well-being, and non-violent vs violent discipline. Results: Apapacho was associated with short-term improvements in responsive-caregiving beliefs (β=0.17), reductions in approval of violent discipline (β=0.12), and increases in stimulation (β=0.19) and non-violent discipline (β=0.12); qualitative findings indicated improved caregiver-child relationships, understanding of children’s needs, emotional awareness/self-regulation, and non-violent discipline. Conclusions: Apapacho is a promising strategy for promoting positive parenting and preventing violence against children.</t>
         </is>
       </c>
+      <c r="DG62" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="DH62" s="2" t="inlineStr">
+        <is>
+          <t>51.9</t>
+        </is>
+      </c>
+      <c r="DI62" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DJ62" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK62" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -15665,6 +17084,31 @@
           <t>Increasingly, parents of young children need postsecondary credentials to compete in the labor market and meet basic family needs. This study uses a quasi-experimental design to examine the effects of CareerAdvance, a two-generation education intervention that offers postsecondary career training in healthcare for parents paired with Head Start for children. Overall, we find that CareerAdvance promotes low-income parents' educational advancement during the first three years after program entry, with weaker evidence of benefits to career progress and psychological wellbeing, and no evidence of economic gains. The two-generation program promotes greater educational and career advancement among parents without postsecondary credentials at baseline, than for parents who began the program with postsecondary credentials. In contrast, exploratory analyses suggest that parents entering the program with postsecondary credentials experienced benefits to some individual markers of economic and psychological wellbeing within three years.</t>
         </is>
       </c>
+      <c r="DG63" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DH63" s="2" t="inlineStr">
+        <is>
+          <t>44.7</t>
+        </is>
+      </c>
+      <c r="DI63" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ63" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK63" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -15925,6 +17369,31 @@
           <t>Importance: Children experiencing poverty are more likely to experience worse health outcomes, including injury, chronic illness, worse nutrition, and poorer sleep. The extent to which poverty reduction improves these outcomes is unknown. Objective: To evaluate the effect of a 3-year, monthly unconditional cash transfer on health, nutrition, sleep, and health care utilization among children experiencing poverty who were healthy at birth. Design, Setting, and Participants: This longitudinal randomized clinical trial recruited 1000 mother-infant dyads between May 2018 and June 2019. Dyads were recruited from postpartum wards in 12 hospitals in 4 US cities: New York, New York; Omaha, Nebraska; New Orleans, Louisiana; and Minneapolis/St Paul, Minnesota. Eligibility criteria included an annual income less than the federal poverty line, legal age for consent, English or Spanish speaking, residing in the state of recruitment, and an infant admitted to the well-baby nursery who will be discharged to the mother's custody. Data analysis was conducted from July 2022 to August 2023. Intervention: Mothers were randomly assigned to receive either a high-cash gift ($333/mo, or $3996/y) or a low-cash gift ($20/mo, or $240/y) for the first several years of their child's life. Main Outcomes and Measures: Primary preregistered outcomes reported here include an index of child health and medical care and child sleep disturbances. Secondary preregistered outcomes reported include children's consumption of healthy and unhealthy foods. Results: A total of 1000 mother-infant dyads were enrolled, with 400 randomized to the high-cash gift group and 600 to the low-cash gift group. Participants were majority Black (42%) and Hispanic (41%); 857 mothers participated in all 3 waves of data collection. We found no statistically detectable differences between the high-cash and low-cash gift groups in maternal assessments of children's health (effect size [ES] range, 0.01-0.08; SE range, 0.02-0.07),</t>
         </is>
       </c>
+      <c r="DG64" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="DH64" s="2" t="inlineStr">
+        <is>
+          <t>55.6</t>
+        </is>
+      </c>
+      <c r="DI64" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="DJ64" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK64" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -16183,6 +17652,31 @@
       <c r="DF65" s="2" t="inlineStr">
         <is>
           <t>We present the 2-year experimental mixed-methods findings of a two-generation English as a second language (ESL) program. This program combines a high-dosage, child-oriented curriculum for parents with Head Start for children in addition to family-based supportive services. At baseline and after 2 years, 189 Latinx and Zomi immigrant parents completed surveys while children completed skill assessments. A subset of 67 parents participated in focus groups regarding their experiences. Treatment parents reported significantly higher English writing skills and self-esteem and significantly lower language brokering and material hardship. There were no significant differences in children’s outcomes. Possible explanatory mechanisms across multiple contexts were identified in the qualitative data. Evidence is promising that a Two-Generation ESL Program improves some outcomes for parents.</t>
+        </is>
+      </c>
+      <c r="DG65" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="DH65" s="2" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="DI65" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ65" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="DK65" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -16417,6 +17911,31 @@
           <t>Abstract Interest in two-generation approaches to improve the developmental outcomes of children and their caregivers and the economic well-being of families has increased amid persistent child and family poverty worldwide. Grounded in a dual developmental science perspective and the theory of linked lives, these approaches maximize developmental potential by addressing the interrelated educational, economic, and developmental needs of children and their caregivers. They offer coordinated, aligned, and simultaneous services for at least two generations in the same family. In this article, we propose that from a global perspective, two-generation approaches that harness synergies among children and their caregivers are likely to be more effective than single-generation approaches in alleviating poverty and improving human development. We identify five models in different geographic regions of the world that promote the development of young children (0–6 years), the education and livelihood of their caregivers, and the well-being of both, which we group by type of program: quality child care, early childhood development + nonformal education for parents, and cash transfers + parenting. We close with a call for more research on two-generation programs and policies globally.</t>
         </is>
       </c>
+      <c r="DG66" s="2" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="DH66" s="2" t="inlineStr">
+        <is>
+          <t>54.3</t>
+        </is>
+      </c>
+      <c r="DI66" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="DJ66" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="DK66" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -16673,6 +18192,31 @@
           <t>Can cash transfers improve maternal well-being and family processes among families with young children? Using the Baby’s First Years randomized controlled trial (monthly unconditional cash transfers of $333 vs $20), this paper experimentally analyzes impacts of poverty reduction on maternal well-being and family processes among low-income U.S. mothers of young children.</t>
         </is>
       </c>
+      <c r="DG67" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="DH67" s="2" t="inlineStr">
+        <is>
+          <t>64.8</t>
+        </is>
+      </c>
+      <c r="DI67" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="DJ67" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK67" s="2" t="inlineStr">
+        <is>
+          <t>81</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -16935,6 +18479,31 @@
       <c r="DF68" s="2" t="inlineStr">
         <is>
           <t>Research on early language input and socioeconomic status typically relies on correlations in small convenience samples. Using data from Baby's First Years, this paper assesses the causal impact of monthly, unconditional cash transfers on child-directed speech and child vocalizations among a large, racially diverse sample of low-income U.S. mothers and their 1-year-olds (N = 563; 48% girls; 2019-2020). The monthly, unconditional cash transfers did not impact mothers' child-directed speech during a 10-min at-home play session (effect sizes range from -.08 to.02), though there was wide variability within this sample. Future work will assess the impact of the continued cash transfer on children's language input and development over time.</t>
+        </is>
+      </c>
+      <c r="DG68" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DH68" s="2" t="inlineStr">
+        <is>
+          <t>54.2</t>
+        </is>
+      </c>
+      <c r="DI68" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ68" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK68" s="2" t="inlineStr">
+        <is>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -17191,6 +18760,31 @@
       <c r="DF69" s="2" t="inlineStr">
         <is>
           <t>For refugee caregivers who may live in remote areas or be highly mobile, parenting programs that fit their needs can be beneficial. This RCT evaluated a 6-month, audio-only early childhood development intervention delivered via phone (3 calls/month) to caregivers of Syrian and Jordanian backgrounds in Jordan. Stipended community health volunteers (CHVs; N=99) and their caseloads of caregivers (n=2,298) were randomized to calls with health/nutrition content (control) or calls additionally including parenting and caregiver-focused content (adapted from Reach Up and Learn). Exposure to the treatment condition produced a statistically significant reduction in caregivers’ depressive symptoms (d=−0.11); no other statistically significant impacts were found on anxiety, parenting stress, harsh discipline, parent–child learning activities, parenting self-efficacy, or child development.</t>
+        </is>
+      </c>
+      <c r="DG69" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="DH69" s="2" t="inlineStr">
+        <is>
+          <t>78.0</t>
+        </is>
+      </c>
+      <c r="DI69" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="DJ69" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK69" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
         </is>
       </c>
     </row>
@@ -17465,6 +19059,31 @@
           <t>This study explores the effects of the two-generation program CareerAdvance-which combines education and training for parents in healthcare with Head Start for children-on children's academic, language, mathematics, and inhibitory control followed for 3 years. The sample (collected in Tulsa, Oklahoma from 2011 to 2018) includes 147 children in the CareerAdvance group and 139 children in a matched comparison group (n = 286; 40% Black, 17%, White, 10% Hispanic, 33% Mixed Race, or Other Race; M = 3.6 years old; 47% female). Overall, the effect of CareerAdvance on child outcomes is neither greater nor less than Head Start alone. These findings suggest that children's developmental outcomes do not worsen or improve in the short term when their parents return to school.</t>
         </is>
       </c>
+      <c r="DG70" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="DH70" s="2" t="inlineStr">
+        <is>
+          <t>41.1</t>
+        </is>
+      </c>
+      <c r="DI70" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="DJ70" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK70" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -17715,6 +19334,31 @@
       <c r="DF71" s="2" t="inlineStr">
         <is>
           <t>Financial scarcity has been posited to reduce adults’ cognitive bandwidth, but causal evidence is thin, especially in the U.S. and for parents of young children. We examine the impact of a monthly unconditional cash transfer on the cognitive bandwidth of U.S. mothers with low income (N=828). Preregistered intent-to-treat analyses find no differences in cognitive bandwidth of mothers after receiving a high-cash gift ($333/month) versus a low-cash gift ($20/month) for 48 months after childbirth.</t>
+        </is>
+      </c>
+      <c r="DG71" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="DH71" s="2" t="inlineStr">
+        <is>
+          <t>44.0</t>
+        </is>
+      </c>
+      <c r="DI71" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ71" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK71" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -17929,6 +19573,31 @@
           <t>Abstract The climate crisis encompasses a constellation of risks that threaten human livelihoods, well-being, and survival globally. In this article, we present a new framework based on bioecological and dynamic systems perspectives, and on evidence for conceptualizing how the distinctive dual time frame of both acute (e.g., extreme weather events) and chronic (e.g., ecological degradation) climate change-related risks experienced prenatally and early in life across multiple ecological contexts can threaten human development. We conclude with a call to developmental researchers, practitioners, and policymakers to invest more efforts in understanding and addressing the climate crisis and its developmental consequences to ensure a sustainable future for all.</t>
         </is>
       </c>
+      <c r="DG72" s="2" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="DH72" s="2" t="inlineStr">
+        <is>
+          <t>42.1</t>
+        </is>
+      </c>
+      <c r="DI72" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="DJ72" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DK72" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18191,6 +19860,31 @@
       <c r="DF73" s="2" t="inlineStr">
         <is>
           <t>Economic disadvantage has often been associated with poorer performance on measures of early childhood development. However, the causal impacts of income on child development remain unclear. The present study uses data from the Baby's First Years randomized control trial to identify the causal impact of unconditional cash transfers on maternal reports of early childhood development. One thousand racially and ethnically diverse mothers residing in poverty were recruited from four U.S. metropolitan areas shortly after giving birth. Mothers were randomized to receive either a $333/month or $20/month unconditional cash transfer for the first several years of their child's life. Maternal reports of language and socioemotional development, concerns for developmental delay, and enrollment in early intervention services were collected annually at the time of the child's first, second, and third birthdays. In this registered report, we document no statistically detectable impacts of the high-cash gift on maternal reports of child development. We discuss the significance and implications of these findings. (PsycInfo Database Record (c) 2024 APA, all rights reserved).</t>
+        </is>
+      </c>
+      <c r="DG73" s="2" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="DH73" s="2" t="inlineStr">
+        <is>
+          <t>55.8</t>
+        </is>
+      </c>
+      <c r="DI73" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DJ73" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK73" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
         </is>
       </c>
     </row>
@@ -18449,6 +20143,31 @@
           <t>Baby’s First Years (BFY) is a randomized control study identifying the causal impact of a poverty-reduction intervention (monthly unconditional cash, $333 vs $20) on early childhood development. One thousand mothers with incomes at or near the federal poverty line and their newborns were recruited from 12 hospitals in four diverse U.S. communities in 2018–2019. This brief reports three-year follow-up findings on food security, spending, and consumption, situating cash transfers alongside SNAP and WIC in reducing child poverty and hunger and supporting child development.</t>
         </is>
       </c>
+      <c r="DG74" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="DH74" s="2" t="inlineStr">
+        <is>
+          <t>48.1</t>
+        </is>
+      </c>
+      <c r="DI74" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DJ74" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK74" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -18705,6 +20424,31 @@
           <t>Poverty interferes with parents' breastfeeding, child-care, and employment options and ability to meet their parenting goals. This study-the first randomized controlled trial of early childhood poverty reduction in the United States-investigates how increased economic resources affect 1,000 low-income US mothers' breastfeeding, child-care, and employment practices and the ability to meet their intentions for these practices in the first year of their infant's life. The likelihood and length of breastfeeding, use of nonparental child care, and maternal employment did not statistically differ among mothers who received a high ($333) or low ($20) monthly unconditional cash gift. The higher monthly cash gift, however, delayed the starting age of child care by almost 1 month and increased mothers' ability to meet their breastfeeding intentions reported at birth.</t>
         </is>
       </c>
+      <c r="DG75" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="DH75" s="2" t="inlineStr">
+        <is>
+          <t>50.3</t>
+        </is>
+      </c>
+      <c r="DI75" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="DJ75" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK75" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -18977,6 +20721,31 @@
           <t>Importance: Mothers and children in low-income households are more likely to experience worse mental and physical health than those from higher-income households. Objective: To determine the effect of 4 years of monthly unconditional cash transfers on the mental health of mothers with low-income and the physical health of mothers and children. Design, Setting, and Participants: This was a parallel-group, randomized clinical trial conducted from May 2018 to July 2023. Mother-infant dyads were recruited (May 2018-June 2019) from postpartum wards in 12 hospitals in 4 cities: Omaha, Nebraska; Minneapolis/St Paul, Minnesota; New Orleans, Louisiana; and New York, New York. Data were analyzed from September 2023 to February 2025. Interventions: Mothers were randomly assigned to receive either a high-cash gift ($333 per month) or a low-cash gift ($20 per month) on debit cards. The cash gifts continued for the first 6 years of their children's lives. Data analyzed here were collected after 4 years of monthly transfers. Main Outcomes and Measures: Outcomes were preregistered and measured around the child's fourth birthday. Maternal outcomes included depression, anxiety, and body mass index (BMI). Child outcomes included age- and sex-adjusted BMI percentile and maternal report of child health (overall health, times sick in the past year, and presence of chronic health conditions). Results: A total of 1000 mother-infant dyads (mean [SD] maternal age, 27.0 [5.8] years) were included in this study. Among those mothers, 400 were randomly assigned to receive the $333 high-cash gift and 600 received the $20 low-cash gift on debit cards. Data were available from 891 mother-child dyads. No statistically detectable group differences were found in maternal depressive symptoms (effect size [ES], 0.04; 95% CI, -0.08 to 0.17; P =.51), anxiety (ES, 0.12; 95% CI, -0.02 to 0.25; P =.09), or BMI (ES, -0.06; 95% CI, -0.21 to 0.09; P =.42). In addition, there were no statistically detectable</t>
         </is>
       </c>
+      <c r="DG76" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="DH76" s="2" t="inlineStr">
+        <is>
+          <t>58.3</t>
+        </is>
+      </c>
+      <c r="DI76" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ76" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK76" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -19225,6 +20994,31 @@
           <t>PURPOSE: As of 2024, 123.2 million people had been forcibly displaced as a result of persecution, armed conflict or climate-related catastrophes, and these numbers are predicted to rise. There is a growing awareness of possible intergenerational effects of trauma on life-course health and well-being, however few studies have followed individuals longitudinally starting prenatally. This paper describes the first large prenatal birth cohort study in a refugee context in a lower middle-income country. This study aims to investigate the potential lifespan health and developmental implications of being born into a protracted humanitarian context, and what factors can buffer from the adversity posed by conflict and displacement. PARTICIPANTS: We outline our approach of recruiting, consenting and gathering data from pregnant Rohingya refugee and host community women (N=2888; 80% Rohingya) over the course of 12 months in Cox's Bazar, Bangladesh. FINDINGS TO DATE: A fifth wave of data collection, when children were 6 months old, was completed in April 2025. Rohingya women were substantially less literate; were marrying and having children at slightly younger ages, were more likely to live in crowded, resource-limited households and exhibited higher rates of clinically significant post-traumatic stress disorder and anxiety than host community women. FUTURE PLANS: There is a critical need for research in displaced populations in order to elucidate potentially lasting transgenerational impacts of experiencing conflict and displacement trauma, and the prenatal and postnatal factors that support health and development across the life span. The next follow-up is planned when the children turn 36 months of age (starting March 2026).</t>
         </is>
       </c>
+      <c r="DG77" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="DH77" s="2" t="inlineStr">
+        <is>
+          <t>59.7</t>
+        </is>
+      </c>
+      <c r="DI77" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ77" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK77" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -19475,6 +21269,31 @@
       <c r="DF78" s="2" t="inlineStr">
         <is>
           <t>Despite the long-standing debate over the assumed universality of maternal sensitivity predicting attachment security (i.e., sensitivity hypothesis), few long-term longitudinal investigations on attachment have been conducted outside the Western context. We leveraged data from a prospective 9-year longitudinal study of middle-class families (N = 356; female = 48.9%) in China to examine if early maternal sensitivity predicts attachment representations in middle childhood. Maternal sensitivity was assessed from lab-based observed interactions at 14 and 24 months. At 10 years old, children completed the Chinese version of the Attachment Script Assessment. Maternal sensitivity positively predicted the child's attachment representations at age 10 years (β = 0.20, p &lt; 0.01). These results supported the view that maternal sensitivity is prospectively related to secure attachment across cultures.</t>
+        </is>
+      </c>
+      <c r="DG78" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="DH78" s="2" t="inlineStr">
+        <is>
+          <t>41.1</t>
+        </is>
+      </c>
+      <c r="DI78" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="DJ78" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK78" s="2" t="inlineStr">
+        <is>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -19753,6 +21572,31 @@
           <t>Developmental differences between children growing up in poverty and their higher-income peers are frequently reported.However, the extent to which such differences are caused by differences in family income is unclear.To study the causal role of income on children's development, the Baby's First Years randomized control trial provided families with monthly unconditional cash transfers.One thousand racially and ethnically diverse mothers with incomes below the U.S. federal poverty line were recruited from postpartum wards in 2018-19, and randomized to receive either $333/month or$20/month for the first several years of their children's lives.After the first four years of the intervention (n=891), we find no statistically significant impacts of the cash transfers on four preregistered primary outcomes (language, executive function, social-emotional problems, and high-frequency brain activity) nor on three secondary outcomes (visual processing/spatial perception, pre-literacy, maternal reports of developmental diagnoses).Possible explanations for these results are discussed.</t>
         </is>
       </c>
+      <c r="DG79" s="2" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="DH79" s="2" t="inlineStr">
+        <is>
+          <t>50.8</t>
+        </is>
+      </c>
+      <c r="DI79" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DJ79" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK79" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -20001,6 +21845,31 @@
           <t>To contextualize findings on how the Baby’s First Years cash-gift intervention affected Latina families, this report summarizes economic outcomes and family investments in child-specific goods and time for the full sample and Latina families. Over three years and ~36 months of cash-gift receipt after childbirth, high-cash gift households spent more on child-specific goods and more time on child-specific early-learning activities than low-cash households, and reported lower rates of public-benefit receipt and fewer residing in poverty.</t>
         </is>
       </c>
+      <c r="DG80" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="DH80" s="2" t="inlineStr">
+        <is>
+          <t>44.4</t>
+        </is>
+      </c>
+      <c r="DI80" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="DJ80" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK80" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -20287,6 +22156,31 @@
       <c r="DF81" s="2" t="inlineStr">
         <is>
           <t>BACKGROUND: This study evaluates a 6-month early childhood father engagement intervention delivered in-person to fathers in the Rohingya camps and surrounding host communities in Cox's Bazar, Bangladesh. The intervention is an added component to an existing intervention that works with mothers of 0-3-year-old children to improve positive outcomes of child development and targets fathers with children below 3 years, with objectives to promote fathers' wellbeing by improving their emotional literacy, encouraging fathers to strengthen relationships with their spouses and children, and encouraging responsive and stimulating caregiving practices among fathers. METHODS: We used a cluster-randomized controlled trial design (total N = 2002 fathers, 786 in the Rohingya camps and 1216 in the host communities) to assess the impact of the program on fathers' parenting and engagement with family (reported by both fathers and mothers), fathers' mental health, and child development. RESULTS: We find that the program has a positive impact on the fathers' parenting (father reported) and engagement with family (father and mother reported), as well as on father-reported child social-emotional development, compared to the mother-only program. While the program did not have a main effect on directly assessed child development outcomes, we do find that baseline mother-reported stimulation with child and mother health moderate the impact on father-reported child social-emotional development in the camp community (larger positive impacts for fathers from households with lower baseline mother-reported stimulating behaviors and health). We also find that child gender and mother-reported stimulating behaviors moderate impacts on multiple mother-reported child developmental outcomes in both host and camp communities (treatment effects on these outcomes were negative for boys and positive but weak for girls, and larger positive impacts on mother-reported motor development were found among mothe</t>
+        </is>
+      </c>
+      <c r="DG81" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="DH81" s="2" t="inlineStr">
+        <is>
+          <t>67.1</t>
+        </is>
+      </c>
+      <c r="DI81" s="2" t="inlineStr">
+        <is>
+          <t>79</t>
+        </is>
+      </c>
+      <c r="DJ81" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK81" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -20529,6 +22423,31 @@
           <t>Research on father engagement is heavily focused on Western families and often individualistic, neglecting collective-care cultures and refugee contexts. This study asks how Rohingya fathers perceive children’s play in both structured (Humanitarian Play Labs) and unstructured (home and surrounding) settings in the Rohingya camps in Cox’s Bazar, Bangladesh. Using semi-structured interviews with 25 Rohingya fathers (aged 23–48), each with a child in BRAC’s 0–6 early-childhood range, the study explores playing with children, discipline/behavior management, and child participation in the Humanitarian Play Lab.</t>
         </is>
       </c>
+      <c r="DG82" s="2" t="inlineStr">
+        <is>
+          <t>86</t>
+        </is>
+      </c>
+      <c r="DH82" s="2" t="inlineStr">
+        <is>
+          <t>38.6</t>
+        </is>
+      </c>
+      <c r="DI82" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="DJ82" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK82" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -20793,6 +22712,31 @@
           <t>Early childhood poverty is associated with neurodevelopmental differences, but causal evidence linking income to brain development is sparse. In the present study, we examine whether four years of monthly unconditional cash transfers to mothers experiencing low income cause differences in their preschoolers’ brain activity. Shortly after giving birth, mothers were randomized to receive $333/month or $20/month. We find no impact on our primary preregistered outcome (an aggregated index of mid-to-high-frequency brain activity) or our secondary preregistered outcome frontal gamma power. In additional analyses that were part of our pre-registered analytic plan, we find that preschoolers in the high-cash gift group have higher alpha power than those in the low-cash gift group, but no differences in theta, beta, or gamma power. These findings suggest monthly unconditional cash transfers may have impacts on children’s alpha power during the preschool years, although this evidence needs further investigation and replication.</t>
         </is>
       </c>
+      <c r="DG83" s="2" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="DH83" s="2" t="inlineStr">
+        <is>
+          <t>42.3</t>
+        </is>
+      </c>
+      <c r="DI83" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="DJ83" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK83" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -21059,6 +23003,31 @@
       <c r="DF84" s="2" t="inlineStr">
         <is>
           <t>Universal, school-based social-emotional learning (SEL) interventions hold the promise to promote children's academic learning and social and emotional skills necessary to cope with adversity in education in conflict and crisis. This study evaluated the sequential implementation of two sets of skill-targeted SEL activities—first the impact of an 11-week Mindfulness implementation alone, then the combined effect of Mindfulness and Brain Games over 22 weeks—with Nigerian refugee and Nigerien local second-to-fourth graders (n=1,795) attending remedial education programming in Diffa, Niger, via a cluster randomized controlled trial. Positive impacts of Mindfulness activities were observed on a select number of SEL outcomes, with additional benefits for refugees and girls, demonstrating the potential for low-cost SEL approaches to support vulnerable children at scale in crisis-affected contexts.</t>
+        </is>
+      </c>
+      <c r="DG84" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="DH84" s="2" t="inlineStr">
+        <is>
+          <t>65.7</t>
+        </is>
+      </c>
+      <c r="DI84" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ84" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK84" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -21331,6 +23300,31 @@
       <c r="DF85" s="2" t="inlineStr">
         <is>
           <t>Despite widespread enthusiasm for remedial education programming with refugee populations, there is little rigorous evidence on how to design and implement such programs. We employ a cluster-randomized design of non-equivalent treatment groups to test the impact of two types of program enhancement—longer program duration and the addition of skill-targeted social and emotional learning (SEL) activities—for Syrian refugees enrolled in Lebanese public schools. Compared to 10 weeks of programming, 26 weeks marginally increases students' literacy skills (ES=0.04) and significantly improves behavioral regulation (ES=0.31), but students reported less positive perceptions of their public school environment (ES=-0.83 to -0.89) and remedial tutoring site (ES=-0.15 to -0.24). The addition of skill-targeted SEL activities to 26 weeks results in higher student reports of school-related stress compared to programming without skill-targeted activities (ES=0.21). Implications for program and policy are discussed.</t>
+        </is>
+      </c>
+      <c r="DG85" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="DH85" s="2" t="inlineStr">
+        <is>
+          <t>65.7</t>
+        </is>
+      </c>
+      <c r="DI85" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ85" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK85" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -21569,6 +23563,31 @@
           <t>Book chapter reviewing the state of social and emotional learning (SEL) research and practice in countries affected by armed conflicts and protracted crises (CAC), and arguing for an inclusive, representative, and generalizable SEL science that integrates CAC contexts into the broader field.</t>
         </is>
       </c>
+      <c r="DG86" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="DH86" s="2" t="inlineStr">
+        <is>
+          <t>58.8</t>
+        </is>
+      </c>
+      <c r="DI86" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="DJ86" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK86" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -21791,6 +23810,31 @@
       <c r="DF87" s="2" t="inlineStr">
         <is>
           <t>Most studies of corporal punishment and child development focus on the U.S. and other high-income countries. This rapid review examined associations between corporal punishment and children’s cognitive and social-emotional development in LMICs, reviewing &gt;42 studies of children &lt;18 in 64 LMICs. Reviewed studies show associations between corporal punishment and negative cognitive and social-emotional outcomes, with no evidence of positive developmental outcomes; validity issues are common. Evidence indicates corporal punishment might increase the risk of detrimental outcomes in LMICs; stronger methodological designs across multiple settings are warranted.</t>
+        </is>
+      </c>
+      <c r="DG87" s="2" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
+      <c r="DH87" s="2" t="inlineStr">
+        <is>
+          <t>50.7</t>
+        </is>
+      </c>
+      <c r="DI87" s="2" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="DJ87" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="DK87" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -22037,6 +24081,31 @@
           <t>Digital technologies have the potential to transform early childhood development (ECD) interventions by delivering personalized support at scale. We conducted a cluster-randomized controlled trial in rural Peru to evaluate the effectiveness and cost-effectiveness of an artificial intelligence–supported digital parenting chatbot as well as traditional home visits to improve child development. Among 2,461 caregiver–child dyads, both the digital and home-visiting interventions improved child development outcomes at 2.5 years of age, with standardized effect sizes of 0.11 and 0.17, respectively. At 1/15 of the cost of in-person support, the digital intervention yielded superior cost-effectiveness. These findings suggest that digital platforms can be a viable, scalable alternative to support children’s development in resource-constrained settings.</t>
         </is>
       </c>
+      <c r="DG88" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="DH88" s="2" t="inlineStr">
+        <is>
+          <t>49.8</t>
+        </is>
+      </c>
+      <c r="DI88" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ88" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK88" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -22245,6 +24314,31 @@
       <c r="DD89" s="2" t="inlineStr"/>
       <c r="DE89" s="2" t="inlineStr"/>
       <c r="DF89" s="2" t="inlineStr"/>
+      <c r="DG89" s="2" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
+      <c r="DH89" s="2" t="inlineStr">
+        <is>
+          <t>50.4</t>
+        </is>
+      </c>
+      <c r="DI89" s="2" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="DJ89" s="2" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="DK89" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -22489,6 +24583,31 @@
           <t>This study examined associations between family stimulation and early childhood development across five LMIC longitudinal studies. Random-effects and more conservative child-fixed-effects models indicate that family stimulation—caregivers’ engagement in nine activities (e.g., reading, playing, singing)—predicted increments in children’s early numeracy, literacy, social-emotional, motor, and executive-function skills (standardized associations 0.05–0.11 SD). Study-specific models showed variability, with null associations in two of the five studies. Findings indicate the need for additional research on culturally specific ways caregivers stimulate young children’s development.</t>
         </is>
       </c>
+      <c r="DG90" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DH90" s="2" t="inlineStr">
+        <is>
+          <t>46.2</t>
+        </is>
+      </c>
+      <c r="DI90" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="DJ90" s="2" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="DK90" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -22745,6 +24864,31 @@
           <t>This study leverages natural variation in the timing and location of community homicides to estimate their acute effects on the regulatory, behavioral, and developmental outcomes of Brazilian 3-year-olds (N=3,241; M age=41.05 months; 53% female) from seven low-income São Paulo neighborhoods. Recent exposure to community homicides was associated with lower effortful control, higher behavior problems, and lower overall developmental performance (d=.05–.20). Effects were consistent across subgroups but generally largest when community-violence exposure was geographically proximal (within 600 m of home) and recent (within 2 weeks prior to assessment). Results highlight the pervasive effects of community violence on young children and the need to expand support to mitigate these effects and prevent inequities early in life.</t>
         </is>
       </c>
+      <c r="DG91" s="2" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="DH91" s="2" t="inlineStr">
+        <is>
+          <t>34.2</t>
+        </is>
+      </c>
+      <c r="DI91" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="DJ91" s="2" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
+      <c r="DK91" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -23011,6 +25155,31 @@
       <c r="DF92" s="2" t="inlineStr">
         <is>
           <t>This five-year randomised controlled trial explored the impact of the Lifestart home-visiting parenting programme on parent and child development outcomes. Lifestart is a universal, structured, child-centred programme of information and practical activity for parents of children from birth to five years. In total, 424 parents and children participated, with outcomes measured at pre-test (child age &lt;12 months), mid-point (age 3) and post-test (age 5). Compared to the control group, parents who received Lifestart reported reduced parenting-related stress, increased knowledge of their child’s development, and improved confidence in their parenting role. There was no evidence of change in child development outcomes (cognitive, behavioural, social or emotional) and no clear evidence of consistent differential effects by gender, first-time motherhood, high pre-test anxiety or low maternal education. Results are commensurate with evaluations of similar programmes and align with the hypothesised theory of change.</t>
+        </is>
+      </c>
+      <c r="DG92" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="DH92" s="2" t="inlineStr">
+        <is>
+          <t>49.8</t>
+        </is>
+      </c>
+      <c r="DI92" s="2" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="DJ92" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK92" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -23229,6 +25398,31 @@
           <t>Theresa S Betancourt and colleagues argue that implementation and systems strengthening are urgently needed to integrate mental health and psychosocial support interventions across health, education, and social protection platforms to reach children affected by conflict.</t>
         </is>
       </c>
+      <c r="DG93" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="DH93" s="2" t="inlineStr">
+        <is>
+          <t>46.9</t>
+        </is>
+      </c>
+      <c r="DI93" s="2" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="DJ93" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK93" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -23439,6 +25633,31 @@
       <c r="DF94" s="2" t="inlineStr">
         <is>
           <t>Policy brief arguing that Early Childhood Development (ECD) is a catalyst for intergenerational peacebuilding and community stability. ECD interventions—encompassing learning, stimulation, and social cohesion—foster vital skills for peaceful societies, with nutrition serving as a critical entry point.</t>
+        </is>
+      </c>
+      <c r="DG94" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="DH94" s="2" t="inlineStr">
+        <is>
+          <t>66.8</t>
+        </is>
+      </c>
+      <c r="DI94" s="2" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="DJ94" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK94" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -23665,6 +25884,31 @@
           <t>Approximately 250 million children worldwide are out of school. Save the Children developed the Remote Assessment of Learning (ReAL) to assess 5–14-year-old children’s foundational learning. Children (N=4,840) were sampled from Cambodia, Mozambique, Niger, the occupied Palestinian territories, the Philippines, and Sudan, with an approximately equal proportion of male and female children within each country. The study assessed inter-rater reliability, factor structure, item slope and difficulty, criterion validity, and test–retest reliability. Results show moderate evidence that ReAL is valid and reliable for literacy and numeracy in low-resource and crisis-affected contexts.</t>
         </is>
       </c>
+      <c r="DG95" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="DH95" s="2" t="inlineStr">
+        <is>
+          <t>52.5</t>
+        </is>
+      </c>
+      <c r="DI95" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ95" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="DK95" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -23895,6 +26139,31 @@
       <c r="DF96" s="2" t="inlineStr">
         <is>
           <t>This article provides a systematic review and meta-analysis of current evidence for universal school-based (USB) social and emotional learning (SEL) interventions for K-12 students, 2008–2020. The sample includes 424 studies from 53 countries, reflecting 252 discrete USB SEL interventions involving 575,361 students. Compared to control conditions, students who participated in USB SEL interventions experienced significantly improved skills, attitudes, behaviors, school climate and safety, peer relationships, school functioning, and academic achievement. Significant heterogeneity in SEL content, intervention features, context, and implementation quality moderated student experiences and outcomes.</t>
+        </is>
+      </c>
+      <c r="DG96" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="DH96" s="2" t="inlineStr">
+        <is>
+          <t>52.5</t>
+        </is>
+      </c>
+      <c r="DI96" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="DJ96" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DK96" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -24109,6 +26378,31 @@
           <t>Understanding the effectiveness of universal school-based SEL interventions for minoritized students in K-12 settings is a critical area of inquiry. Drawing on evidence from a recent systematic review and meta-analysis of thirteen years of universal school-based SEL interventions, results revealed that the field knows a great deal about variation in effects of SEL programs but very little about the experiences of students with marginalized and minoritized identities within them. This manuscript details key findings and critical areas for future development in the service of gender-, racially-, ethnically-, linguistically-, and ability-minoritized youth.</t>
         </is>
       </c>
+      <c r="DG97" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="DH97" s="2" t="inlineStr">
+        <is>
+          <t>58.0</t>
+        </is>
+      </c>
+      <c r="DI97" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="DJ97" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DK97" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -24337,6 +26631,31 @@
           <t>This study systematically reviewed and meta-analyzed evidence for universal school-based SEL programming within the United States to understand nation-specific trends in SEL implementation and effectiveness and provide recommendations for marginalized students (minority gender, racial-ethnic, linguistic, and disability identities). Analyzing 90 universal school-based SEL studies (47 discrete programs; 20,626 students in grades K-12, 2008–2020), students who participated experienced significantly improved academic achievement, school functioning, and social-emotional outcomes.</t>
         </is>
       </c>
+      <c r="DG98" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="DH98" s="2" t="inlineStr">
+        <is>
+          <t>62.2</t>
+        </is>
+      </c>
+      <c r="DI98" s="2" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="DJ98" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DK98" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -24557,6 +26876,31 @@
           <t>This systematic review and meta-analysis disentangles the effects of social and emotional learning (SEL) programs on student academic achievement across grades 1–12. After removing duplicates (n=9,745) and screening, 258 SEL studies implemented in universal K-12 education settings met selection criteria, with near-perfect interrater reliability across screening stages. The review examines how universal school-based SEL programming relates to academic achievement.</t>
         </is>
       </c>
+      <c r="DG99" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DH99" s="2" t="inlineStr">
+        <is>
+          <t>48.3</t>
+        </is>
+      </c>
+      <c r="DI99" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ99" s="2" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="DK99" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -24811,6 +27155,31 @@
       <c r="DF100" s="2" t="inlineStr">
         <is>
           <t>Question: We compared the effectiveness of different types of parenting interventions based on an a priori taxonomy, and the impact of waitlists versus treatment as usual (TAU), in reducing child internalising problems. Study selection and analysis: Systematic review and network meta-analysis of published and unpublished randomised controlled trials (RCTs) until 1 October 2022 that investigated parenting interventions with children younger than 4 years; excluded children born preterm or with intellectual disabilities and families receiving support for current abuse, neglect, and substance misuse. Random-effects network meta-analysis estimated standardised mean differences (SMDs) with 95% credible intervals (CrIs). Findings: Of 20,520 citations identified, 59 RCTs (18,349 participants) were eligible. Parenting interventions focusing on the dyadic relationship (SMD: −0.26, 95% CrI: −0.43 to −0.08) and those with mixed focus (−0.09, −0.17 to −0.02) were more effective in reducing internalising problems than TAU at the first time point; all interventions were more effective than waitlist, which increased the risk of internalising problems compared with TAU (0.36, 0.19 to 0.52). There was weak evidence that all parenting interventions improved self-efficacy and that home visiting reduced parental depressive symptoms. Most studies were rated 'high risk' or 'some concerns' for bias. Conclusions: Preliminary evidence that relationship-focused and mixed parenting interventions reduced child internalising problems, and the waitlist comparator increased internalising problems with implications for waiting times between referral and support. Given the high risk of bias of most included studies, findings should be interpreted with caution.</t>
+        </is>
+      </c>
+      <c r="DG100" s="2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="DH100" s="2" t="inlineStr">
+        <is>
+          <t>64.5</t>
+        </is>
+      </c>
+      <c r="DI100" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="DJ100" s="2" t="inlineStr">
+        <is>
+          <t>95</t>
+        </is>
+      </c>
+      <c r="DK100" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -25049,6 +27418,31 @@
           <t>Protocol for a two-arm cluster randomised Type I hybrid effectiveness-implementation trial of the Resettled Refugee Families for Healing (RRF4H) intervention, addressing the intergenerational impact of war trauma and promoting resilience among second-generation refugee children in the USA. Compared with usual care, RRF4H participants are hypothesised to show improvements in primary mental health outcomes; a minimum sample of 128 (64/arm) provides 80% power (α=0.05) to detect a medium effect (0.5).</t>
         </is>
       </c>
+      <c r="DG101" s="2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="DH101" s="2" t="inlineStr">
+        <is>
+          <t>53.7</t>
+        </is>
+      </c>
+      <c r="DI101" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="DJ101" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="DK101" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -25283,6 +27677,31 @@
       <c r="DF102" s="2" t="inlineStr">
         <is>
           <t>Task-shared mental-health and psychosocial support interventions rely on nonspecialists' quality of delivery. Using data from the Sugira Muryango cluster-RCT in Rwanda, this study used a parallel-process latent growth model to examine factors associated with nonspecialists' fidelity and competence over time. Sugira Muryango improved responsive caregiving (d=0.87) and reduced violent discipline (OR=0.30) vs control; delivery quality varied significantly across agents, with district and education-level differences in initial scores and growth.</t>
+        </is>
+      </c>
+      <c r="DG102" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="DH102" s="2" t="inlineStr">
+        <is>
+          <t>49.2</t>
+        </is>
+      </c>
+      <c r="DI102" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ102" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="DK102" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -25501,6 +27920,31 @@
           <t>Families in LMICs face significant mental-health and psychosocial care gaps, increasingly addressed by task-sharing evidence-based interventions to nonspecialist community providers. This qualitative study, using data from the Sugira Muryango cluster-RCT in Rwanda, explored nonspecialists' preparedness to deliver the program. Nonspecialists used rapport-building, empathy, and active listening, and their community embeddedness eased trust; barriers included limited supervisor availability, delayed compensation, and technology issues.</t>
         </is>
       </c>
+      <c r="DG103" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="DH103" s="2" t="inlineStr">
+        <is>
+          <t>46.5</t>
+        </is>
+      </c>
+      <c r="DI103" s="2" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="DJ103" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK103" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -25727,6 +28171,31 @@
       <c r="DF104" s="2" t="inlineStr">
         <is>
           <t>Caregivers of children with disabilities are at elevated risk of depression, yet evidence from LMICs is scarce. Using baseline data from the Sugira Muryango cluster-RCT in rural Rwanda, 65% of caregivers of children with disabilities met the clinical cut-off for likely depression. Economic hardship, food insecurity, and caregiver illness were significant risk factors; family unity was protective. Findings suggest parenting programmes should also promote economic empowerment, reduce family conflict, and strengthen family unity.</t>
+        </is>
+      </c>
+      <c r="DG104" s="2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="DH104" s="2" t="inlineStr">
+        <is>
+          <t>52.8</t>
+        </is>
+      </c>
+      <c r="DI104" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="DJ104" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="DK104" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -25941,6 +28410,31 @@
           <t>A Conflict Observatory report by the Humanitarian Research Lab at Yale School of Public Health documenting Belarus' collaboration with Russia in the systematic deportation of Ukraine's children. At least 2,442 children (aged 6–17) were transported to 13 facilities across six Belarus regions after Russia's February 2022 invasion; ~85% went to the Dubrava facility. At least eight facilities conducted 're-education,' and consent could not be considered freely given.</t>
         </is>
       </c>
+      <c r="DG105" s="2" t="inlineStr">
+        <is>
+          <t>93</t>
+        </is>
+      </c>
+      <c r="DH105" s="2" t="inlineStr">
+        <is>
+          <t>34.9</t>
+        </is>
+      </c>
+      <c r="DI105" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DJ105" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK105" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -26145,6 +28639,31 @@
           <t>A Conflict Observatory report by the Humanitarian Research Lab at Yale School of Public Health providing the largest high-confidence public count to date of Ukrainian children in Russia's program of coerced adoption and fostering: 314 individually identified children since February 2022, plus 166 placed with Russian citizens, across at least 21 Russian regions. 80.4% were taken from Donetsk oblast. The program is assessed as systematic, intentional, and widespread, initiated by Putin and subordinates to 'Russify' the children.</t>
         </is>
       </c>
+      <c r="DG106" s="2" t="inlineStr">
+        <is>
+          <t>94</t>
+        </is>
+      </c>
+      <c r="DH106" s="2" t="inlineStr">
+        <is>
+          <t>34.9</t>
+        </is>
+      </c>
+      <c r="DI106" s="2" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="DJ106" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK106" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -26365,6 +28884,31 @@
           <t>A data-analysis dossier by Fondazione S.O.S. Il Telefono Azzurro ETS analysing cases recorded by its free 24/7 listening and counselling helpline 1.96.96 (phone and chat) for children, adolescents, and adults during 2025 in Italy. It maps the main areas of need, how needs overlap into multidimensional situations, and documents a clear preference for chat over telephone. Framed by WHO data on adolescent mental disorders and youth suicide.</t>
         </is>
       </c>
+      <c r="DG107" s="2" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="DH107" s="2" t="inlineStr">
+        <is>
+          <t>33.7</t>
+        </is>
+      </c>
+      <c r="DI107" s="2" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="DJ107" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="DK107" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -26603,6 +29147,31 @@
       <c r="DF108" s="2" t="inlineStr">
         <is>
           <t>Book chapter presenting the Early Years Media Initiative for Children Revised Toddler Module, which builds toddlers' social-emotional resilience through staff training (12 topics, micro-training videos), co-regulation techniques, and problem-solving activities. A controlled trial showed marked improvements in children's social-emotional functioning and reduced stress among staff and parents; the programme is being scaled nationally and internationally.</t>
+        </is>
+      </c>
+      <c r="DG108" s="2" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="DH108" s="2" t="inlineStr">
+        <is>
+          <t>53.4</t>
+        </is>
+      </c>
+      <c r="DI108" s="2" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
+      <c r="DJ108" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="DK108" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -26825,6 +29394,31 @@
           <t>Book chapter describing how Early Years (Northern Ireland) pioneered a culture of respecting difference with young children, their families and communities through the Media Initiative for Children / Respecting Difference programme. The approach has been evaluated with rigorous independent research, including a large randomised controlled trial and qualitative evaluations.</t>
         </is>
       </c>
+      <c r="DG109" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DH109" s="2" t="inlineStr">
+        <is>
+          <t>48.9</t>
+        </is>
+      </c>
+      <c r="DI109" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="DJ109" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DK109" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -27045,6 +29639,31 @@
           <t>Book chapter describing how inspiration from the Media Initiative for Children in Northern Ireland developed into a strategic approach to actively develop respect for diversity from the early years in Serbia and the Western Balkans, led by Pomoć deci. It addresses ethnic, religious, economic and language divisions, particularly for children with multiple differences and displaced families.</t>
         </is>
       </c>
+      <c r="DG110" s="2" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="DH110" s="2" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="DI110" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="DJ110" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="DK110" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -27257,6 +29876,31 @@
           <t>A UNICEF Office of Strategy and Evidence – Innocenti global data story on children's play, using internationally comparable data (2010–2024; 93 countries, ~60% of the global under-5 population; comparable play data for ages 2–4). It documents the developmental importance of play, age-based play patterns, drivers of digital play, and gaps in globally comparable data, and describes UNICEF's work to expand MICS measurement of play and playthings.</t>
         </is>
       </c>
+      <c r="DG111" s="2" t="inlineStr">
+        <is>
+          <t>92</t>
+        </is>
+      </c>
+      <c r="DH111" s="2" t="inlineStr">
+        <is>
+          <t>35.4</t>
+        </is>
+      </c>
+      <c r="DI111" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="DJ111" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="DK111" s="2" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add one-page advocacy shortlist (top 15) as doc + Excel tab
ADVOCACY_SHORTLIST.md and an "Advocacy shortlist" tab in the review Excel:
top 15 papers by the ToC-aligned relevance rank, each with the single most
quotable statistic and the Theory-of-Change outcome it supports. Caveats
flagged (U.S.-poverty context, Pruett attribution, conceptual framing).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/ECPC_Repository_for_review.xlsx
+++ b/pipeline/ECPC_Repository_for_review.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ECPC Repository" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Advocacy shortlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ECPC Repository" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,8 +29,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -46,8 +51,13 @@
         <fgColor rgb="00FFFFCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,11 +65,16 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -68,6 +83,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -435,6 +456,713 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="64" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>ECPC member (year)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Journal / source</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Context</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Quotable finding</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Use for (ToC outcome)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>DOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Black (2025)</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Child Psychology and Psychiatry</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Rwanda</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Hybrid Type-2 Implementation-Effectiveness study with an embedded cluster trial</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Sugira Muryango, delivered at scale through government child-protection volunteers, cut harsh discipline (OR=0.34) and raised father involvement (IRR=1.18) and home stimulation (d=0.20–0.37).</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Caregiver practices ↑ / violence ↓ + scaling through government (vertical cohesion)</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr"/>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcpp.14160</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Yoshikawa (2024)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Early Childhood Research Quarterly</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Cluster randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>A 6-month audio-only phone programme for 2,298 Syrian &amp; Jordanian refugee caregivers significantly reduced caregiver depression (ES=−0.11) — remote delivery for hard-to-reach families.</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Caregiver mental health (pathway a) in displacement</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ecresq.2024.07.004</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Betancourt (2024)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Comprehensive Psychiatry</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Low- and middle-income countries</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Systematic review</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Across 80 LMIC/humanitarian studies (n=18,193), 43 improved child/adolescent mental health and only 3 found no effect; active ingredients = caregiver psychoeducation, communication skills, father engagement.</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Evidence base: what works in caregiver/family interventions</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>most-cited (44)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.comppsych.2024.152483</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Panter-Brick (2024)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Child and Family Studies</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Prospective longitudinal</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>In Syrian refugee families, spousal DISAGREEMENT about father involvement — not the level of it — predicted worse outcomes: child social-emotional learning was &gt;1 SD (43%) lower in the most discordant families.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Caregiver dyad / family unity → child SEL</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10826-024-02809-y</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Leckman (2024)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Journal of the American Academy of Child &amp; Adolescent Psychiatry</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Scoping review</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Of 6,843 records, only 6 studies evaluated digital mental-health tools for war/disaster-affected youth, and &lt;10% of relevant interventions were built in the LMICs where war actually occurs.</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Evidence gap in crisis contexts (call to action)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jaac.2024.02.017</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Betancourt (2024)</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>BMC Psychiatry</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Sierra Leone</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Pilot randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>A community-health-worker–delivered family intervention improved observed caregiver–child interaction (HOME +3.08; responsiveness subscale +1.66, p&lt;.001) and trended toward less intimate-partner violence.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Nurturing care via non-specialist delivery</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s12888-024-06209-w</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Yoshikawa (2026)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>BMC Global and Public Health</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Bangladesh</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Cluster randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>A father-engagement add-on for 2,002 fathers in Rohingya camps &amp; host communities improved fathers' parenting, family engagement, and father-reported child social-emotional development vs a mother-only programme.</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Father engagement in displacement (family unit)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s44263-026-00266-x</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Hein (2024)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Yale Jackson School of Global Affairs (Policy Brief)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Policy brief / conceptual synthesis</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Frames ECD as a catalyst for intergenerational peacebuilding and community stability, with nutrition as a critical entry point.</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>HEADLINE framing: ECD → peace</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>⚠ conceptual — framing, not a data point</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Aber (2026)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Research on Educational Effectiveness</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Niger</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Cluster RCT</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Cluster-RCT, 1,795 grade 2–4 students (19% Nigerian refugees), Diffa, Niger: adding Mindfulness to remedial tutoring cut sadness dysregulation (ES=−0.30), with larger gains for girls and refugees.</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>SEL / self-regulation in education-in-emergencies</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/19345747.2025.2591604</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Aber (2023)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>AERA Open</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Lebanon</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Cluster RCT</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Cluster-RCT, 4,017 Syrian refugee students: 26 weeks of Healing Classroom Tutoring improved behavioral regulation (ES=0.31) — but longer/more-intensive isn't automatically better (it lowered school perceptions).</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>SEL in conflict education (with a dosage caution)</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/23328584231209268</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Yoshikawa (2024)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SSRN Electronic Journal</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Baby's First Years RCT ($333 vs $20/mo): unconditional cash alone showed little effect on child development — evidence that income support must be paired with nurturing-care/ECD services.</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Economic pathway — cash alone is insufficient</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>⚠ U.S. poverty, not conflict</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2139/ssrn.4955765</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Pruett (2023)</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>BMJ Mental Health</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; network meta-analysis of RCTs</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Network meta-analysis of 59 RCTs (18,349 children &lt;4): relationship-focused parenting interventions reduced child internalising (SMD=−0.26); being on a waitlist actively increased problems — evidence against delay.</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>What works + the cost of delay</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>⚠ authorship attribution to verify</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/bmjment-2023-300811</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>McCarthy (2024)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Social and Emotional Learning: Research, Practice, and Policy</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Systematic review &amp; meta-analysis</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Meta-analysis of 90 U.S. studies (20,626 students): universal school-based SEL improved academics, school functioning and social-emotional outcomes and cut distress/externalizing — strongest when teachers deliver it.</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>SEL evidence base (individual competencies)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>⚠ U.S., not crisis</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.sel.2024.100029</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Black (2025)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>American Journal of Community Psychology</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Hybrid Type II Implementation-Effectiveness trial</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Among resettled Somali Bantu &amp; Bhutanese refugee families (COVID-19), a family intervention improved parental supervision (B=−0.49) and reduced children's conduct problems (β=−9.20, p=.01).</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>Family strengthening for resettled refugees</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/ajcp.70021</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Cuartas (2024)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>The Lancet</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Lancet Series: failing to invest in the 'next 1000 days' (ages 2–5) carries large human-capital and economic costs; a minimum package (e.g., 1 year of ECCE for all) is worthwhile.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>Economic / cost case for investment</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>highly cited (32)</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>10.1016/s0140-6736(24)01390-4</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:DK111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>